<commit_message>
Rebuild 2027 projections (run 36895277181)
Verification PASSED.

Regenerated by .github/workflows/refresh-projections.yml.
Verification and the full baseline audit are in the run summary:
https://github.com/pmammino/DFSSimsFull/actions/runs/36895277181
</commit_message>
<xml_diff>
--- a/out/mlb_2027_what_if.xlsx
+++ b/out/mlb_2027_what_if.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="What-If" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What-If" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -660,11 +660,7 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C6" s="2" t="n"/>
       <c r="D6" s="5" t="n">
         <v>756.9</v>
       </c>
@@ -713,16 +709,16 @@
         <v/>
       </c>
       <c r="P6" s="8" t="n">
-        <v>0.11547</v>
+        <v>0.1159</v>
       </c>
       <c r="Q6" s="8" t="n">
-        <v>0.04586</v>
+        <v>0.0464</v>
       </c>
       <c r="R6" s="8" t="n">
-        <v>0.00162</v>
+        <v>0.00265</v>
       </c>
       <c r="S6" s="8" t="n">
-        <v>0.04932</v>
+        <v>0.05036</v>
       </c>
       <c r="T6" s="8" t="n">
         <v>0.11343</v>
@@ -737,13 +733,13 @@
         <v>0.23479</v>
       </c>
       <c r="X6" s="8" t="n">
-        <v>0.0035</v>
+        <v>0.00351</v>
       </c>
       <c r="Y6" s="8" t="n">
-        <v>0.1341583992102379</v>
+        <v>0.1356278495509935</v>
       </c>
       <c r="Z6" s="8" t="n">
-        <v>0.1428421065045733</v>
+        <v>0.1444066703582942</v>
       </c>
     </row>
     <row r="7">
@@ -757,11 +753,7 @@
           <t>LAA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C7" s="2" t="n"/>
       <c r="D7" s="5" t="n">
         <v>723.7</v>
       </c>
@@ -810,16 +802,16 @@
         <v/>
       </c>
       <c r="P7" s="8" t="n">
-        <v>0.11264</v>
+        <v>0.11325</v>
       </c>
       <c r="Q7" s="8" t="n">
-        <v>0.05052</v>
+        <v>0.05157</v>
       </c>
       <c r="R7" s="8" t="n">
-        <v>0.00285</v>
+        <v>0.00344</v>
       </c>
       <c r="S7" s="8" t="n">
-        <v>0.04638</v>
+        <v>0.04717</v>
       </c>
       <c r="T7" s="8" t="n">
         <v>0.07695</v>
@@ -834,13 +826,13 @@
         <v>0.26759</v>
       </c>
       <c r="X7" s="8" t="n">
-        <v>0.03718</v>
+        <v>0.03728</v>
       </c>
       <c r="Y7" s="8" t="n">
-        <v>0.1355976174039096</v>
+        <v>0.1352631682233155</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>0.1154729260212444</v>
+        <v>0.1151881140442495</v>
       </c>
     </row>
     <row r="8">
@@ -854,11 +846,7 @@
           <t>WSH</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C8" s="2" t="n"/>
       <c r="D8" s="5" t="n">
         <v>718.8</v>
       </c>
@@ -907,16 +895,16 @@
         <v/>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0.12016</v>
+        <v>0.12046</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>0.04789</v>
+        <v>0.04611</v>
       </c>
       <c r="R8" s="8" t="n">
-        <v>0.00281</v>
+        <v>0.00318</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>0.04368</v>
+        <v>0.04535</v>
       </c>
       <c r="T8" s="8" t="n">
         <v>0.13536</v>
@@ -931,13 +919,13 @@
         <v>0.29519</v>
       </c>
       <c r="X8" s="8" t="n">
-        <v>0.02913</v>
+        <v>0.02916</v>
       </c>
       <c r="Y8" s="8" t="n">
-        <v>0.1362901213796398</v>
+        <v>0.1360751883771715</v>
       </c>
       <c r="Z8" s="8" t="n">
-        <v>0.1233214066095435</v>
+        <v>0.123126925601508</v>
       </c>
     </row>
     <row r="9">
@@ -951,11 +939,7 @@
           <t>MIA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C9" s="2" t="n"/>
       <c r="D9" s="5" t="n">
         <v>715.8</v>
       </c>
@@ -1004,16 +988,16 @@
         <v/>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0.17747</v>
+        <v>0.17372</v>
       </c>
       <c r="Q9" s="8" t="n">
-        <v>0.04102</v>
+        <v>0.04159</v>
       </c>
       <c r="R9" s="8" t="n">
-        <v>0.00427</v>
+        <v>0.0052</v>
       </c>
       <c r="S9" s="8" t="n">
-        <v>0.02175</v>
+        <v>0.02088</v>
       </c>
       <c r="T9" s="8" t="n">
         <v>0.06506000000000001</v>
@@ -1028,13 +1012,13 @@
         <v>0.14717</v>
       </c>
       <c r="X9" s="8" t="n">
-        <v>0.03694</v>
+        <v>0.03639</v>
       </c>
       <c r="Y9" s="8" t="n">
-        <v>0.1199205075982292</v>
+        <v>0.1199913682433856</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>0.10732529230514</v>
+        <v>0.1073887104777833</v>
       </c>
     </row>
     <row r="10">
@@ -1048,11 +1032,7 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C10" s="2" t="n"/>
       <c r="D10" s="5" t="n">
         <v>712.3</v>
       </c>
@@ -1101,16 +1081,16 @@
         <v/>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0.11312</v>
+        <v>0.11398</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>0.04206</v>
+        <v>0.04236</v>
       </c>
       <c r="R10" s="8" t="n">
-        <v>0.00219</v>
+        <v>0.00308</v>
       </c>
       <c r="S10" s="8" t="n">
-        <v>0.03906</v>
+        <v>0.04067</v>
       </c>
       <c r="T10" s="8" t="n">
         <v>0.09832</v>
@@ -1125,13 +1105,13 @@
         <v>0.26083</v>
       </c>
       <c r="X10" s="8" t="n">
-        <v>0.01702</v>
+        <v>0.01709</v>
       </c>
       <c r="Y10" s="8" t="n">
-        <v>0.1254161500689744</v>
+        <v>0.1267898456820705</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>0.1274553577369701</v>
+        <v>0.1288513889952457</v>
       </c>
     </row>
     <row r="11">
@@ -1145,11 +1125,7 @@
           <t>WSH</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C11" s="2" t="n"/>
       <c r="D11" s="5" t="n">
         <v>683.4</v>
       </c>
@@ -1198,16 +1174,16 @@
         <v/>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0.14729</v>
+        <v>0.14452</v>
       </c>
       <c r="Q11" s="8" t="n">
-        <v>0.04819</v>
+        <v>0.04806</v>
       </c>
       <c r="R11" s="8" t="n">
-        <v>0.01377</v>
+        <v>0.01393</v>
       </c>
       <c r="S11" s="8" t="n">
-        <v>0.02999</v>
+        <v>0.03044</v>
       </c>
       <c r="T11" s="8" t="n">
         <v>0.06332</v>
@@ -1222,13 +1198,13 @@
         <v>0.18752</v>
       </c>
       <c r="X11" s="8" t="n">
-        <v>0.0269</v>
+        <v>0.02656</v>
       </c>
       <c r="Y11" s="8" t="n">
-        <v>0.1204647308713135</v>
+        <v>0.1202747549138809</v>
       </c>
       <c r="Z11" s="8" t="n">
-        <v>0.1179639040139702</v>
+        <v>0.1177778719243665</v>
       </c>
     </row>
     <row r="12">
@@ -1242,11 +1218,7 @@
           <t>WSH</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C12" s="2" t="n"/>
       <c r="D12" s="5" t="n">
         <v>682.3</v>
       </c>
@@ -1295,16 +1267,16 @@
         <v/>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0.13451</v>
+        <v>0.13371</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>0.04545</v>
+        <v>0.04495</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>0.00992</v>
+        <v>0.00763</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>0.03286</v>
+        <v>0.03736</v>
       </c>
       <c r="T12" s="8" t="n">
         <v>0.06557</v>
@@ -1319,13 +1291,13 @@
         <v>0.2111</v>
       </c>
       <c r="X12" s="8" t="n">
-        <v>0.04808</v>
+        <v>0.04791</v>
       </c>
       <c r="Y12" s="8" t="n">
-        <v>0.1350940737522148</v>
+        <v>0.1348810269474038</v>
       </c>
       <c r="Z12" s="8" t="n">
-        <v>0.114998496673247</v>
+        <v>0.1148171411067605</v>
       </c>
     </row>
     <row r="13">
@@ -1339,11 +1311,7 @@
           <t>BAL</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C13" s="2" t="n"/>
       <c r="D13" s="5" t="n">
         <v>663.1</v>
       </c>
@@ -1392,16 +1360,16 @@
         <v/>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0.13699</v>
+        <v>0.1293</v>
       </c>
       <c r="Q13" s="8" t="n">
-        <v>0.0417</v>
+        <v>0.0455</v>
       </c>
       <c r="R13" s="8" t="n">
-        <v>0.00056</v>
+        <v>0.0009700000000000001</v>
       </c>
       <c r="S13" s="8" t="n">
-        <v>0.0571</v>
+        <v>0.05837</v>
       </c>
       <c r="T13" s="8" t="n">
         <v>0.09995</v>
@@ -1416,13 +1384,13 @@
         <v>0.22978</v>
       </c>
       <c r="X13" s="8" t="n">
-        <v>0.00456</v>
+        <v>0.00442</v>
       </c>
       <c r="Y13" s="8" t="n">
-        <v>0.1289383385169633</v>
+        <v>0.1277046627066473</v>
       </c>
       <c r="Z13" s="8" t="n">
-        <v>0.1554959064240461</v>
+        <v>0.1540081290836139</v>
       </c>
     </row>
     <row r="14">
@@ -1436,11 +1404,7 @@
           <t>BAL</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C14" s="2" t="n"/>
       <c r="D14" s="5" t="n">
         <v>656.6</v>
       </c>
@@ -1489,16 +1453,16 @@
         <v/>
       </c>
       <c r="P14" s="8" t="n">
-        <v>0.1448</v>
+        <v>0.14625</v>
       </c>
       <c r="Q14" s="8" t="n">
-        <v>0.04728</v>
+        <v>0.04722</v>
       </c>
       <c r="R14" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.00611</v>
       </c>
       <c r="S14" s="8" t="n">
-        <v>0.02969</v>
+        <v>0.02949</v>
       </c>
       <c r="T14" s="8" t="n">
         <v>0.09762</v>
@@ -1513,13 +1477,13 @@
         <v>0.22572</v>
       </c>
       <c r="X14" s="8" t="n">
-        <v>0.02667</v>
+        <v>0.02686</v>
       </c>
       <c r="Y14" s="8" t="n">
-        <v>0.13520125727237</v>
+        <v>0.1339076581571674</v>
       </c>
       <c r="Z14" s="8" t="n">
-        <v>0.1073571980922817</v>
+        <v>0.1059250369607924</v>
       </c>
     </row>
     <row r="15">
@@ -1533,11 +1497,7 @@
           <t>TB</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C15" s="2" t="n"/>
       <c r="D15" s="5" t="n">
         <v>654.2</v>
       </c>
@@ -1586,16 +1546,16 @@
         <v/>
       </c>
       <c r="P15" s="8" t="n">
-        <v>0.13867</v>
+        <v>0.13837</v>
       </c>
       <c r="Q15" s="8" t="n">
-        <v>0.0412</v>
+        <v>0.04281</v>
       </c>
       <c r="R15" s="8" t="n">
-        <v>0.00116</v>
+        <v>0.00131</v>
       </c>
       <c r="S15" s="8" t="n">
-        <v>0.05393</v>
+        <v>0.05456</v>
       </c>
       <c r="T15" s="8" t="n">
         <v>0.08722000000000001</v>
@@ -1610,13 +1570,13 @@
         <v>0.19273</v>
       </c>
       <c r="X15" s="8" t="n">
-        <v>0.00902</v>
+        <v>0.009010000000000001</v>
       </c>
       <c r="Y15" s="8" t="n">
-        <v>0.1291435705941901</v>
+        <v>0.1297262751223533</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>0.1399846845360544</v>
+        <v>0.1406163049038152</v>
       </c>
     </row>
     <row r="16">
@@ -1630,11 +1590,7 @@
           <t>LAA</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C16" s="2" t="n"/>
       <c r="D16" s="5" t="n">
         <v>651.7</v>
       </c>
@@ -1683,16 +1639,16 @@
         <v/>
       </c>
       <c r="P16" s="8" t="n">
-        <v>0.11508</v>
+        <v>0.11213</v>
       </c>
       <c r="Q16" s="8" t="n">
-        <v>0.03682</v>
+        <v>0.03651</v>
       </c>
       <c r="R16" s="8" t="n">
-        <v>0.00296</v>
+        <v>0.00319</v>
       </c>
       <c r="S16" s="8" t="n">
-        <v>0.04358</v>
+        <v>0.04617</v>
       </c>
       <c r="T16" s="8" t="n">
         <v>0.14365</v>
@@ -1707,13 +1663,13 @@
         <v>0.27722</v>
       </c>
       <c r="X16" s="8" t="n">
-        <v>0.01244</v>
+        <v>0.0123</v>
       </c>
       <c r="Y16" s="8" t="n">
-        <v>0.1402627161059547</v>
+        <v>0.1399167605400114</v>
       </c>
       <c r="Z16" s="8" t="n">
-        <v>0.1126381980373055</v>
+        <v>0.1123603778679071</v>
       </c>
     </row>
     <row r="17">
@@ -1727,11 +1683,7 @@
           <t>PIT</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C17" s="2" t="n"/>
       <c r="D17" s="5" t="n">
         <v>648.7</v>
       </c>
@@ -1780,16 +1732,16 @@
         <v/>
       </c>
       <c r="P17" s="8" t="n">
-        <v>0.13764</v>
+        <v>0.13876</v>
       </c>
       <c r="Q17" s="8" t="n">
-        <v>0.04857</v>
+        <v>0.04963</v>
       </c>
       <c r="R17" s="8" t="n">
-        <v>0.00551</v>
+        <v>0.00579</v>
       </c>
       <c r="S17" s="8" t="n">
-        <v>0.03526</v>
+        <v>0.03495</v>
       </c>
       <c r="T17" s="8" t="n">
         <v>0.09682</v>
@@ -1804,13 +1756,13 @@
         <v>0.23447</v>
       </c>
       <c r="X17" s="8" t="n">
-        <v>0.0128</v>
+        <v>0.01286</v>
       </c>
       <c r="Y17" s="8" t="n">
-        <v>0.1270838595031016</v>
+        <v>0.1272588983856731</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>0.1196477403082826</v>
+        <v>0.119812537056254</v>
       </c>
     </row>
     <row r="18">
@@ -1824,11 +1776,7 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C18" s="2" t="n"/>
       <c r="D18" s="5" t="n">
         <v>646.3</v>
       </c>
@@ -1877,16 +1825,16 @@
         <v/>
       </c>
       <c r="P18" s="8" t="n">
-        <v>0.162</v>
+        <v>0.15943</v>
       </c>
       <c r="Q18" s="8" t="n">
-        <v>0.04816</v>
+        <v>0.04719</v>
       </c>
       <c r="R18" s="8" t="n">
-        <v>0.00192</v>
+        <v>0.00193</v>
       </c>
       <c r="S18" s="8" t="n">
-        <v>0.03602</v>
+        <v>0.03986</v>
       </c>
       <c r="T18" s="8" t="n">
         <v>0.07289</v>
@@ -1901,13 +1849,13 @@
         <v>0.1569</v>
       </c>
       <c r="X18" s="8" t="n">
-        <v>0.008959999999999999</v>
+        <v>0.008869999999999999</v>
       </c>
       <c r="Y18" s="8" t="n">
-        <v>0.1122565395014482</v>
+        <v>0.1118902270637113</v>
       </c>
       <c r="Z18" s="8" t="n">
-        <v>0.1332646565569908</v>
+        <v>0.1328297910121916</v>
       </c>
     </row>
     <row r="19">
@@ -1921,11 +1869,7 @@
           <t>MIA</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C19" s="2" t="n"/>
       <c r="D19" s="5" t="n">
         <v>645</v>
       </c>
@@ -1974,16 +1918,16 @@
         <v/>
       </c>
       <c r="P19" s="8" t="n">
-        <v>0.18358</v>
+        <v>0.18613</v>
       </c>
       <c r="Q19" s="8" t="n">
-        <v>0.03157</v>
+        <v>0.03128</v>
       </c>
       <c r="R19" s="8" t="n">
-        <v>0.00671</v>
+        <v>0.0054</v>
       </c>
       <c r="S19" s="8" t="n">
-        <v>0.00746</v>
+        <v>0.00735</v>
       </c>
       <c r="T19" s="8" t="n">
         <v>0.09626999999999999</v>
@@ -1998,13 +1942,13 @@
         <v>0.15252</v>
       </c>
       <c r="X19" s="8" t="n">
-        <v>0.0425</v>
+        <v>0.04288</v>
       </c>
       <c r="Y19" s="8" t="n">
-        <v>0.1134044309081393</v>
+        <v>0.1134714412243787</v>
       </c>
       <c r="Z19" s="8" t="n">
-        <v>0.08150795055052711</v>
+        <v>0.081556113338336</v>
       </c>
     </row>
     <row r="20">
@@ -2018,11 +1962,7 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C20" s="2" t="n"/>
       <c r="D20" s="5" t="n">
         <v>643.4</v>
       </c>
@@ -2071,16 +2011,16 @@
         <v/>
       </c>
       <c r="P20" s="8" t="n">
-        <v>0.13855</v>
+        <v>0.13754</v>
       </c>
       <c r="Q20" s="8" t="n">
-        <v>0.04364</v>
+        <v>0.04465</v>
       </c>
       <c r="R20" s="8" t="n">
-        <v>0.00373</v>
+        <v>0.00361</v>
       </c>
       <c r="S20" s="8" t="n">
-        <v>0.03338</v>
+        <v>0.03181</v>
       </c>
       <c r="T20" s="8" t="n">
         <v>0.07461</v>
@@ -2095,13 +2035,13 @@
         <v>0.26529</v>
       </c>
       <c r="X20" s="8" t="n">
-        <v>0.02474</v>
+        <v>0.02463</v>
       </c>
       <c r="Y20" s="8" t="n">
-        <v>0.1172051599990816</v>
+        <v>0.1168226993596811</v>
       </c>
       <c r="Z20" s="8" t="n">
-        <v>0.1216645632612075</v>
+        <v>0.1212675508203079</v>
       </c>
     </row>
     <row r="21">
@@ -2115,11 +2055,7 @@
           <t>MIA</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C21" s="2" t="n"/>
       <c r="D21" s="5" t="n">
         <v>641.8</v>
       </c>
@@ -2168,16 +2104,16 @@
         <v/>
       </c>
       <c r="P21" s="8" t="n">
-        <v>0.13955</v>
+        <v>0.14507</v>
       </c>
       <c r="Q21" s="8" t="n">
-        <v>0.04158</v>
+        <v>0.03977</v>
       </c>
       <c r="R21" s="8" t="n">
-        <v>0.00711</v>
+        <v>0.00773</v>
       </c>
       <c r="S21" s="8" t="n">
-        <v>0.01659</v>
+        <v>0.01777</v>
       </c>
       <c r="T21" s="8" t="n">
         <v>0.11438</v>
@@ -2192,13 +2128,13 @@
         <v>0.20699</v>
       </c>
       <c r="X21" s="8" t="n">
-        <v>0.04315</v>
+        <v>0.04402</v>
       </c>
       <c r="Y21" s="8" t="n">
-        <v>0.1232165405595429</v>
+        <v>0.1232893488200553</v>
       </c>
       <c r="Z21" s="8" t="n">
-        <v>0.0875016012669218</v>
+        <v>0.0875533056838074</v>
       </c>
     </row>
     <row r="22">
@@ -2212,11 +2148,7 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C22" s="2" t="n"/>
       <c r="D22" s="5" t="n">
         <v>640.6</v>
       </c>
@@ -2265,16 +2197,16 @@
         <v/>
       </c>
       <c r="P22" s="8" t="n">
-        <v>0.18285</v>
+        <v>0.1849</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>0.04521</v>
+        <v>0.04563</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>0.00645</v>
+        <v>0.00677</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>0.01285</v>
+        <v>0.01461</v>
       </c>
       <c r="T22" s="8" t="n">
         <v>0.06451</v>
@@ -2289,13 +2221,13 @@
         <v>0.11457</v>
       </c>
       <c r="X22" s="8" t="n">
-        <v>0.01927</v>
+        <v>0.01942</v>
       </c>
       <c r="Y22" s="8" t="n">
-        <v>0.1160787254839419</v>
+        <v>0.1173501473533214</v>
       </c>
       <c r="Z22" s="8" t="n">
-        <v>0.0954817523397373</v>
+        <v>0.0965275735058925</v>
       </c>
     </row>
     <row r="23">
@@ -2309,11 +2241,7 @@
           <t>TB</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C23" s="2" t="n"/>
       <c r="D23" s="5" t="n">
         <v>639.3</v>
       </c>
@@ -2362,16 +2290,16 @@
         <v/>
       </c>
       <c r="P23" s="8" t="n">
-        <v>0.17927</v>
+        <v>0.17746</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>0.03612</v>
+        <v>0.03655</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>0.00147</v>
+        <v>0.00175</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>0.02873</v>
+        <v>0.0297</v>
       </c>
       <c r="T23" s="8" t="n">
         <v>0.09376</v>
@@ -2386,13 +2314,13 @@
         <v>0.14607</v>
       </c>
       <c r="X23" s="8" t="n">
-        <v>0.00389</v>
+        <v>0.00386</v>
       </c>
       <c r="Y23" s="8" t="n">
-        <v>0.1201252988195419</v>
+        <v>0.1206673122952964</v>
       </c>
       <c r="Z23" s="8" t="n">
-        <v>0.1150021529390503</v>
+        <v>0.1155210504339684</v>
       </c>
     </row>
     <row r="24">
@@ -2406,11 +2334,7 @@
           <t>ATL</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C24" s="2" t="n"/>
       <c r="D24" s="5" t="n">
         <v>636.7</v>
       </c>
@@ -2459,16 +2383,16 @@
         <v/>
       </c>
       <c r="P24" s="8" t="n">
-        <v>0.11691</v>
+        <v>0.11702</v>
       </c>
       <c r="Q24" s="8" t="n">
-        <v>0.05002</v>
+        <v>0.04952</v>
       </c>
       <c r="R24" s="8" t="n">
-        <v>0.00106</v>
+        <v>0.00159</v>
       </c>
       <c r="S24" s="8" t="n">
-        <v>0.04779</v>
+        <v>0.0474</v>
       </c>
       <c r="T24" s="8" t="n">
         <v>0.11183</v>
@@ -2486,10 +2410,10 @@
         <v>0.00144</v>
       </c>
       <c r="Y24" s="8" t="n">
-        <v>0.1304079096905565</v>
+        <v>0.1310147578828488</v>
       </c>
       <c r="Z24" s="8" t="n">
-        <v>0.1370584690275515</v>
+        <v>0.1376962653419398</v>
       </c>
     </row>
     <row r="25">
@@ -2503,11 +2427,7 @@
           <t>OAK</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C25" s="2" t="n"/>
       <c r="D25" s="5" t="n">
         <v>630.1</v>
       </c>
@@ -2556,16 +2476,16 @@
         <v/>
       </c>
       <c r="P25" s="8" t="n">
-        <v>0.1167</v>
+        <v>0.11416</v>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>0.05089</v>
+        <v>0.04894</v>
       </c>
       <c r="R25" s="8" t="n">
-        <v>0.00196</v>
+        <v>0.00234</v>
       </c>
       <c r="S25" s="8" t="n">
-        <v>0.04621</v>
+        <v>0.04986</v>
       </c>
       <c r="T25" s="8" t="n">
         <v>0.09322</v>
@@ -2580,13 +2500,13 @@
         <v>0.27187</v>
       </c>
       <c r="X25" s="8" t="n">
-        <v>0.0111</v>
+        <v>0.01097</v>
       </c>
       <c r="Y25" s="8" t="n">
-        <v>0.1317495293660145</v>
+        <v>0.1320226496966209</v>
       </c>
       <c r="Z25" s="8" t="n">
-        <v>0.1518455588623568</v>
+        <v>0.1521603388045483</v>
       </c>
     </row>
     <row r="26">
@@ -2600,11 +2520,7 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Catcher - Primary</t>
-        </is>
-      </c>
+      <c r="C26" s="2" t="n"/>
       <c r="D26" s="5" t="n">
         <v>627</v>
       </c>
@@ -2653,16 +2569,16 @@
         <v/>
       </c>
       <c r="P26" s="8" t="n">
-        <v>0.1461</v>
+        <v>0.14537</v>
       </c>
       <c r="Q26" s="8" t="n">
-        <v>0.03735</v>
+        <v>0.039</v>
       </c>
       <c r="R26" s="8" t="n">
-        <v>0.00134</v>
+        <v>0.00154</v>
       </c>
       <c r="S26" s="8" t="n">
-        <v>0.02886</v>
+        <v>0.03148</v>
       </c>
       <c r="T26" s="8" t="n">
         <v>0.10017</v>
@@ -2677,13 +2593,13 @@
         <v>0.1972</v>
       </c>
       <c r="X26" s="8" t="n">
-        <v>0.01172</v>
+        <v>0.01169</v>
       </c>
       <c r="Y26" s="8" t="n">
-        <v>0.1254277727651113</v>
+        <v>0.1250184803229466</v>
       </c>
       <c r="Z26" s="8" t="n">
-        <v>0.1080323368333163</v>
+        <v>0.1076798086969994</v>
       </c>
     </row>
     <row r="27">
@@ -2697,11 +2613,7 @@
           <t>BOS</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C27" s="2" t="n"/>
       <c r="D27" s="5" t="n">
         <v>626.4</v>
       </c>
@@ -2750,16 +2662,16 @@
         <v/>
       </c>
       <c r="P27" s="8" t="n">
-        <v>0.13858</v>
+        <v>0.14208</v>
       </c>
       <c r="Q27" s="8" t="n">
-        <v>0.04909</v>
+        <v>0.0436</v>
       </c>
       <c r="R27" s="8" t="n">
-        <v>0.00843</v>
+        <v>0.009259999999999999</v>
       </c>
       <c r="S27" s="8" t="n">
-        <v>0.02885</v>
+        <v>0.02767</v>
       </c>
       <c r="T27" s="8" t="n">
         <v>0.07454</v>
@@ -2774,13 +2686,13 @@
         <v>0.24629</v>
       </c>
       <c r="X27" s="8" t="n">
-        <v>0.03918</v>
+        <v>0.0397</v>
       </c>
       <c r="Y27" s="8" t="n">
-        <v>0.1195156859297895</v>
+        <v>0.1194097821141954</v>
       </c>
       <c r="Z27" s="8" t="n">
-        <v>0.1063469467681195</v>
+        <v>0.1062527118787666</v>
       </c>
     </row>
     <row r="28">
@@ -2794,11 +2706,7 @@
           <t>TB</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C28" s="2" t="n"/>
       <c r="D28" s="5" t="n">
         <v>622.5</v>
       </c>
@@ -2847,16 +2755,16 @@
         <v/>
       </c>
       <c r="P28" s="8" t="n">
-        <v>0.1488</v>
+        <v>0.14648</v>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>0.04081</v>
+        <v>0.04311</v>
       </c>
       <c r="R28" s="8" t="n">
-        <v>0.00154</v>
+        <v>0.0018</v>
       </c>
       <c r="S28" s="8" t="n">
-        <v>0.0368</v>
+        <v>0.03674</v>
       </c>
       <c r="T28" s="8" t="n">
         <v>0.09927</v>
@@ -2871,13 +2779,13 @@
         <v>0.24651</v>
       </c>
       <c r="X28" s="8" t="n">
-        <v>0.00288</v>
+        <v>0.00285</v>
       </c>
       <c r="Y28" s="8" t="n">
-        <v>0.1164604266728232</v>
+        <v>0.1169859039974925</v>
       </c>
       <c r="Z28" s="8" t="n">
-        <v>0.123723013623258</v>
+        <v>0.1242812602316223</v>
       </c>
     </row>
     <row r="29">
@@ -2891,11 +2799,7 @@
           <t>DET</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C29" s="2" t="n"/>
       <c r="D29" s="5" t="n">
         <v>621.4</v>
       </c>
@@ -2944,16 +2848,16 @@
         <v/>
       </c>
       <c r="P29" s="8" t="n">
-        <v>0.13743</v>
+        <v>0.13921</v>
       </c>
       <c r="Q29" s="8" t="n">
-        <v>0.04412</v>
+        <v>0.0433</v>
       </c>
       <c r="R29" s="8" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.00796</v>
       </c>
       <c r="S29" s="8" t="n">
-        <v>0.02891</v>
+        <v>0.02958</v>
       </c>
       <c r="T29" s="8" t="n">
         <v>0.12728</v>
@@ -2968,13 +2872,13 @@
         <v>0.15307</v>
       </c>
       <c r="X29" s="8" t="n">
-        <v>0.0179</v>
+        <v>0.01801</v>
       </c>
       <c r="Y29" s="8" t="n">
-        <v>0.1339483182450487</v>
+        <v>0.1344348915759913</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>0.1058357082430014</v>
+        <v>0.1062201612452277</v>
       </c>
     </row>
     <row r="30">
@@ -2988,11 +2892,7 @@
           <t>PHI</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C30" s="2" t="n"/>
       <c r="D30" s="5" t="n">
         <v>621.2</v>
       </c>
@@ -3041,16 +2941,16 @@
         <v/>
       </c>
       <c r="P30" s="8" t="n">
-        <v>0.09801</v>
+        <v>0.09617000000000001</v>
       </c>
       <c r="Q30" s="8" t="n">
-        <v>0.03609</v>
+        <v>0.03752</v>
       </c>
       <c r="R30" s="8" t="n">
-        <v>0.00107</v>
+        <v>0.00156</v>
       </c>
       <c r="S30" s="8" t="n">
-        <v>0.06174</v>
+        <v>0.06181</v>
       </c>
       <c r="T30" s="8" t="n">
         <v>0.14883</v>
@@ -3065,13 +2965,13 @@
         <v>0.29076</v>
       </c>
       <c r="X30" s="8" t="n">
-        <v>0.00762</v>
+        <v>0.00756</v>
       </c>
       <c r="Y30" s="8" t="n">
-        <v>0.1413977977449429</v>
+        <v>0.1423728272751787</v>
       </c>
       <c r="Z30" s="8" t="n">
-        <v>0.1443505853409703</v>
+        <v>0.1453459762569459</v>
       </c>
     </row>
     <row r="33">
@@ -3199,13 +3099,9 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C35" s="2" t="n"/>
       <c r="D35" s="5" t="n">
-        <v>213.1</v>
+        <v>214.3</v>
       </c>
       <c r="E35" s="6">
         <f>D35*N35</f>
@@ -3244,7 +3140,7 @@
         <v/>
       </c>
       <c r="N35" s="8" t="n">
-        <v>4.131</v>
+        <v>4.149</v>
       </c>
       <c r="O35" s="8" t="n">
         <v>0.22256</v>
@@ -3253,19 +3149,19 @@
         <v>0.05642</v>
       </c>
       <c r="Q35" s="8" t="n">
-        <v>0.02109</v>
+        <v>0.02063</v>
       </c>
       <c r="R35" s="8" t="n">
-        <v>0.16703</v>
+        <v>0.16886</v>
       </c>
       <c r="S35" s="8" t="n">
-        <v>0.03934</v>
+        <v>0.03954</v>
       </c>
       <c r="T35" s="8" t="n">
-        <v>0.00315</v>
+        <v>0.00459</v>
       </c>
       <c r="U35" s="8" t="n">
-        <v>3.60444</v>
+        <v>3.68534</v>
       </c>
     </row>
     <row r="36">
@@ -3279,13 +3175,9 @@
           <t>MIA</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C36" s="2" t="n"/>
       <c r="D36" s="5" t="n">
-        <v>198.6</v>
+        <v>198.5</v>
       </c>
       <c r="E36" s="6">
         <f>D36*N36</f>
@@ -3324,7 +3216,7 @@
         <v/>
       </c>
       <c r="N36" s="8" t="n">
-        <v>4.192</v>
+        <v>4.196</v>
       </c>
       <c r="O36" s="8" t="n">
         <v>0.19525</v>
@@ -3333,19 +3225,19 @@
         <v>0.0675</v>
       </c>
       <c r="Q36" s="8" t="n">
-        <v>0.02624</v>
+        <v>0.02625</v>
       </c>
       <c r="R36" s="8" t="n">
-        <v>0.15207</v>
+        <v>0.15274</v>
       </c>
       <c r="S36" s="8" t="n">
-        <v>0.04551</v>
+        <v>0.0454</v>
       </c>
       <c r="T36" s="8" t="n">
-        <v>0.00402</v>
+        <v>0.00407</v>
       </c>
       <c r="U36" s="8" t="n">
-        <v>4.04033</v>
+        <v>4.0536</v>
       </c>
     </row>
     <row r="37">
@@ -3359,13 +3251,9 @@
           <t>NYM</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C37" s="2" t="n"/>
       <c r="D37" s="5" t="n">
-        <v>190.5</v>
+        <v>190.8</v>
       </c>
       <c r="E37" s="6">
         <f>D37*N37</f>
@@ -3404,7 +3292,7 @@
         <v/>
       </c>
       <c r="N37" s="8" t="n">
-        <v>4.187</v>
+        <v>4.178</v>
       </c>
       <c r="O37" s="8" t="n">
         <v>0.26058</v>
@@ -3413,19 +3301,19 @@
         <v>0.09081</v>
       </c>
       <c r="Q37" s="8" t="n">
-        <v>0.02161</v>
+        <v>0.02106</v>
       </c>
       <c r="R37" s="8" t="n">
-        <v>0.1359</v>
+        <v>0.1335</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>0.03576</v>
+        <v>0.03692</v>
       </c>
       <c r="T37" s="8" t="n">
-        <v>0.00254</v>
+        <v>0.00292</v>
       </c>
       <c r="U37" s="8" t="n">
-        <v>3.50547</v>
+        <v>3.4797</v>
       </c>
     </row>
     <row r="38">
@@ -3439,13 +3327,9 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C38" s="2" t="n"/>
       <c r="D38" s="5" t="n">
-        <v>183.4</v>
+        <v>186.4</v>
       </c>
       <c r="E38" s="6">
         <f>D38*N38</f>
@@ -3484,7 +3368,7 @@
         <v/>
       </c>
       <c r="N38" s="8" t="n">
-        <v>4.291</v>
+        <v>4.306</v>
       </c>
       <c r="O38" s="8" t="n">
         <v>0.16701</v>
@@ -3493,19 +3377,19 @@
         <v>0.0849</v>
       </c>
       <c r="Q38" s="8" t="n">
-        <v>0.0206</v>
+        <v>0.02037</v>
       </c>
       <c r="R38" s="8" t="n">
-        <v>0.16803</v>
+        <v>0.17137</v>
       </c>
       <c r="S38" s="8" t="n">
-        <v>0.03818</v>
+        <v>0.03658</v>
       </c>
       <c r="T38" s="8" t="n">
-        <v>0.00298</v>
+        <v>0.00377</v>
       </c>
       <c r="U38" s="8" t="n">
-        <v>4.05009</v>
+        <v>4.09268</v>
       </c>
     </row>
     <row r="39">
@@ -3519,13 +3403,9 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C39" s="2" t="n"/>
       <c r="D39" s="5" t="n">
-        <v>181.9</v>
+        <v>185.6</v>
       </c>
       <c r="E39" s="6">
         <f>D39*N39</f>
@@ -3573,19 +3453,19 @@
         <v>0.06342</v>
       </c>
       <c r="Q39" s="8" t="n">
-        <v>0.03523</v>
+        <v>0.03286</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>0.16246</v>
+        <v>0.16221</v>
       </c>
       <c r="S39" s="8" t="n">
-        <v>0.04488</v>
+        <v>0.0469</v>
       </c>
       <c r="T39" s="8" t="n">
-        <v>0.00354</v>
+        <v>0.00406</v>
       </c>
       <c r="U39" s="8" t="n">
-        <v>4.58968</v>
+        <v>4.54391</v>
       </c>
     </row>
     <row r="40">
@@ -3599,13 +3479,9 @@
           <t>PHI</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C40" s="2" t="n"/>
       <c r="D40" s="5" t="n">
-        <v>178.4</v>
+        <v>177.5</v>
       </c>
       <c r="E40" s="6">
         <f>D40*N40</f>
@@ -3644,7 +3520,7 @@
         <v/>
       </c>
       <c r="N40" s="8" t="n">
-        <v>4.069</v>
+        <v>4.082</v>
       </c>
       <c r="O40" s="8" t="n">
         <v>0.24571</v>
@@ -3653,19 +3529,19 @@
         <v>0.0568</v>
       </c>
       <c r="Q40" s="8" t="n">
-        <v>0.01812</v>
+        <v>0.01995</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>0.16204</v>
+        <v>0.16146</v>
       </c>
       <c r="S40" s="8" t="n">
-        <v>0.0386</v>
+        <v>0.03927</v>
       </c>
       <c r="T40" s="8" t="n">
-        <v>0.00213</v>
+        <v>0.00238</v>
       </c>
       <c r="U40" s="8" t="n">
-        <v>3.24158</v>
+        <v>3.35609</v>
       </c>
     </row>
     <row r="41">
@@ -3679,13 +3555,9 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>End-of-Rotation Starter (SP4-5)</t>
-        </is>
-      </c>
+      <c r="C41" s="2" t="n"/>
       <c r="D41" s="5" t="n">
-        <v>173.2</v>
+        <v>176.3</v>
       </c>
       <c r="E41" s="6">
         <f>D41*N41</f>
@@ -3724,7 +3596,7 @@
         <v/>
       </c>
       <c r="N41" s="8" t="n">
-        <v>4.283</v>
+        <v>4.293</v>
       </c>
       <c r="O41" s="8" t="n">
         <v>0.20666</v>
@@ -3733,19 +3605,19 @@
         <v>0.07776</v>
       </c>
       <c r="Q41" s="8" t="n">
-        <v>0.03388</v>
+        <v>0.03621</v>
       </c>
       <c r="R41" s="8" t="n">
-        <v>0.14875</v>
+        <v>0.14829</v>
       </c>
       <c r="S41" s="8" t="n">
-        <v>0.04841</v>
+        <v>0.04779</v>
       </c>
       <c r="T41" s="8" t="n">
-        <v>0.0029</v>
+        <v>0.00321</v>
       </c>
       <c r="U41" s="8" t="n">
-        <v>4.56966</v>
+        <v>4.68366</v>
       </c>
     </row>
     <row r="42">
@@ -3759,13 +3631,9 @@
           <t>KC</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C42" s="2" t="n"/>
       <c r="D42" s="5" t="n">
-        <v>173</v>
+        <v>175.7</v>
       </c>
       <c r="E42" s="6">
         <f>D42*N42</f>
@@ -3804,7 +3672,7 @@
         <v/>
       </c>
       <c r="N42" s="8" t="n">
-        <v>4.148</v>
+        <v>4.142</v>
       </c>
       <c r="O42" s="8" t="n">
         <v>0.20002</v>
@@ -3813,19 +3681,19 @@
         <v>0.06744</v>
       </c>
       <c r="Q42" s="8" t="n">
-        <v>0.03138</v>
+        <v>0.03093</v>
       </c>
       <c r="R42" s="8" t="n">
-        <v>0.13852</v>
+        <v>0.1375</v>
       </c>
       <c r="S42" s="8" t="n">
-        <v>0.04814</v>
+        <v>0.04817</v>
       </c>
       <c r="T42" s="8" t="n">
-        <v>0.00522</v>
+        <v>0.00557</v>
       </c>
       <c r="U42" s="8" t="n">
-        <v>4.1109</v>
+        <v>4.08053</v>
       </c>
     </row>
     <row r="43">
@@ -3839,13 +3707,9 @@
           <t>PIT</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C43" s="2" t="n"/>
       <c r="D43" s="5" t="n">
-        <v>169.8</v>
+        <v>172.5</v>
       </c>
       <c r="E43" s="6">
         <f>D43*N43</f>
@@ -3884,7 +3748,7 @@
         <v/>
       </c>
       <c r="N43" s="8" t="n">
-        <v>3.961</v>
+        <v>3.981</v>
       </c>
       <c r="O43" s="8" t="n">
         <v>0.29012</v>
@@ -3893,19 +3757,19 @@
         <v>0.06511</v>
       </c>
       <c r="Q43" s="8" t="n">
-        <v>0.02063</v>
+        <v>0.0228</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>0.12723</v>
+        <v>0.12776</v>
       </c>
       <c r="S43" s="8" t="n">
-        <v>0.03713</v>
+        <v>0.03736</v>
       </c>
       <c r="T43" s="8" t="n">
-        <v>0.00274</v>
+        <v>0.00356</v>
       </c>
       <c r="U43" s="8" t="n">
-        <v>2.83098</v>
+        <v>2.98867</v>
       </c>
     </row>
     <row r="44">
@@ -3919,13 +3783,9 @@
           <t>HOU</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C44" s="2" t="n"/>
       <c r="D44" s="5" t="n">
-        <v>166.7</v>
+        <v>166.9</v>
       </c>
       <c r="E44" s="6">
         <f>D44*N44</f>
@@ -3964,7 +3824,7 @@
         <v/>
       </c>
       <c r="N44" s="8" t="n">
-        <v>4.121</v>
+        <v>4.103</v>
       </c>
       <c r="O44" s="8" t="n">
         <v>0.26634</v>
@@ -3973,39 +3833,35 @@
         <v>0.08998</v>
       </c>
       <c r="Q44" s="8" t="n">
-        <v>0.0213</v>
+        <v>0.02009</v>
       </c>
       <c r="R44" s="8" t="n">
-        <v>0.14089</v>
+        <v>0.13948</v>
       </c>
       <c r="S44" s="8" t="n">
-        <v>0.02828</v>
+        <v>0.02789</v>
       </c>
       <c r="T44" s="8" t="n">
-        <v>0.00323</v>
+        <v>0.00302</v>
       </c>
       <c r="U44" s="8" t="n">
-        <v>3.22958</v>
+        <v>3.118</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Sean Manaea</t>
+          <t>Garrett Crochet</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>NYM</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>End-of-Rotation Starter (SP4-5)</t>
-        </is>
-      </c>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n"/>
       <c r="D45" s="5" t="n">
-        <v>166</v>
+        <v>165.8</v>
       </c>
       <c r="E45" s="6">
         <f>D45*N45</f>
@@ -4044,48 +3900,44 @@
         <v/>
       </c>
       <c r="N45" s="8" t="n">
-        <v>4.201</v>
+        <v>4.021</v>
       </c>
       <c r="O45" s="8" t="n">
-        <v>0.24101</v>
+        <v>0.30629</v>
       </c>
       <c r="P45" s="8" t="n">
-        <v>0.07418</v>
+        <v>0.06553</v>
       </c>
       <c r="Q45" s="8" t="n">
-        <v>0.03999</v>
+        <v>0.02877</v>
       </c>
       <c r="R45" s="8" t="n">
-        <v>0.12796</v>
+        <v>0.13146</v>
       </c>
       <c r="S45" s="8" t="n">
-        <v>0.04591</v>
+        <v>0.03912</v>
       </c>
       <c r="T45" s="8" t="n">
-        <v>0.00344</v>
+        <v>0.0025</v>
       </c>
       <c r="U45" s="8" t="n">
-        <v>4.41162</v>
+        <v>3.30921</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Framber Valdez</t>
+          <t>Sean Manaea</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n"/>
       <c r="D46" s="5" t="n">
-        <v>164.4</v>
+        <v>165.6</v>
       </c>
       <c r="E46" s="6">
         <f>D46*N46</f>
@@ -4124,48 +3976,44 @@
         <v/>
       </c>
       <c r="N46" s="8" t="n">
-        <v>4.21</v>
+        <v>4.209</v>
       </c>
       <c r="O46" s="8" t="n">
-        <v>0.2228</v>
+        <v>0.24101</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>0.08168</v>
+        <v>0.07418</v>
       </c>
       <c r="Q46" s="8" t="n">
-        <v>0.01838</v>
+        <v>0.03819</v>
       </c>
       <c r="R46" s="8" t="n">
-        <v>0.15138</v>
+        <v>0.12973</v>
       </c>
       <c r="S46" s="8" t="n">
-        <v>0.04148</v>
+        <v>0.0473</v>
       </c>
       <c r="T46" s="8" t="n">
-        <v>0.00284</v>
+        <v>0.00341</v>
       </c>
       <c r="U46" s="8" t="n">
-        <v>3.66027</v>
+        <v>4.39733</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Garrett Crochet</t>
+          <t>Framber Valdez</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>BOS</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n"/>
       <c r="D47" s="5" t="n">
-        <v>163.7</v>
+        <v>165.4</v>
       </c>
       <c r="E47" s="6">
         <f>D47*N47</f>
@@ -4204,28 +4052,28 @@
         <v/>
       </c>
       <c r="N47" s="8" t="n">
-        <v>4.014</v>
+        <v>4.221</v>
       </c>
       <c r="O47" s="8" t="n">
-        <v>0.30629</v>
+        <v>0.2228</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>0.06553</v>
+        <v>0.08168</v>
       </c>
       <c r="Q47" s="8" t="n">
-        <v>0.02932</v>
+        <v>0.01934</v>
       </c>
       <c r="R47" s="8" t="n">
-        <v>0.13205</v>
+        <v>0.15248</v>
       </c>
       <c r="S47" s="8" t="n">
-        <v>0.03687</v>
+        <v>0.04064</v>
       </c>
       <c r="T47" s="8" t="n">
-        <v>0.0023</v>
+        <v>0.00338</v>
       </c>
       <c r="U47" s="8" t="n">
-        <v>3.27204</v>
+        <v>3.73175</v>
       </c>
     </row>
     <row r="48">
@@ -4239,13 +4087,9 @@
           <t>SEA</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C48" s="2" t="n"/>
       <c r="D48" s="5" t="n">
-        <v>162.1</v>
+        <v>163.5</v>
       </c>
       <c r="E48" s="6">
         <f>D48*N48</f>
@@ -4284,7 +4128,7 @@
         <v/>
       </c>
       <c r="N48" s="8" t="n">
-        <v>3.998</v>
+        <v>4.007</v>
       </c>
       <c r="O48" s="8" t="n">
         <v>0.26736</v>
@@ -4293,19 +4137,19 @@
         <v>0.05806</v>
       </c>
       <c r="Q48" s="8" t="n">
-        <v>0.0345</v>
+        <v>0.03611</v>
       </c>
       <c r="R48" s="8" t="n">
-        <v>0.12806</v>
+        <v>0.12887</v>
       </c>
       <c r="S48" s="8" t="n">
-        <v>0.04121</v>
+        <v>0.04026</v>
       </c>
       <c r="T48" s="8" t="n">
-        <v>0.00234</v>
+        <v>0.00255</v>
       </c>
       <c r="U48" s="8" t="n">
-        <v>3.50564</v>
+        <v>3.58381</v>
       </c>
     </row>
     <row r="49">
@@ -4319,13 +4163,9 @@
           <t>PIT</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C49" s="2" t="n"/>
       <c r="D49" s="5" t="n">
-        <v>160.2</v>
+        <v>162.7</v>
       </c>
       <c r="E49" s="6">
         <f>D49*N49</f>
@@ -4364,7 +4204,7 @@
         <v/>
       </c>
       <c r="N49" s="8" t="n">
-        <v>4.288</v>
+        <v>4.313</v>
       </c>
       <c r="O49" s="8" t="n">
         <v>0.21069</v>
@@ -4373,19 +4213,19 @@
         <v>0.07349</v>
       </c>
       <c r="Q49" s="8" t="n">
-        <v>0.02862</v>
+        <v>0.02911</v>
       </c>
       <c r="R49" s="8" t="n">
-        <v>0.15226</v>
+        <v>0.15338</v>
       </c>
       <c r="S49" s="8" t="n">
-        <v>0.0464</v>
+        <v>0.04865</v>
       </c>
       <c r="T49" s="8" t="n">
-        <v>0.00383</v>
+        <v>0.00397</v>
       </c>
       <c r="U49" s="8" t="n">
-        <v>4.39618</v>
+        <v>4.53342</v>
       </c>
     </row>
     <row r="50">
@@ -4399,13 +4239,9 @@
           <t>WSH</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C50" s="2" t="n"/>
       <c r="D50" s="5" t="n">
-        <v>158.8</v>
+        <v>161</v>
       </c>
       <c r="E50" s="6">
         <f>D50*N50</f>
@@ -4444,7 +4280,7 @@
         <v/>
       </c>
       <c r="N50" s="8" t="n">
-        <v>4.291</v>
+        <v>4.308</v>
       </c>
       <c r="O50" s="8" t="n">
         <v>0.19519</v>
@@ -4453,19 +4289,19 @@
         <v>0.08477</v>
       </c>
       <c r="Q50" s="8" t="n">
-        <v>0.03949</v>
+        <v>0.04251</v>
       </c>
       <c r="R50" s="8" t="n">
-        <v>0.13996</v>
+        <v>0.13807</v>
       </c>
       <c r="S50" s="8" t="n">
-        <v>0.04231</v>
+        <v>0.0437</v>
       </c>
       <c r="T50" s="8" t="n">
-        <v>0.00406</v>
+        <v>0.00424</v>
       </c>
       <c r="U50" s="8" t="n">
-        <v>4.70877</v>
+        <v>4.8931</v>
       </c>
     </row>
     <row r="51">
@@ -4479,13 +4315,9 @@
           <t>KC</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C51" s="2" t="n"/>
       <c r="D51" s="5" t="n">
-        <v>158.7</v>
+        <v>160.7</v>
       </c>
       <c r="E51" s="6">
         <f>D51*N51</f>
@@ -4524,7 +4356,7 @@
         <v/>
       </c>
       <c r="N51" s="8" t="n">
-        <v>4.155</v>
+        <v>4.161</v>
       </c>
       <c r="O51" s="8" t="n">
         <v>0.21127</v>
@@ -4533,19 +4365,19 @@
         <v>0.07836</v>
       </c>
       <c r="Q51" s="8" t="n">
-        <v>0.02823</v>
+        <v>0.02991</v>
       </c>
       <c r="R51" s="8" t="n">
-        <v>0.14139</v>
+        <v>0.14032</v>
       </c>
       <c r="S51" s="8" t="n">
-        <v>0.04152</v>
+        <v>0.04166</v>
       </c>
       <c r="T51" s="8" t="n">
-        <v>0.00305</v>
+        <v>0.00326</v>
       </c>
       <c r="U51" s="8" t="n">
-        <v>3.84718</v>
+        <v>3.92851</v>
       </c>
     </row>
     <row r="52">
@@ -4559,13 +4391,9 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>End-of-Rotation Starter (SP4-5)</t>
-        </is>
-      </c>
+      <c r="C52" s="2" t="n"/>
       <c r="D52" s="5" t="n">
-        <v>158.6</v>
+        <v>159.6</v>
       </c>
       <c r="E52" s="6">
         <f>D52*N52</f>
@@ -4604,7 +4432,7 @@
         <v/>
       </c>
       <c r="N52" s="8" t="n">
-        <v>4.258</v>
+        <v>4.276</v>
       </c>
       <c r="O52" s="8" t="n">
         <v>0.21758</v>
@@ -4613,39 +4441,35 @@
         <v>0.10525</v>
       </c>
       <c r="Q52" s="8" t="n">
-        <v>0.02081</v>
+        <v>0.01903</v>
       </c>
       <c r="R52" s="8" t="n">
-        <v>0.13642</v>
+        <v>0.14067</v>
       </c>
       <c r="S52" s="8" t="n">
-        <v>0.04346</v>
+        <v>0.04297</v>
       </c>
       <c r="T52" s="8" t="n">
-        <v>0.00308</v>
+        <v>0.00397</v>
       </c>
       <c r="U52" s="8" t="n">
-        <v>3.83839</v>
+        <v>3.85549</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Freddy Peralta</t>
+          <t>Jeffrey Springs</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+          <t>OAK</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n"/>
       <c r="D53" s="5" t="n">
-        <v>158.5</v>
+        <v>159.2</v>
       </c>
       <c r="E53" s="6">
         <f>D53*N53</f>
@@ -4684,28 +4508,28 @@
         <v/>
       </c>
       <c r="N53" s="8" t="n">
-        <v>4.132</v>
+        <v>4.205</v>
       </c>
       <c r="O53" s="8" t="n">
-        <v>0.26165</v>
+        <v>0.21018</v>
       </c>
       <c r="P53" s="8" t="n">
-        <v>0.08762</v>
+        <v>0.0786</v>
       </c>
       <c r="Q53" s="8" t="n">
-        <v>0.02861</v>
+        <v>0.03903</v>
       </c>
       <c r="R53" s="8" t="n">
-        <v>0.12714</v>
+        <v>0.13634</v>
       </c>
       <c r="S53" s="8" t="n">
-        <v>0.0373</v>
+        <v>0.04539</v>
       </c>
       <c r="T53" s="8" t="n">
-        <v>0.003</v>
+        <v>0.00285</v>
       </c>
       <c r="U53" s="8" t="n">
-        <v>3.6085</v>
+        <v>4.42429</v>
       </c>
     </row>
     <row r="54">
@@ -4719,13 +4543,9 @@
           <t>SEA</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C54" s="2" t="n"/>
       <c r="D54" s="5" t="n">
-        <v>158.1</v>
+        <v>159.1</v>
       </c>
       <c r="E54" s="6">
         <f>D54*N54</f>
@@ -4764,7 +4584,7 @@
         <v/>
       </c>
       <c r="N54" s="8" t="n">
-        <v>3.996</v>
+        <v>4.015</v>
       </c>
       <c r="O54" s="8" t="n">
         <v>0.24713</v>
@@ -4773,39 +4593,35 @@
         <v>0.05432</v>
       </c>
       <c r="Q54" s="8" t="n">
-        <v>0.02697</v>
+        <v>0.02757</v>
       </c>
       <c r="R54" s="8" t="n">
-        <v>0.13568</v>
+        <v>0.13952</v>
       </c>
       <c r="S54" s="8" t="n">
-        <v>0.0417</v>
+        <v>0.04067</v>
       </c>
       <c r="T54" s="8" t="n">
-        <v>0.00259</v>
+        <v>0.00276</v>
       </c>
       <c r="U54" s="8" t="n">
-        <v>3.30168</v>
+        <v>3.38315</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Jesús Luzardo</t>
+          <t>Seth Lugo</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>PHI</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+          <t>KC</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n"/>
       <c r="D55" s="5" t="n">
-        <v>157.8</v>
+        <v>158.2</v>
       </c>
       <c r="E55" s="6">
         <f>D55*N55</f>
@@ -4844,48 +4660,44 @@
         <v/>
       </c>
       <c r="N55" s="8" t="n">
-        <v>4.07</v>
+        <v>4.254</v>
       </c>
       <c r="O55" s="8" t="n">
-        <v>0.28049</v>
+        <v>0.20784</v>
       </c>
       <c r="P55" s="8" t="n">
-        <v>0.07592</v>
+        <v>0.07088</v>
       </c>
       <c r="Q55" s="8" t="n">
-        <v>0.02197</v>
+        <v>0.03581</v>
       </c>
       <c r="R55" s="8" t="n">
-        <v>0.14219</v>
+        <v>0.14661</v>
       </c>
       <c r="S55" s="8" t="n">
-        <v>0.0335</v>
+        <v>0.04731</v>
       </c>
       <c r="T55" s="8" t="n">
-        <v>0.00227</v>
+        <v>0.00491</v>
       </c>
       <c r="U55" s="8" t="n">
-        <v>3.17118</v>
+        <v>4.59133</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Yusei Kikuchi</t>
+          <t>George Kirby</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>LAA</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n"/>
       <c r="D56" s="5" t="n">
-        <v>156.4</v>
+        <v>157.8</v>
       </c>
       <c r="E56" s="6">
         <f>D56*N56</f>
@@ -4924,48 +4736,44 @@
         <v/>
       </c>
       <c r="N56" s="8" t="n">
-        <v>4.202</v>
+        <v>4.102</v>
       </c>
       <c r="O56" s="8" t="n">
-        <v>0.24802</v>
+        <v>0.22773</v>
       </c>
       <c r="P56" s="8" t="n">
-        <v>0.08527</v>
+        <v>0.04721</v>
       </c>
       <c r="Q56" s="8" t="n">
-        <v>0.03067</v>
+        <v>0.02597</v>
       </c>
       <c r="R56" s="8" t="n">
-        <v>0.13474</v>
+        <v>0.16155</v>
       </c>
       <c r="S56" s="8" t="n">
-        <v>0.04612</v>
+        <v>0.04328</v>
       </c>
       <c r="T56" s="8" t="n">
-        <v>0.00271</v>
+        <v>0.00344</v>
       </c>
       <c r="U56" s="8" t="n">
-        <v>4.05927</v>
+        <v>3.74893</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>George Kirby</t>
+          <t>Jesús Luzardo</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>SEA</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="n"/>
       <c r="D57" s="5" t="n">
-        <v>156.4</v>
+        <v>157.2</v>
       </c>
       <c r="E57" s="6">
         <f>D57*N57</f>
@@ -5004,48 +4812,44 @@
         <v/>
       </c>
       <c r="N57" s="8" t="n">
-        <v>4.092</v>
+        <v>4.077</v>
       </c>
       <c r="O57" s="8" t="n">
-        <v>0.22773</v>
+        <v>0.28049</v>
       </c>
       <c r="P57" s="8" t="n">
-        <v>0.04721</v>
+        <v>0.07592</v>
       </c>
       <c r="Q57" s="8" t="n">
-        <v>0.0248</v>
+        <v>0.02302</v>
       </c>
       <c r="R57" s="8" t="n">
-        <v>0.16157</v>
+        <v>0.14091</v>
       </c>
       <c r="S57" s="8" t="n">
-        <v>0.04265</v>
+        <v>0.03492</v>
       </c>
       <c r="T57" s="8" t="n">
-        <v>0.0035</v>
+        <v>0.00238</v>
       </c>
       <c r="U57" s="8" t="n">
-        <v>3.66944</v>
+        <v>3.24807</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Seth Lugo</t>
+          <t>Freddy Peralta</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+          <t>TB</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n"/>
       <c r="D58" s="5" t="n">
-        <v>156.1</v>
+        <v>156.3</v>
       </c>
       <c r="E58" s="6">
         <f>D58*N58</f>
@@ -5084,48 +4888,44 @@
         <v/>
       </c>
       <c r="N58" s="8" t="n">
-        <v>4.251</v>
+        <v>4.145</v>
       </c>
       <c r="O58" s="8" t="n">
-        <v>0.20784</v>
+        <v>0.26165</v>
       </c>
       <c r="P58" s="8" t="n">
-        <v>0.07088</v>
+        <v>0.08762</v>
       </c>
       <c r="Q58" s="8" t="n">
-        <v>0.03395</v>
+        <v>0.02812</v>
       </c>
       <c r="R58" s="8" t="n">
-        <v>0.14697</v>
+        <v>0.12887</v>
       </c>
       <c r="S58" s="8" t="n">
-        <v>0.04837</v>
+        <v>0.03802</v>
       </c>
       <c r="T58" s="8" t="n">
-        <v>0.00483</v>
+        <v>0.00331</v>
       </c>
       <c r="U58" s="8" t="n">
-        <v>4.52825</v>
+        <v>3.65415</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Jeffrey Springs</t>
+          <t>Max Fried</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>OAK</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n"/>
       <c r="D59" s="5" t="n">
-        <v>155.1</v>
+        <v>155.8</v>
       </c>
       <c r="E59" s="6">
         <f>D59*N59</f>
@@ -5164,28 +4964,28 @@
         <v/>
       </c>
       <c r="N59" s="8" t="n">
-        <v>4.164</v>
+        <v>4.041</v>
       </c>
       <c r="O59" s="8" t="n">
-        <v>0.21018</v>
+        <v>0.23617</v>
       </c>
       <c r="P59" s="8" t="n">
-        <v>0.0786</v>
+        <v>0.06723</v>
       </c>
       <c r="Q59" s="8" t="n">
-        <v>0.03713</v>
+        <v>0.01702</v>
       </c>
       <c r="R59" s="8" t="n">
-        <v>0.134</v>
+        <v>0.14871</v>
       </c>
       <c r="S59" s="8" t="n">
-        <v>0.04349</v>
+        <v>0.03565</v>
       </c>
       <c r="T59" s="8" t="n">
         <v>0.00217</v>
       </c>
       <c r="U59" s="8" t="n">
-        <v>4.17555</v>
+        <v>3.02681</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild 2027 projections (run 36902482834)
Verification PASSED.

Regenerated by .github/workflows/refresh-projections.yml.
Verification and the full baseline audit are in the run summary:
https://github.com/pmammino/DFSSimsFull/actions/runs/36902482834
</commit_message>
<xml_diff>
--- a/out/mlb_2027_what_if.xlsx
+++ b/out/mlb_2027_what_if.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="What-If" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What-If" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -660,11 +660,7 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C6" s="2" t="n"/>
       <c r="D6" s="5" t="n">
         <v>760</v>
       </c>
@@ -713,37 +709,37 @@
         <v/>
       </c>
       <c r="P6" s="8" t="n">
-        <v>0.1154316087404422</v>
+        <v>0.11547</v>
       </c>
       <c r="Q6" s="8" t="n">
-        <v>0.0462379454665884</v>
+        <v>0.04625</v>
       </c>
       <c r="R6" s="8" t="n">
-        <v>0.0026209303255674</v>
+        <v>0.00263</v>
       </c>
       <c r="S6" s="8" t="n">
-        <v>0.0501567119074266</v>
+        <v>0.05016</v>
       </c>
       <c r="T6" s="8" t="n">
-        <v>0.1111412589760419</v>
+        <v>0.11112</v>
       </c>
       <c r="U6" s="8" t="n">
-        <v>0.0084858635863501</v>
+        <v>0.008489999999999999</v>
       </c>
       <c r="V6" s="8" t="n">
-        <v>0.0060899960457531</v>
+        <v>0.00609</v>
       </c>
       <c r="W6" s="8" t="n">
-        <v>0.2394914934582596</v>
+        <v>0.23936</v>
       </c>
       <c r="X6" s="8" t="n">
         <v>0.00351</v>
       </c>
       <c r="Y6" s="8" t="n">
-        <v>0.131109349566687</v>
+        <v>0.1311443884698552</v>
       </c>
       <c r="Z6" s="8" t="n">
-        <v>0.1395957001931852</v>
+        <v>0.1396361774803498</v>
       </c>
     </row>
     <row r="7">
@@ -757,11 +753,7 @@
           <t>LAA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C7" s="2" t="n"/>
       <c r="D7" s="5" t="n">
         <v>733.8</v>
       </c>
@@ -810,37 +802,37 @@
         <v/>
       </c>
       <c r="P7" s="8" t="n">
-        <v>0.1126784726035775</v>
+        <v>0.11271</v>
       </c>
       <c r="Q7" s="8" t="n">
-        <v>0.051338019139698</v>
+        <v>0.05135</v>
       </c>
       <c r="R7" s="8" t="n">
-        <v>0.0033988302336306</v>
+        <v>0.0034</v>
       </c>
       <c r="S7" s="8" t="n">
-        <v>0.0469321706410692</v>
+        <v>0.04693</v>
       </c>
       <c r="T7" s="8" t="n">
-        <v>0.0753212350183647</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="U7" s="8" t="n">
-        <v>0.0260929691537631</v>
+        <v>0.0261</v>
       </c>
       <c r="V7" s="8" t="n">
-        <v>0.0036993728049062</v>
+        <v>0.0037</v>
       </c>
       <c r="W7" s="8" t="n">
-        <v>0.2726727914749802</v>
+        <v>0.27253</v>
       </c>
       <c r="X7" s="8" t="n">
         <v>0.03728</v>
       </c>
       <c r="Y7" s="8" t="n">
-        <v>0.1306702740480629</v>
+        <v>0.1307057166175846</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>0.1112768732755967</v>
+        <v>0.1113103729849251</v>
       </c>
     </row>
     <row r="8">
@@ -854,11 +846,7 @@
           <t>WSH</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C8" s="2" t="n"/>
       <c r="D8" s="5" t="n">
         <v>727.5</v>
       </c>
@@ -907,37 +895,37 @@
         <v/>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0.1198384715382225</v>
+        <v>0.11988</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>0.0458973657420166</v>
+        <v>0.04591</v>
       </c>
       <c r="R8" s="8" t="n">
-        <v>0.0031415849804145</v>
+        <v>0.00315</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>0.0451162212703495</v>
+        <v>0.04512</v>
       </c>
       <c r="T8" s="8" t="n">
-        <v>0.1324798463289067</v>
+        <v>0.13246</v>
       </c>
       <c r="U8" s="8" t="n">
-        <v>0.0055698855718849</v>
+        <v>0.00557</v>
       </c>
       <c r="V8" s="8" t="n">
-        <v>0.0042876452747517</v>
+        <v>0.00429</v>
       </c>
       <c r="W8" s="8" t="n">
-        <v>0.300762874906709</v>
+        <v>0.30062</v>
       </c>
       <c r="X8" s="8" t="n">
         <v>0.02916</v>
       </c>
       <c r="Y8" s="8" t="n">
-        <v>0.1315406284895754</v>
+        <v>0.1315714761985192</v>
       </c>
       <c r="Z8" s="8" t="n">
-        <v>0.1190238527006049</v>
+        <v>0.1190587159930348</v>
       </c>
     </row>
     <row r="9">
@@ -951,11 +939,7 @@
           <t>MIA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C9" s="2" t="n"/>
       <c r="D9" s="5" t="n">
         <v>725.6</v>
       </c>
@@ -1004,37 +988,37 @@
         <v/>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0.173228141304772</v>
+        <v>0.17326</v>
       </c>
       <c r="Q9" s="8" t="n">
-        <v>0.0414950966713211</v>
+        <v>0.0415</v>
       </c>
       <c r="R9" s="8" t="n">
-        <v>0.005149205898074</v>
+        <v>0.00515</v>
       </c>
       <c r="S9" s="8" t="n">
-        <v>0.0208209788659798</v>
+        <v>0.02082</v>
       </c>
       <c r="T9" s="8" t="n">
-        <v>0.0638246954777765</v>
+        <v>0.06381000000000001</v>
       </c>
       <c r="U9" s="8" t="n">
-        <v>0.0075023547974578</v>
+        <v>0.0075</v>
       </c>
       <c r="V9" s="8" t="n">
-        <v>0.0090182437458341</v>
+        <v>0.00902</v>
       </c>
       <c r="W9" s="8" t="n">
-        <v>0.1502993487391389</v>
+        <v>0.1502</v>
       </c>
       <c r="X9" s="8" t="n">
         <v>0.03639</v>
       </c>
       <c r="Y9" s="8" t="n">
-        <v>0.1159977375820328</v>
+        <v>0.1160265509827313</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>0.1038145296585654</v>
+        <v>0.1038432404446151</v>
       </c>
     </row>
     <row r="10">
@@ -1048,11 +1032,7 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C10" s="2" t="n"/>
       <c r="D10" s="5" t="n">
         <v>720.8</v>
       </c>
@@ -1101,37 +1081,37 @@
         <v/>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0.1134100172015939</v>
+        <v>0.11344</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>0.0421713933681382</v>
+        <v>0.04218</v>
       </c>
       <c r="R10" s="8" t="n">
-        <v>0.0030432790038211</v>
+        <v>0.00305</v>
       </c>
       <c r="S10" s="8" t="n">
-        <v>0.0404668090632161</v>
+        <v>0.04047</v>
       </c>
       <c r="T10" s="8" t="n">
-        <v>0.09624334330328251</v>
+        <v>0.09622</v>
       </c>
       <c r="U10" s="8" t="n">
-        <v>0.0048124497891999</v>
+        <v>0.00481</v>
       </c>
       <c r="V10" s="8" t="n">
-        <v>0.007193011374728</v>
+        <v>0.00719</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>0.2657966415056796</v>
+        <v>0.26566</v>
       </c>
       <c r="X10" s="8" t="n">
         <v>0.01709</v>
       </c>
       <c r="Y10" s="8" t="n">
-        <v>0.1225657875876504</v>
+        <v>0.1225934232293224</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>0.1245586497010641</v>
+        <v>0.1245955523456179</v>
       </c>
     </row>
     <row r="11">
@@ -1145,11 +1125,7 @@
           <t>WSH</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C11" s="2" t="n"/>
       <c r="D11" s="5" t="n">
         <v>691.6</v>
       </c>
@@ -1198,37 +1174,37 @@
         <v/>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0.1439902872503698</v>
+        <v>0.14403</v>
       </c>
       <c r="Q11" s="8" t="n">
-        <v>0.0479102290515192</v>
+        <v>0.04792</v>
       </c>
       <c r="R11" s="8" t="n">
-        <v>0.0137823936877652</v>
+        <v>0.01378</v>
       </c>
       <c r="S11" s="8" t="n">
-        <v>0.0303285688660164</v>
+        <v>0.03033</v>
       </c>
       <c r="T11" s="8" t="n">
-        <v>0.0620657801838578</v>
+        <v>0.06204</v>
       </c>
       <c r="U11" s="8" t="n">
-        <v>0.009764374478881999</v>
+        <v>0.009769999999999999</v>
       </c>
       <c r="V11" s="8" t="n">
-        <v>0.009551146771735301</v>
+        <v>0.009549999999999999</v>
       </c>
       <c r="W11" s="8" t="n">
-        <v>0.1913471612405931</v>
+        <v>0.19123</v>
       </c>
       <c r="X11" s="8" t="n">
         <v>0.02656</v>
       </c>
       <c r="Y11" s="8" t="n">
-        <v>0.1162667275458699</v>
+        <v>0.116295645916114</v>
       </c>
       <c r="Z11" s="8" t="n">
-        <v>0.1138530505072955</v>
+        <v>0.1138878277062259</v>
       </c>
     </row>
     <row r="12">
@@ -1242,11 +1218,7 @@
           <t>WSH</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C12" s="2" t="n"/>
       <c r="D12" s="5" t="n">
         <v>690.5</v>
       </c>
@@ -1295,37 +1267,37 @@
         <v/>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0.1331802567061698</v>
+        <v>0.13322</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>0.0447965832404903</v>
+        <v>0.04481</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>0.007546903318134</v>
+        <v>0.00755</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>0.0372121575119224</v>
+        <v>0.03722</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>0.06425208276199219</v>
+        <v>0.06424000000000001</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>0.0218781459128366</v>
+        <v>0.02188</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>0.0063164191352833</v>
+        <v>0.00631</v>
       </c>
       <c r="W12" s="8" t="n">
-        <v>0.2153442977137196</v>
+        <v>0.21522</v>
       </c>
       <c r="X12" s="8" t="n">
         <v>0.04791</v>
       </c>
       <c r="Y12" s="8" t="n">
-        <v>0.1303862612102571</v>
+        <v>0.1304267757380806</v>
       </c>
       <c r="Z12" s="8" t="n">
-        <v>0.1109909828726225</v>
+        <v>0.1110162084477117</v>
       </c>
     </row>
     <row r="13">
@@ -1339,11 +1311,7 @@
           <t>BAL</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C13" s="2" t="n"/>
       <c r="D13" s="5" t="n">
         <v>670.8</v>
       </c>
@@ -1392,37 +1360,37 @@
         <v/>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0.1288028811011704</v>
+        <v>0.12884</v>
       </c>
       <c r="Q13" s="8" t="n">
-        <v>0.0453500410830584</v>
+        <v>0.04536</v>
       </c>
       <c r="R13" s="8" t="n">
-        <v>0.0009595488217646</v>
+        <v>0.00096</v>
       </c>
       <c r="S13" s="8" t="n">
-        <v>0.0581458562325176</v>
+        <v>0.05815</v>
       </c>
       <c r="T13" s="8" t="n">
-        <v>0.09795258884610281</v>
+        <v>0.09793</v>
       </c>
       <c r="U13" s="8" t="n">
-        <v>0.0203915072782139</v>
+        <v>0.0204</v>
       </c>
       <c r="V13" s="8" t="n">
-        <v>0.0087929397380818</v>
+        <v>0.008789999999999999</v>
       </c>
       <c r="W13" s="8" t="n">
-        <v>0.2344274490816751</v>
+        <v>0.2343</v>
       </c>
       <c r="X13" s="8" t="n">
         <v>0.00442</v>
       </c>
       <c r="Y13" s="8" t="n">
-        <v>0.1233476294266796</v>
+        <v>0.1233803607544251</v>
       </c>
       <c r="Z13" s="8" t="n">
-        <v>0.1487536729848238</v>
+        <v>0.1487906166084317</v>
       </c>
     </row>
     <row r="14">
@@ -1436,11 +1404,7 @@
           <t>BAL</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C14" s="2" t="n"/>
       <c r="D14" s="5" t="n">
         <v>664.1</v>
       </c>
@@ -1489,37 +1453,37 @@
         <v/>
       </c>
       <c r="P14" s="8" t="n">
-        <v>0.1456511753541733</v>
+        <v>0.1457</v>
       </c>
       <c r="Q14" s="8" t="n">
-        <v>0.0470525686555999</v>
+        <v>0.04706</v>
       </c>
       <c r="R14" s="8" t="n">
-        <v>0.0060426524861461</v>
+        <v>0.00604</v>
       </c>
       <c r="S14" s="8" t="n">
-        <v>0.0293693892686431</v>
+        <v>0.02937</v>
       </c>
       <c r="T14" s="8" t="n">
-        <v>0.0956451581747773</v>
+        <v>0.09562</v>
       </c>
       <c r="U14" s="8" t="n">
-        <v>0.009341736230862799</v>
+        <v>0.009339999999999999</v>
       </c>
       <c r="V14" s="8" t="n">
-        <v>0.0049208469023935</v>
+        <v>0.00492</v>
       </c>
       <c r="W14" s="8" t="n">
-        <v>0.2302275778536174</v>
+        <v>0.2301</v>
       </c>
       <c r="X14" s="8" t="n">
         <v>0.02686</v>
       </c>
       <c r="Y14" s="8" t="n">
-        <v>0.1293389908065198</v>
+        <v>0.1293702734936025</v>
       </c>
       <c r="Z14" s="8" t="n">
-        <v>0.102311081906699</v>
+        <v>0.1023416557133602</v>
       </c>
     </row>
     <row r="15">
@@ -1533,11 +1497,7 @@
           <t>TB</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C15" s="2" t="n"/>
       <c r="D15" s="5" t="n">
         <v>661.2</v>
       </c>
@@ -1586,37 +1546,37 @@
         <v/>
       </c>
       <c r="P15" s="8" t="n">
-        <v>0.1378711867340206</v>
+        <v>0.1379</v>
       </c>
       <c r="Q15" s="8" t="n">
-        <v>0.0426791770049525</v>
+        <v>0.04269</v>
       </c>
       <c r="R15" s="8" t="n">
-        <v>0.0012961974361437</v>
+        <v>0.0013</v>
       </c>
       <c r="S15" s="8" t="n">
-        <v>0.0543635687502354</v>
+        <v>0.05437</v>
       </c>
       <c r="T15" s="8" t="n">
-        <v>0.08549756042090841</v>
+        <v>0.08548</v>
       </c>
       <c r="U15" s="8" t="n">
-        <v>0.005257309942395</v>
+        <v>0.00526</v>
       </c>
       <c r="V15" s="8" t="n">
-        <v>0.0062892021703844</v>
+        <v>0.00629</v>
       </c>
       <c r="W15" s="8" t="n">
-        <v>0.1966754163935763</v>
+        <v>0.19656</v>
       </c>
       <c r="X15" s="8" t="n">
         <v>0.009010000000000001</v>
       </c>
       <c r="Y15" s="8" t="n">
-        <v>0.1255055040433496</v>
+        <v>0.1255411479114942</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>0.1360412160683838</v>
+        <v>0.1360720231242267</v>
       </c>
     </row>
     <row r="16">
@@ -1630,11 +1590,7 @@
           <t>LAA</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C16" s="2" t="n"/>
       <c r="D16" s="5" t="n">
         <v>660.8</v>
       </c>
@@ -1683,37 +1639,37 @@
         <v/>
       </c>
       <c r="P16" s="8" t="n">
-        <v>0.1116352822567691</v>
+        <v>0.11167</v>
       </c>
       <c r="Q16" s="8" t="n">
-        <v>0.0363689465039138</v>
+        <v>0.03638</v>
       </c>
       <c r="R16" s="8" t="n">
-        <v>0.0031538325073089</v>
+        <v>0.00316</v>
       </c>
       <c r="S16" s="8" t="n">
-        <v>0.0459665121245808</v>
+        <v>0.04597</v>
       </c>
       <c r="T16" s="8" t="n">
-        <v>0.1406991100760794</v>
+        <v>0.14068</v>
       </c>
       <c r="U16" s="8" t="n">
-        <v>0.013745484840232</v>
+        <v>0.01375</v>
       </c>
       <c r="V16" s="8" t="n">
-        <v>0.0050272863428303</v>
+        <v>0.00503</v>
       </c>
       <c r="W16" s="8" t="n">
-        <v>0.2826658845283855</v>
+        <v>0.28253</v>
       </c>
       <c r="X16" s="8" t="n">
         <v>0.0123</v>
       </c>
       <c r="Y16" s="8" t="n">
-        <v>0.1351658524920535</v>
+        <v>0.1351966789637865</v>
       </c>
       <c r="Z16" s="8" t="n">
-        <v>0.1085451535772362</v>
+        <v>0.108569014719431</v>
       </c>
     </row>
     <row r="17">
@@ -1727,11 +1683,7 @@
           <t>PIT</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C17" s="2" t="n"/>
       <c r="D17" s="5" t="n">
         <v>656.6</v>
       </c>
@@ -1780,37 +1732,37 @@
         <v/>
       </c>
       <c r="P17" s="8" t="n">
-        <v>0.1381793734734412</v>
+        <v>0.13822</v>
       </c>
       <c r="Q17" s="8" t="n">
-        <v>0.0494495608078465</v>
+        <v>0.04947</v>
       </c>
       <c r="R17" s="8" t="n">
-        <v>0.0057256629801136</v>
+        <v>0.00573</v>
       </c>
       <c r="S17" s="8" t="n">
-        <v>0.0348039176394667</v>
+        <v>0.03481</v>
       </c>
       <c r="T17" s="8" t="n">
-        <v>0.0948527821698493</v>
+        <v>0.09483</v>
       </c>
       <c r="U17" s="8" t="n">
-        <v>0.0143713534984104</v>
+        <v>0.01437</v>
       </c>
       <c r="V17" s="8" t="n">
-        <v>0.0050971838056443</v>
+        <v>0.0051</v>
       </c>
       <c r="W17" s="8" t="n">
-        <v>0.2391307332244535</v>
+        <v>0.239</v>
       </c>
       <c r="X17" s="8" t="n">
         <v>0.01286</v>
       </c>
       <c r="Y17" s="8" t="n">
-        <v>0.1229879629561983</v>
+        <v>0.1230230418459303</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>0.1157915089324837</v>
+        <v>0.115812686628736</v>
       </c>
     </row>
     <row r="18">
@@ -1824,11 +1776,7 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C18" s="2" t="n"/>
       <c r="D18" s="5" t="n">
         <v>654.2</v>
       </c>
@@ -1877,37 +1825,37 @@
         <v/>
       </c>
       <c r="P18" s="8" t="n">
-        <v>0.1589578537429866</v>
+        <v>0.15899</v>
       </c>
       <c r="Q18" s="8" t="n">
-        <v>0.0470761737419287</v>
+        <v>0.04709</v>
       </c>
       <c r="R18" s="8" t="n">
-        <v>0.00191089816217</v>
+        <v>0.00192</v>
       </c>
       <c r="S18" s="8" t="n">
-        <v>0.0397421412616588</v>
+        <v>0.03974</v>
       </c>
       <c r="T18" s="8" t="n">
-        <v>0.07149669423783769</v>
+        <v>0.07148</v>
       </c>
       <c r="U18" s="8" t="n">
-        <v>0.007179888182962</v>
+        <v>0.00718</v>
       </c>
       <c r="V18" s="8" t="n">
-        <v>0.0071094212871136</v>
+        <v>0.0071</v>
       </c>
       <c r="W18" s="8" t="n">
-        <v>0.1602153311593029</v>
+        <v>0.16011</v>
       </c>
       <c r="X18" s="8" t="n">
         <v>0.008869999999999999</v>
       </c>
       <c r="Y18" s="8" t="n">
-        <v>0.1081380809993775</v>
+        <v>0.1081688846180165</v>
       </c>
       <c r="Z18" s="8" t="n">
-        <v>0.1283754540191236</v>
+        <v>0.1284077807000251</v>
       </c>
     </row>
     <row r="19">
@@ -1921,11 +1869,7 @@
           <t>MIA</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C19" s="2" t="n"/>
       <c r="D19" s="5" t="n">
         <v>653.8</v>
       </c>
@@ -1974,37 +1918,37 @@
         <v/>
       </c>
       <c r="P19" s="8" t="n">
-        <v>0.1856534512275325</v>
+        <v>0.1857</v>
       </c>
       <c r="Q19" s="8" t="n">
-        <v>0.0312171053150348</v>
+        <v>0.03122</v>
       </c>
       <c r="R19" s="8" t="n">
-        <v>0.0053487056571803</v>
+        <v>0.00534</v>
       </c>
       <c r="S19" s="8" t="n">
-        <v>0.0073312159589503</v>
+        <v>0.00733</v>
       </c>
       <c r="T19" s="8" t="n">
-        <v>0.0944677755461298</v>
+        <v>0.09444</v>
       </c>
       <c r="U19" s="8" t="n">
-        <v>0.0028360761478797</v>
+        <v>0.00284</v>
       </c>
       <c r="V19" s="8" t="n">
-        <v>0.007928767815208499</v>
+        <v>0.00793</v>
       </c>
       <c r="W19" s="8" t="n">
-        <v>0.1558054447182011</v>
+        <v>0.15571</v>
       </c>
       <c r="X19" s="8" t="n">
         <v>0.04288</v>
       </c>
       <c r="Y19" s="8" t="n">
-        <v>0.1096948110092585</v>
+        <v>0.1097258217418803</v>
       </c>
       <c r="Z19" s="8" t="n">
-        <v>0.0788417097973404</v>
+        <v>0.0788589008153579</v>
       </c>
     </row>
     <row r="20">
@@ -2018,11 +1962,7 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C20" s="2" t="n"/>
       <c r="D20" s="5" t="n">
         <v>651.3</v>
       </c>
@@ -2071,37 +2011,37 @@
         <v/>
       </c>
       <c r="P20" s="8" t="n">
-        <v>0.1367928652167036</v>
+        <v>0.13683</v>
       </c>
       <c r="Q20" s="8" t="n">
-        <v>0.044431924551</v>
+        <v>0.04444</v>
       </c>
       <c r="R20" s="8" t="n">
-        <v>0.0035654136077995</v>
+        <v>0.00356</v>
       </c>
       <c r="S20" s="8" t="n">
-        <v>0.0316373514867605</v>
+        <v>0.03164</v>
       </c>
       <c r="T20" s="8" t="n">
-        <v>0.07300246651891359</v>
+        <v>0.07299</v>
       </c>
       <c r="U20" s="8" t="n">
-        <v>0.0086489359627908</v>
+        <v>0.00865</v>
       </c>
       <c r="V20" s="8" t="n">
-        <v>0.0052477388796809</v>
+        <v>0.00525</v>
       </c>
       <c r="W20" s="8" t="n">
-        <v>0.2702243556799588</v>
+        <v>0.27008</v>
       </c>
       <c r="X20" s="8" t="n">
         <v>0.02463</v>
       </c>
       <c r="Y20" s="8" t="n">
-        <v>0.1129051469234198</v>
+        <v>0.1129403520129875</v>
       </c>
       <c r="Z20" s="8" t="n">
-        <v>0.1172009439728419</v>
+        <v>0.1172243610493367</v>
       </c>
     </row>
     <row r="21">
@@ -2115,11 +2055,7 @@
           <t>MIA</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C21" s="2" t="n"/>
       <c r="D21" s="5" t="n">
         <v>650.6</v>
       </c>
@@ -2168,37 +2104,37 @@
         <v/>
       </c>
       <c r="P21" s="8" t="n">
-        <v>0.1446074645276915</v>
+        <v>0.14464</v>
       </c>
       <c r="Q21" s="8" t="n">
-        <v>0.0396650427703261</v>
+        <v>0.03968</v>
       </c>
       <c r="R21" s="8" t="n">
-        <v>0.0076517519681991</v>
+        <v>0.00765</v>
       </c>
       <c r="S21" s="8" t="n">
-        <v>0.0177134253905958</v>
+        <v>0.01771</v>
       </c>
       <c r="T21" s="8" t="n">
-        <v>0.1121680733301804</v>
+        <v>0.11214</v>
       </c>
       <c r="U21" s="8" t="n">
-        <v>0.018739431730198</v>
+        <v>0.01874</v>
       </c>
       <c r="V21" s="8" t="n">
-        <v>0.0027035213464776</v>
+        <v>0.0027</v>
       </c>
       <c r="W21" s="8" t="n">
-        <v>0.211315643671226</v>
+        <v>0.2112</v>
       </c>
       <c r="X21" s="8" t="n">
         <v>0.04402</v>
       </c>
       <c r="Y21" s="8" t="n">
-        <v>0.1191859526268617</v>
+        <v>0.1192101773713967</v>
       </c>
       <c r="Z21" s="8" t="n">
-        <v>0.0846392996915394</v>
+        <v>0.0846559518514351</v>
       </c>
     </row>
     <row r="22">
@@ -2212,11 +2148,7 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C22" s="2" t="n"/>
       <c r="D22" s="5" t="n">
         <v>648.3</v>
       </c>
@@ -2265,37 +2197,37 @@
         <v/>
       </c>
       <c r="P22" s="8" t="n">
-        <v>0.184523212697718</v>
+        <v>0.18455</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>0.0455621070933989</v>
+        <v>0.04557</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>0.0067092048847082</v>
+        <v>0.00671</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>0.0145802958491529</v>
+        <v>0.01458</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>0.0633355003357082</v>
+        <v>0.06331000000000001</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>0.0101313633828165</v>
+        <v>0.01013</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>0.0072439579285827</v>
+        <v>0.00724</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>0.1170992715380788</v>
+        <v>0.11702</v>
       </c>
       <c r="X22" s="8" t="n">
         <v>0.01942</v>
       </c>
       <c r="Y22" s="8" t="n">
-        <v>0.113440576857809</v>
+        <v>0.1134704210984195</v>
       </c>
       <c r="Z22" s="8" t="n">
-        <v>0.09331171598978889</v>
+        <v>0.0933307774753884</v>
       </c>
     </row>
     <row r="23">
@@ -2309,11 +2241,7 @@
           <t>TB</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C23" s="2" t="n"/>
       <c r="D23" s="5" t="n">
         <v>646.1</v>
       </c>
@@ -2362,37 +2290,37 @@
         <v/>
       </c>
       <c r="P23" s="8" t="n">
-        <v>0.1770523085610501</v>
+        <v>0.17709</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>0.0364861243081768</v>
+        <v>0.0365</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>0.0017338337596773</v>
+        <v>0.00173</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>0.0296319061923731</v>
+        <v>0.02963</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>0.09202901694213469</v>
+        <v>0.09200999999999999</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>0.0106454004675448</v>
+        <v>0.01064</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>0.0057169087169998</v>
+        <v>0.00571</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>0.1492558389626138</v>
+        <v>0.14916</v>
       </c>
       <c r="X23" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="Y23" s="8" t="n">
-        <v>0.1167412834207547</v>
+        <v>0.1167654185675505</v>
       </c>
       <c r="Z23" s="8" t="n">
-        <v>0.1117624602160041</v>
+        <v>0.1117892907197758</v>
       </c>
     </row>
     <row r="24">
@@ -2406,11 +2334,7 @@
           <t>ATL</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C24" s="2" t="n"/>
       <c r="D24" s="5" t="n">
         <v>643</v>
       </c>
@@ -2459,37 +2383,37 @@
         <v/>
       </c>
       <c r="P24" s="8" t="n">
-        <v>0.116516541649391</v>
+        <v>0.11655</v>
       </c>
       <c r="Q24" s="8" t="n">
-        <v>0.0493341174597428</v>
+        <v>0.04935</v>
       </c>
       <c r="R24" s="8" t="n">
-        <v>0.0015721461114881</v>
+        <v>0.00157</v>
       </c>
       <c r="S24" s="8" t="n">
-        <v>0.0471962896536999</v>
+        <v>0.0472</v>
       </c>
       <c r="T24" s="8" t="n">
-        <v>0.109544829680604</v>
+        <v>0.10952</v>
       </c>
       <c r="U24" s="8" t="n">
-        <v>0.0067129719336031</v>
+        <v>0.00672</v>
       </c>
       <c r="V24" s="8" t="n">
-        <v>0.0066874201996218</v>
+        <v>0.00669</v>
       </c>
       <c r="W24" s="8" t="n">
-        <v>0.2466180220104759</v>
+        <v>0.24649</v>
       </c>
       <c r="X24" s="8" t="n">
         <v>0.00144</v>
       </c>
       <c r="Y24" s="8" t="n">
-        <v>0.1267156579007921</v>
+        <v>0.1267409005075677</v>
       </c>
       <c r="Z24" s="8" t="n">
-        <v>0.133177919306525</v>
+        <v>0.1332102973321215</v>
       </c>
     </row>
     <row r="25">
@@ -2503,11 +2427,7 @@
           <t>OAK</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C25" s="2" t="n"/>
       <c r="D25" s="5" t="n">
         <v>637.2</v>
       </c>
@@ -2556,37 +2476,37 @@
         <v/>
       </c>
       <c r="P25" s="8" t="n">
-        <v>0.113565720453934</v>
+        <v>0.1136</v>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>0.0487120605391216</v>
+        <v>0.04873</v>
       </c>
       <c r="R25" s="8" t="n">
-        <v>0.0023116253436968</v>
+        <v>0.00231</v>
       </c>
       <c r="S25" s="8" t="n">
-        <v>0.0496006763588236</v>
+        <v>0.04961</v>
       </c>
       <c r="T25" s="8" t="n">
-        <v>0.09123226696019821</v>
+        <v>0.09121</v>
       </c>
       <c r="U25" s="8" t="n">
-        <v>0.01076017091825</v>
+        <v>0.01076</v>
       </c>
       <c r="V25" s="8" t="n">
-        <v>0.0057100550294672</v>
+        <v>0.00571</v>
       </c>
       <c r="W25" s="8" t="n">
-        <v>0.2769897966899819</v>
+        <v>0.27684</v>
       </c>
       <c r="X25" s="8" t="n">
         <v>0.01097</v>
       </c>
       <c r="Y25" s="8" t="n">
-        <v>0.1275977994252371</v>
+        <v>0.1276311387344904</v>
       </c>
       <c r="Z25" s="8" t="n">
-        <v>0.147060556926209</v>
+        <v>0.1470909543443185</v>
       </c>
     </row>
     <row r="26">
@@ -2600,11 +2520,7 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Catcher - Primary</t>
-        </is>
-      </c>
+      <c r="C26" s="2" t="n"/>
       <c r="D26" s="5" t="n">
         <v>634.7</v>
       </c>
@@ -2653,37 +2569,37 @@
         <v/>
       </c>
       <c r="P26" s="8" t="n">
-        <v>0.1449552098444916</v>
+        <v>0.145</v>
       </c>
       <c r="Q26" s="8" t="n">
-        <v>0.0389101478523344</v>
+        <v>0.03892</v>
       </c>
       <c r="R26" s="8" t="n">
-        <v>0.0015249234709046</v>
+        <v>0.00152</v>
       </c>
       <c r="S26" s="8" t="n">
-        <v>0.0313903231344219</v>
+        <v>0.03139</v>
       </c>
       <c r="T26" s="8" t="n">
-        <v>0.0982658872728548</v>
+        <v>0.09823999999999999</v>
       </c>
       <c r="U26" s="8" t="n">
-        <v>0.0314994515272335</v>
+        <v>0.03151</v>
       </c>
       <c r="V26" s="8" t="n">
-        <v>0.0078477640776586</v>
+        <v>0.00784</v>
       </c>
       <c r="W26" s="8" t="n">
-        <v>0.2013887160947818</v>
+        <v>0.20128</v>
       </c>
       <c r="X26" s="8" t="n">
         <v>0.01169</v>
       </c>
       <c r="Y26" s="8" t="n">
-        <v>0.1208260891622276</v>
+        <v>0.1208521761413874</v>
       </c>
       <c r="Z26" s="8" t="n">
-        <v>0.104068855524292</v>
+        <v>0.1040911079641611</v>
       </c>
     </row>
     <row r="27">
@@ -2697,11 +2613,7 @@
           <t>BOS</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C27" s="2" t="n"/>
       <c r="D27" s="5" t="n">
         <v>633.8</v>
       </c>
@@ -2750,37 +2662,37 @@
         <v/>
       </c>
       <c r="P27" s="8" t="n">
-        <v>0.141388647336861</v>
+        <v>0.14142</v>
       </c>
       <c r="Q27" s="8" t="n">
-        <v>0.0434117522599666</v>
+        <v>0.04343</v>
       </c>
       <c r="R27" s="8" t="n">
-        <v>0.0091508380092136</v>
+        <v>0.00915</v>
       </c>
       <c r="S27" s="8" t="n">
-        <v>0.0275354877951152</v>
+        <v>0.02754</v>
       </c>
       <c r="T27" s="8" t="n">
-        <v>0.0729754946019683</v>
+        <v>0.07296</v>
       </c>
       <c r="U27" s="8" t="n">
-        <v>0.0114736565904009</v>
+        <v>0.01147</v>
       </c>
       <c r="V27" s="8" t="n">
-        <v>0.0060064383256631</v>
+        <v>0.00601</v>
       </c>
       <c r="W27" s="8" t="n">
-        <v>0.2510137743215936</v>
+        <v>0.25088</v>
       </c>
       <c r="X27" s="8" t="n">
         <v>0.0397</v>
       </c>
       <c r="Y27" s="8" t="n">
-        <v>0.1154229986504771</v>
+        <v>0.1154503661598059</v>
       </c>
       <c r="Z27" s="8" t="n">
-        <v>0.1027052089255464</v>
+        <v>0.102729920964542</v>
       </c>
     </row>
     <row r="28">
@@ -2794,11 +2706,7 @@
           <t>TB</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C28" s="2" t="n"/>
       <c r="D28" s="5" t="n">
         <v>629.2</v>
       </c>
@@ -2847,37 +2755,37 @@
         <v/>
       </c>
       <c r="P28" s="8" t="n">
-        <v>0.1458441006749895</v>
+        <v>0.14589</v>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>0.0429465017636533</v>
+        <v>0.04296</v>
       </c>
       <c r="R28" s="8" t="n">
-        <v>0.0017797185625241</v>
+        <v>0.00178</v>
       </c>
       <c r="S28" s="8" t="n">
-        <v>0.0365806747191188</v>
+        <v>0.03658</v>
       </c>
       <c r="T28" s="8" t="n">
-        <v>0.097237688178367</v>
+        <v>0.09722</v>
       </c>
       <c r="U28" s="8" t="n">
-        <v>0.0161105036141282</v>
+        <v>0.01612</v>
       </c>
       <c r="V28" s="8" t="n">
-        <v>0.0088572944357926</v>
+        <v>0.00885</v>
       </c>
       <c r="W28" s="8" t="n">
-        <v>0.2513704723567836</v>
+        <v>0.25123</v>
       </c>
       <c r="X28" s="8" t="n">
         <v>0.00285</v>
       </c>
       <c r="Y28" s="8" t="n">
-        <v>0.1131796533379555</v>
+        <v>0.1131972648782547</v>
       </c>
       <c r="Z28" s="8" t="n">
-        <v>0.1202376480308325</v>
+        <v>0.1202660666465083</v>
       </c>
     </row>
     <row r="29">
@@ -2891,11 +2799,7 @@
           <t>PHI</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Everyday DH / 1B-DH</t>
-        </is>
-      </c>
+      <c r="C29" s="2" t="n"/>
       <c r="D29" s="5" t="n">
         <v>629.2</v>
       </c>
@@ -2944,37 +2848,37 @@
         <v/>
       </c>
       <c r="P29" s="8" t="n">
-        <v>0.0957151731331384</v>
+        <v>0.09575</v>
       </c>
       <c r="Q29" s="8" t="n">
-        <v>0.037363128917237</v>
+        <v>0.03737</v>
       </c>
       <c r="R29" s="8" t="n">
-        <v>0.001541821371104</v>
+        <v>0.00154</v>
       </c>
       <c r="S29" s="8" t="n">
-        <v>0.0615179622066462</v>
+        <v>0.06153</v>
       </c>
       <c r="T29" s="8" t="n">
-        <v>0.1457262276054725</v>
+        <v>0.1457</v>
       </c>
       <c r="U29" s="8" t="n">
-        <v>0.009462203024157101</v>
+        <v>0.009469999999999999</v>
       </c>
       <c r="V29" s="8" t="n">
-        <v>0.005624446679026</v>
+        <v>0.00563</v>
       </c>
       <c r="W29" s="8" t="n">
-        <v>0.2963773546807472</v>
+        <v>0.29624</v>
       </c>
       <c r="X29" s="8" t="n">
         <v>0.00756</v>
       </c>
       <c r="Y29" s="8" t="n">
-        <v>0.1376908262176333</v>
+        <v>0.1377218230785208</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>0.1405662017201258</v>
+        <v>0.1406036335100544</v>
       </c>
     </row>
     <row r="30">
@@ -2988,11 +2892,7 @@
           <t>DET</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
+      <c r="C30" s="2" t="n"/>
       <c r="D30" s="5" t="n">
         <v>628.3</v>
       </c>
@@ -3041,37 +2941,37 @@
         <v/>
       </c>
       <c r="P30" s="8" t="n">
-        <v>0.1389286686707562</v>
+        <v>0.13896</v>
       </c>
       <c r="Q30" s="8" t="n">
-        <v>0.043236305053078</v>
+        <v>0.04324</v>
       </c>
       <c r="R30" s="8" t="n">
-        <v>0.0078886519958447</v>
+        <v>0.007889999999999999</v>
       </c>
       <c r="S30" s="8" t="n">
-        <v>0.0295203589750204</v>
+        <v>0.02952</v>
       </c>
       <c r="T30" s="8" t="n">
-        <v>0.124964793164522</v>
+        <v>0.12493</v>
       </c>
       <c r="U30" s="8" t="n">
-        <v>0.0048268620624905</v>
+        <v>0.00483</v>
       </c>
       <c r="V30" s="8" t="n">
-        <v>0.0056988078384421</v>
+        <v>0.00569</v>
       </c>
       <c r="W30" s="8" t="n">
-        <v>0.1564518513684717</v>
+        <v>0.15636</v>
       </c>
       <c r="X30" s="8" t="n">
         <v>0.01801</v>
       </c>
       <c r="Y30" s="8" t="n">
-        <v>0.1299513257472775</v>
+        <v>0.1299821007704813</v>
       </c>
       <c r="Z30" s="8" t="n">
-        <v>0.1026775907138984</v>
+        <v>0.1027026562992671</v>
       </c>
     </row>
     <row r="33">
@@ -3199,13 +3099,9 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C35" s="2" t="n"/>
       <c r="D35" s="5" t="n">
-        <v>228.1</v>
+        <v>228.4</v>
       </c>
       <c r="E35" s="6">
         <f>D35*N35</f>
@@ -3244,28 +3140,28 @@
         <v/>
       </c>
       <c r="N35" s="8" t="n">
-        <v>4.175</v>
+        <v>4.174</v>
       </c>
       <c r="O35" s="8" t="n">
-        <v>0.217289061913408</v>
+        <v>0.21751</v>
       </c>
       <c r="P35" s="8" t="n">
-        <v>0.057333703898768</v>
+        <v>0.05737</v>
       </c>
       <c r="Q35" s="8" t="n">
-        <v>0.0209472978593729</v>
+        <v>0.02097</v>
       </c>
       <c r="R35" s="8" t="n">
-        <v>0.1710515608504867</v>
+        <v>0.17092</v>
       </c>
       <c r="S35" s="8" t="n">
-        <v>0.0398919234722861</v>
+        <v>0.03986</v>
       </c>
       <c r="T35" s="8" t="n">
-        <v>0.0049764380649717</v>
+        <v>0.00497</v>
       </c>
       <c r="U35" s="8" t="n">
-        <v>3.799332692437589</v>
+        <v>3.79741</v>
       </c>
     </row>
     <row r="36">
@@ -3279,13 +3175,9 @@
           <t>MIA</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C36" s="2" t="n"/>
       <c r="D36" s="5" t="n">
-        <v>215.3</v>
+        <v>215.5</v>
       </c>
       <c r="E36" s="6">
         <f>D36*N36</f>
@@ -3327,25 +3219,25 @@
         <v>4.221</v>
       </c>
       <c r="O36" s="8" t="n">
-        <v>0.1904615660845947</v>
+        <v>0.19066</v>
       </c>
       <c r="P36" s="8" t="n">
-        <v>0.0685340262116725</v>
+        <v>0.06858</v>
       </c>
       <c r="Q36" s="8" t="n">
-        <v>0.0266307651146757</v>
+        <v>0.02666</v>
       </c>
       <c r="R36" s="8" t="n">
-        <v>0.1545890039612385</v>
+        <v>0.15448</v>
       </c>
       <c r="S36" s="8" t="n">
-        <v>0.0457646053155556</v>
+        <v>0.04573</v>
       </c>
       <c r="T36" s="8" t="n">
-        <v>0.0044088556839223</v>
+        <v>0.00441</v>
       </c>
       <c r="U36" s="8" t="n">
-        <v>4.168280440190198</v>
+        <v>4.16652</v>
       </c>
     </row>
     <row r="37">
@@ -3359,13 +3251,9 @@
           <t>NYM</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C37" s="2" t="n"/>
       <c r="D37" s="5" t="n">
-        <v>210.2</v>
+        <v>210.5</v>
       </c>
       <c r="E37" s="6">
         <f>D37*N37</f>
@@ -3407,25 +3295,25 @@
         <v>4.207</v>
       </c>
       <c r="O37" s="8" t="n">
-        <v>0.2546106730852104</v>
+        <v>0.25484</v>
       </c>
       <c r="P37" s="8" t="n">
-        <v>0.0923539268000669</v>
+        <v>0.0924</v>
       </c>
       <c r="Q37" s="8" t="n">
-        <v>0.0214008941998862</v>
+        <v>0.02142</v>
       </c>
       <c r="R37" s="8" t="n">
-        <v>0.1353400383381686</v>
+        <v>0.13523</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>0.0372781865668496</v>
+        <v>0.03724</v>
       </c>
       <c r="T37" s="8" t="n">
-        <v>0.0031683528536412</v>
+        <v>0.00316</v>
       </c>
       <c r="U37" s="8" t="n">
-        <v>3.596627988339067</v>
+        <v>3.59469</v>
       </c>
     </row>
     <row r="38">
@@ -3439,13 +3327,9 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C38" s="2" t="n"/>
       <c r="D38" s="5" t="n">
-        <v>201.6</v>
+        <v>202.1</v>
       </c>
       <c r="E38" s="6">
         <f>D38*N38</f>
@@ -3484,28 +3368,28 @@
         <v/>
       </c>
       <c r="N38" s="8" t="n">
-        <v>4.333</v>
+        <v>4.332</v>
       </c>
       <c r="O38" s="8" t="n">
-        <v>0.162771645136007</v>
+        <v>0.16294</v>
       </c>
       <c r="P38" s="8" t="n">
-        <v>0.08612517793557629</v>
+        <v>0.08619</v>
       </c>
       <c r="Q38" s="8" t="n">
-        <v>0.0206473982116132</v>
+        <v>0.02067</v>
       </c>
       <c r="R38" s="8" t="n">
-        <v>0.1732928235066811</v>
+        <v>0.17318</v>
       </c>
       <c r="S38" s="8" t="n">
-        <v>0.0368415198333899</v>
+        <v>0.03682</v>
       </c>
       <c r="T38" s="8" t="n">
-        <v>0.0040803065510018</v>
+        <v>0.00408</v>
       </c>
       <c r="U38" s="8" t="n">
-        <v>4.202339066841319</v>
+        <v>4.20085</v>
       </c>
     </row>
     <row r="39">
@@ -3519,13 +3403,9 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C39" s="2" t="n"/>
       <c r="D39" s="5" t="n">
-        <v>200.7</v>
+        <v>201.2</v>
       </c>
       <c r="E39" s="6">
         <f>D39*N39</f>
@@ -3567,25 +3447,25 @@
         <v>4.272</v>
       </c>
       <c r="O39" s="8" t="n">
-        <v>0.1652917130353317</v>
+        <v>0.16546</v>
       </c>
       <c r="P39" s="8" t="n">
-        <v>0.0643487441381419</v>
+        <v>0.06439</v>
       </c>
       <c r="Q39" s="8" t="n">
-        <v>0.0333144969415972</v>
+        <v>0.03336</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>0.1640645687192134</v>
+        <v>0.16395</v>
       </c>
       <c r="S39" s="8" t="n">
-        <v>0.0472452417234243</v>
+        <v>0.04721</v>
       </c>
       <c r="T39" s="8" t="n">
-        <v>0.0043951011224597</v>
+        <v>0.0044</v>
       </c>
       <c r="U39" s="8" t="n">
-        <v>4.661062167261105</v>
+        <v>4.66031</v>
       </c>
     </row>
     <row r="40">
@@ -3599,13 +3479,9 @@
           <t>STL</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>End-of-Rotation Starter (SP4-5)</t>
-        </is>
-      </c>
+      <c r="C40" s="2" t="n"/>
       <c r="D40" s="5" t="n">
-        <v>190.6</v>
+        <v>191.1</v>
       </c>
       <c r="E40" s="6">
         <f>D40*N40</f>
@@ -3644,28 +3520,28 @@
         <v/>
       </c>
       <c r="N40" s="8" t="n">
-        <v>4.321</v>
+        <v>4.32</v>
       </c>
       <c r="O40" s="8" t="n">
-        <v>0.2016177148916599</v>
+        <v>0.20181</v>
       </c>
       <c r="P40" s="8" t="n">
-        <v>0.0789613709536665</v>
+        <v>0.07901</v>
       </c>
       <c r="Q40" s="8" t="n">
-        <v>0.0367399715652176</v>
+        <v>0.03679</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>0.1501044724697726</v>
+        <v>0.14999</v>
       </c>
       <c r="S40" s="8" t="n">
-        <v>0.048180006426364</v>
+        <v>0.04814</v>
       </c>
       <c r="T40" s="8" t="n">
-        <v>0.0034777027682855</v>
+        <v>0.00347</v>
       </c>
       <c r="U40" s="8" t="n">
-        <v>4.812373146577092</v>
+        <v>4.81132</v>
       </c>
     </row>
     <row r="41">
@@ -3679,13 +3555,9 @@
           <t>PHI</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C41" s="2" t="n"/>
       <c r="D41" s="5" t="n">
-        <v>188.8</v>
+        <v>188.9</v>
       </c>
       <c r="E41" s="6">
         <f>D41*N41</f>
@@ -3727,25 +3599,25 @@
         <v>4.106</v>
       </c>
       <c r="O41" s="8" t="n">
-        <v>0.240108862340473</v>
+        <v>0.24035</v>
       </c>
       <c r="P41" s="8" t="n">
-        <v>0.0577723267451491</v>
+        <v>0.0578</v>
       </c>
       <c r="Q41" s="8" t="n">
-        <v>0.0202752531796793</v>
+        <v>0.02029</v>
       </c>
       <c r="R41" s="8" t="n">
-        <v>0.1637041957187458</v>
+        <v>0.16358</v>
       </c>
       <c r="S41" s="8" t="n">
-        <v>0.039655535538133</v>
+        <v>0.03962</v>
       </c>
       <c r="T41" s="8" t="n">
-        <v>0.0025827209218988</v>
+        <v>0.00258</v>
       </c>
       <c r="U41" s="8" t="n">
-        <v>3.462211972119063</v>
+        <v>3.46002</v>
       </c>
     </row>
     <row r="42">
@@ -3759,13 +3631,9 @@
           <t>KC</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C42" s="2" t="n"/>
       <c r="D42" s="5" t="n">
-        <v>188.2</v>
+        <v>188.5</v>
       </c>
       <c r="E42" s="6">
         <f>D42*N42</f>
@@ -3807,25 +3675,25 @@
         <v>4.167</v>
       </c>
       <c r="O42" s="8" t="n">
-        <v>0.1951503884357816</v>
+        <v>0.19534</v>
       </c>
       <c r="P42" s="8" t="n">
-        <v>0.0684856723514187</v>
+        <v>0.06852999999999999</v>
       </c>
       <c r="Q42" s="8" t="n">
-        <v>0.0313844082877594</v>
+        <v>0.03142</v>
       </c>
       <c r="R42" s="8" t="n">
-        <v>0.1391900527757334</v>
+        <v>0.13908</v>
       </c>
       <c r="S42" s="8" t="n">
-        <v>0.048565761566046</v>
+        <v>0.04853</v>
       </c>
       <c r="T42" s="8" t="n">
-        <v>0.0060348483030509</v>
+        <v>0.00603</v>
       </c>
       <c r="U42" s="8" t="n">
-        <v>4.199876484566082</v>
+        <v>4.19852</v>
       </c>
     </row>
     <row r="43">
@@ -3839,13 +3707,9 @@
           <t>PIT</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C43" s="2" t="n"/>
       <c r="D43" s="5" t="n">
-        <v>186.2</v>
+        <v>186.4</v>
       </c>
       <c r="E43" s="6">
         <f>D43*N43</f>
@@ -3884,28 +3748,28 @@
         <v/>
       </c>
       <c r="N43" s="8" t="n">
-        <v>4.006</v>
+        <v>4.005</v>
       </c>
       <c r="O43" s="8" t="n">
-        <v>0.2838273120459706</v>
+        <v>0.28408</v>
       </c>
       <c r="P43" s="8" t="n">
-        <v>0.0662995187317785</v>
+        <v>0.06633</v>
       </c>
       <c r="Q43" s="8" t="n">
-        <v>0.0231979383740248</v>
+        <v>0.02322</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>0.1296823652292026</v>
+        <v>0.12957</v>
       </c>
       <c r="S43" s="8" t="n">
-        <v>0.0377694745522151</v>
+        <v>0.03773</v>
       </c>
       <c r="T43" s="8" t="n">
-        <v>0.0038676011345962</v>
+        <v>0.00386</v>
       </c>
       <c r="U43" s="8" t="n">
-        <v>3.098319547694544</v>
+        <v>3.09649</v>
       </c>
     </row>
     <row r="44">
@@ -3919,13 +3783,9 @@
           <t>NYM</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>End-of-Rotation Starter (SP4-5)</t>
-        </is>
-      </c>
+      <c r="C44" s="2" t="n"/>
       <c r="D44" s="5" t="n">
-        <v>182.4</v>
+        <v>182.6</v>
       </c>
       <c r="E44" s="6">
         <f>D44*N44</f>
@@ -3967,25 +3827,25 @@
         <v>4.237</v>
       </c>
       <c r="O44" s="8" t="n">
-        <v>0.2353623070196711</v>
+        <v>0.23557</v>
       </c>
       <c r="P44" s="8" t="n">
-        <v>0.07540060727075459</v>
+        <v>0.07543999999999999</v>
       </c>
       <c r="Q44" s="8" t="n">
-        <v>0.0387872988088788</v>
+        <v>0.03883</v>
       </c>
       <c r="R44" s="8" t="n">
-        <v>0.1314473308911717</v>
+        <v>0.13134</v>
       </c>
       <c r="S44" s="8" t="n">
-        <v>0.0477332000176569</v>
+        <v>0.04769</v>
       </c>
       <c r="T44" s="8" t="n">
-        <v>0.0036980382093854</v>
+        <v>0.0037</v>
       </c>
       <c r="U44" s="8" t="n">
-        <v>4.529640176548881</v>
+        <v>4.52874</v>
       </c>
     </row>
     <row r="45">
@@ -3999,13 +3859,9 @@
           <t>DET</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C45" s="2" t="n"/>
       <c r="D45" s="5" t="n">
-        <v>178.8</v>
+        <v>179.2</v>
       </c>
       <c r="E45" s="6">
         <f>D45*N45</f>
@@ -4047,25 +3903,25 @@
         <v>4.248</v>
       </c>
       <c r="O45" s="8" t="n">
-        <v>0.2174815412005056</v>
+        <v>0.21769</v>
       </c>
       <c r="P45" s="8" t="n">
-        <v>0.0829868174357693</v>
+        <v>0.08304</v>
       </c>
       <c r="Q45" s="8" t="n">
-        <v>0.0196336802160144</v>
+        <v>0.01966</v>
       </c>
       <c r="R45" s="8" t="n">
-        <v>0.1544292644939418</v>
+        <v>0.15432</v>
       </c>
       <c r="S45" s="8" t="n">
-        <v>0.040993828010479</v>
+        <v>0.04096</v>
       </c>
       <c r="T45" s="8" t="n">
-        <v>0.0036638617785271</v>
+        <v>0.00366</v>
       </c>
       <c r="U45" s="8" t="n">
-        <v>3.84532956904201</v>
+        <v>3.84354</v>
       </c>
     </row>
     <row r="46">
@@ -4079,13 +3935,9 @@
           <t>HOU</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C46" s="2" t="n"/>
       <c r="D46" s="5" t="n">
-        <v>178.6</v>
+        <v>178.9</v>
       </c>
       <c r="E46" s="6">
         <f>D46*N46</f>
@@ -4124,28 +3976,28 @@
         <v/>
       </c>
       <c r="N46" s="8" t="n">
-        <v>4.13</v>
+        <v>4.129</v>
       </c>
       <c r="O46" s="8" t="n">
-        <v>0.2603286156251944</v>
+        <v>0.26056</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>0.0915414247161338</v>
+        <v>0.09159</v>
       </c>
       <c r="Q46" s="8" t="n">
-        <v>0.0204222448174352</v>
+        <v>0.02044</v>
       </c>
       <c r="R46" s="8" t="n">
-        <v>0.1414513043118465</v>
+        <v>0.14134</v>
       </c>
       <c r="S46" s="8" t="n">
-        <v>0.0281703075005635</v>
+        <v>0.02815</v>
       </c>
       <c r="T46" s="8" t="n">
-        <v>0.0032779899817067</v>
+        <v>0.00328</v>
       </c>
       <c r="U46" s="8" t="n">
-        <v>3.227539049014212</v>
+        <v>3.22594</v>
       </c>
     </row>
     <row r="47">
@@ -4159,13 +4011,9 @@
           <t>BOS</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C47" s="2" t="n"/>
       <c r="D47" s="5" t="n">
-        <v>178.5</v>
+        <v>178.8</v>
       </c>
       <c r="E47" s="6">
         <f>D47*N47</f>
@@ -4207,25 +4055,25 @@
         <v>4.047</v>
       </c>
       <c r="O47" s="8" t="n">
-        <v>0.2997817329691249</v>
+        <v>0.30004</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>0.06675728734210309</v>
+        <v>0.06679</v>
       </c>
       <c r="Q47" s="8" t="n">
-        <v>0.0292853377915868</v>
+        <v>0.02932</v>
       </c>
       <c r="R47" s="8" t="n">
-        <v>0.1334982215624146</v>
+        <v>0.13338</v>
       </c>
       <c r="S47" s="8" t="n">
-        <v>0.0395666019623667</v>
+        <v>0.03953</v>
       </c>
       <c r="T47" s="8" t="n">
-        <v>0.0027172370156539</v>
+        <v>0.00272</v>
       </c>
       <c r="U47" s="8" t="n">
-        <v>3.426997755700019</v>
+        <v>3.42538</v>
       </c>
     </row>
     <row r="48">
@@ -4239,13 +4087,9 @@
           <t>PIT</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C48" s="2" t="n"/>
       <c r="D48" s="5" t="n">
-        <v>175.5</v>
+        <v>175.8</v>
       </c>
       <c r="E48" s="6">
         <f>D48*N48</f>
@@ -4287,25 +4131,25 @@
         <v>4.342</v>
       </c>
       <c r="O48" s="8" t="n">
-        <v>0.2055584237440721</v>
+        <v>0.20576</v>
       </c>
       <c r="P48" s="8" t="n">
-        <v>0.07462868137173539</v>
+        <v>0.07467</v>
       </c>
       <c r="Q48" s="8" t="n">
-        <v>0.0295373540679736</v>
+        <v>0.02957</v>
       </c>
       <c r="R48" s="8" t="n">
-        <v>0.1552635791383741</v>
+        <v>0.15515</v>
       </c>
       <c r="S48" s="8" t="n">
-        <v>0.0490491810048639</v>
+        <v>0.04901</v>
       </c>
       <c r="T48" s="8" t="n">
-        <v>0.0043012731979627</v>
+        <v>0.0043</v>
       </c>
       <c r="U48" s="8" t="n">
-        <v>4.662668866194193</v>
+        <v>4.66145</v>
       </c>
     </row>
     <row r="49">
@@ -4319,13 +4163,9 @@
           <t>SEA</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C49" s="2" t="n"/>
       <c r="D49" s="5" t="n">
-        <v>174.9</v>
+        <v>175</v>
       </c>
       <c r="E49" s="6">
         <f>D49*N49</f>
@@ -4367,25 +4207,25 @@
         <v>4.031</v>
       </c>
       <c r="O49" s="8" t="n">
-        <v>0.2614197632904981</v>
+        <v>0.26166</v>
       </c>
       <c r="P49" s="8" t="n">
-        <v>0.0590888014715683</v>
+        <v>0.05912</v>
       </c>
       <c r="Q49" s="8" t="n">
-        <v>0.036720408240436</v>
+        <v>0.03676</v>
       </c>
       <c r="R49" s="8" t="n">
-        <v>0.130738445631195</v>
+        <v>0.13063</v>
       </c>
       <c r="S49" s="8" t="n">
-        <v>0.0406792853810194</v>
+        <v>0.04064</v>
       </c>
       <c r="T49" s="8" t="n">
-        <v>0.002768836621607</v>
+        <v>0.00277</v>
       </c>
       <c r="U49" s="8" t="n">
-        <v>3.699902953452275</v>
+        <v>3.69867</v>
       </c>
     </row>
     <row r="50">
@@ -4399,13 +4239,9 @@
           <t>WSH</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C50" s="2" t="n"/>
       <c r="D50" s="5" t="n">
-        <v>173.6</v>
+        <v>174</v>
       </c>
       <c r="E50" s="6">
         <f>D50*N50</f>
@@ -4444,28 +4280,28 @@
         <v/>
       </c>
       <c r="N50" s="8" t="n">
-        <v>4.337</v>
+        <v>4.336</v>
       </c>
       <c r="O50" s="8" t="n">
-        <v>0.1903497157697418</v>
+        <v>0.19054</v>
       </c>
       <c r="P50" s="8" t="n">
-        <v>0.08604448048721371</v>
+        <v>0.0861</v>
       </c>
       <c r="Q50" s="8" t="n">
-        <v>0.0431145444261728</v>
+        <v>0.04316</v>
       </c>
       <c r="R50" s="8" t="n">
-        <v>0.1397022811671079</v>
+        <v>0.13959</v>
       </c>
       <c r="S50" s="8" t="n">
-        <v>0.0440386163580401</v>
+        <v>0.044</v>
       </c>
       <c r="T50" s="8" t="n">
-        <v>0.00459172310281</v>
+        <v>0.00459</v>
       </c>
       <c r="U50" s="8" t="n">
-        <v>5.027923504208188</v>
+        <v>5.0275</v>
       </c>
     </row>
     <row r="51">
@@ -4479,13 +4315,9 @@
           <t>KC</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C51" s="2" t="n"/>
       <c r="D51" s="5" t="n">
-        <v>172.1</v>
+        <v>172.4</v>
       </c>
       <c r="E51" s="6">
         <f>D51*N51</f>
@@ -4527,25 +4359,25 @@
         <v>4.186</v>
       </c>
       <c r="O51" s="8" t="n">
-        <v>0.2062011727160977</v>
+        <v>0.2064</v>
       </c>
       <c r="P51" s="8" t="n">
-        <v>0.0796038166867063</v>
+        <v>0.07965999999999999</v>
       </c>
       <c r="Q51" s="8" t="n">
-        <v>0.0303604175035703</v>
+        <v>0.0304</v>
       </c>
       <c r="R51" s="8" t="n">
-        <v>0.1420961721365587</v>
+        <v>0.14199</v>
       </c>
       <c r="S51" s="8" t="n">
-        <v>0.0420174918122967</v>
+        <v>0.04199</v>
       </c>
       <c r="T51" s="8" t="n">
-        <v>0.0035333451595329</v>
+        <v>0.00353</v>
       </c>
       <c r="U51" s="8" t="n">
-        <v>4.042495865461776</v>
+        <v>4.04163</v>
       </c>
     </row>
     <row r="52">
@@ -4559,13 +4391,9 @@
           <t>OAK</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C52" s="2" t="n"/>
       <c r="D52" s="5" t="n">
-        <v>171.1</v>
+        <v>171.3</v>
       </c>
       <c r="E52" s="6">
         <f>D52*N52</f>
@@ -4607,25 +4435,25 @@
         <v>4.231</v>
       </c>
       <c r="O52" s="8" t="n">
-        <v>0.2051146152584158</v>
+        <v>0.20531</v>
       </c>
       <c r="P52" s="8" t="n">
-        <v>0.0798387870110642</v>
+        <v>0.07988000000000001</v>
       </c>
       <c r="Q52" s="8" t="n">
-        <v>0.0396133707115901</v>
+        <v>0.03966</v>
       </c>
       <c r="R52" s="8" t="n">
-        <v>0.1380505092143502</v>
+        <v>0.13794</v>
       </c>
       <c r="S52" s="8" t="n">
-        <v>0.0457744317588518</v>
+        <v>0.04574</v>
       </c>
       <c r="T52" s="8" t="n">
-        <v>0.0030886254419302</v>
+        <v>0.00309</v>
       </c>
       <c r="U52" s="8" t="n">
-        <v>4.547148491127893</v>
+        <v>4.54668</v>
       </c>
     </row>
     <row r="53">
@@ -4639,13 +4467,9 @@
           <t>SEA</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C53" s="2" t="n"/>
       <c r="D53" s="5" t="n">
-        <v>170.1</v>
+        <v>170.3</v>
       </c>
       <c r="E53" s="6">
         <f>D53*N53</f>
@@ -4684,28 +4508,28 @@
         <v/>
       </c>
       <c r="N53" s="8" t="n">
-        <v>4.039</v>
+        <v>4.038</v>
       </c>
       <c r="O53" s="8" t="n">
-        <v>0.2415105511990694</v>
+        <v>0.24175</v>
       </c>
       <c r="P53" s="8" t="n">
-        <v>0.0552530894296101</v>
+        <v>0.05528</v>
       </c>
       <c r="Q53" s="8" t="n">
-        <v>0.0280211163837174</v>
+        <v>0.02805</v>
       </c>
       <c r="R53" s="8" t="n">
-        <v>0.1414674781646513</v>
+        <v>0.14136</v>
       </c>
       <c r="S53" s="8" t="n">
-        <v>0.0410716709806772</v>
+        <v>0.04103</v>
       </c>
       <c r="T53" s="8" t="n">
-        <v>0.0029952624878422</v>
+        <v>0.00299</v>
       </c>
       <c r="U53" s="8" t="n">
-        <v>3.491041566912448</v>
+        <v>3.48925</v>
       </c>
     </row>
     <row r="54">
@@ -4719,13 +4543,9 @@
           <t>SF</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>End-of-Rotation Starter (SP4-5)</t>
-        </is>
-      </c>
+      <c r="C54" s="2" t="n"/>
       <c r="D54" s="5" t="n">
-        <v>169.8</v>
+        <v>170.1</v>
       </c>
       <c r="E54" s="6">
         <f>D54*N54</f>
@@ -4767,25 +4587,25 @@
         <v>4.305</v>
       </c>
       <c r="O54" s="8" t="n">
-        <v>0.2123268489093385</v>
+        <v>0.21253</v>
       </c>
       <c r="P54" s="8" t="n">
-        <v>0.1069040630798433</v>
+        <v>0.10696</v>
       </c>
       <c r="Q54" s="8" t="n">
-        <v>0.0193135789081239</v>
+        <v>0.01933</v>
       </c>
       <c r="R54" s="8" t="n">
-        <v>0.1424285109237447</v>
+        <v>0.14232</v>
       </c>
       <c r="S54" s="8" t="n">
-        <v>0.0433320120983815</v>
+        <v>0.0433</v>
       </c>
       <c r="T54" s="8" t="n">
-        <v>0.0043022100889273</v>
+        <v>0.0043</v>
       </c>
       <c r="U54" s="8" t="n">
-        <v>3.972578704848437</v>
+        <v>3.9709</v>
       </c>
     </row>
     <row r="55">
@@ -4799,13 +4619,9 @@
           <t>KC</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C55" s="2" t="n"/>
       <c r="D55" s="5" t="n">
-        <v>169.4</v>
+        <v>169.7</v>
       </c>
       <c r="E55" s="6">
         <f>D55*N55</f>
@@ -4847,25 +4663,25 @@
         <v>4.282</v>
       </c>
       <c r="O55" s="8" t="n">
-        <v>0.2027770373527283</v>
+        <v>0.20298</v>
       </c>
       <c r="P55" s="8" t="n">
-        <v>0.07197795669003069</v>
+        <v>0.07202</v>
       </c>
       <c r="Q55" s="8" t="n">
-        <v>0.0363355709475309</v>
+        <v>0.03637</v>
       </c>
       <c r="R55" s="8" t="n">
-        <v>0.1484098539876353</v>
+        <v>0.1483</v>
       </c>
       <c r="S55" s="8" t="n">
-        <v>0.0476979976452114</v>
+        <v>0.04766</v>
       </c>
       <c r="T55" s="8" t="n">
-        <v>0.0053196896634839</v>
+        <v>0.00532</v>
       </c>
       <c r="U55" s="8" t="n">
-        <v>4.723054561065704</v>
+        <v>4.72189</v>
       </c>
     </row>
     <row r="56">
@@ -4879,13 +4695,9 @@
           <t>SEA</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+      <c r="C56" s="2" t="n"/>
       <c r="D56" s="5" t="n">
-        <v>168.8</v>
+        <v>168.9</v>
       </c>
       <c r="E56" s="6">
         <f>D56*N56</f>
@@ -4924,28 +4736,28 @@
         <v/>
       </c>
       <c r="N56" s="8" t="n">
-        <v>4.127</v>
+        <v>4.126</v>
       </c>
       <c r="O56" s="8" t="n">
-        <v>0.2224027501928272</v>
+        <v>0.22262</v>
       </c>
       <c r="P56" s="8" t="n">
-        <v>0.0479888201653147</v>
+        <v>0.04802</v>
       </c>
       <c r="Q56" s="8" t="n">
-        <v>0.0263772724223659</v>
+        <v>0.02641</v>
       </c>
       <c r="R56" s="8" t="n">
-        <v>0.163695361666137</v>
+        <v>0.16357</v>
       </c>
       <c r="S56" s="8" t="n">
-        <v>0.043678198657425</v>
+        <v>0.04364</v>
       </c>
       <c r="T56" s="8" t="n">
-        <v>0.0037307273869026</v>
+        <v>0.00373</v>
       </c>
       <c r="U56" s="8" t="n">
-        <v>3.861324157252909</v>
+        <v>3.85976</v>
       </c>
     </row>
     <row r="57">
@@ -4959,13 +4771,9 @@
           <t>NYY</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C57" s="2" t="n"/>
       <c r="D57" s="5" t="n">
-        <v>167.6</v>
+        <v>167.8</v>
       </c>
       <c r="E57" s="6">
         <f>D57*N57</f>
@@ -5004,28 +4812,28 @@
         <v/>
       </c>
       <c r="N57" s="8" t="n">
-        <v>4.065</v>
+        <v>4.064</v>
       </c>
       <c r="O57" s="8" t="n">
-        <v>0.2307281028068484</v>
+        <v>0.23096</v>
       </c>
       <c r="P57" s="8" t="n">
-        <v>0.06836361846576421</v>
+        <v>0.0684</v>
       </c>
       <c r="Q57" s="8" t="n">
-        <v>0.0172931197591694</v>
+        <v>0.01731</v>
       </c>
       <c r="R57" s="8" t="n">
-        <v>0.1507389352523212</v>
+        <v>0.15062</v>
       </c>
       <c r="S57" s="8" t="n">
-        <v>0.0359909126516607</v>
+        <v>0.03596</v>
       </c>
       <c r="T57" s="8" t="n">
-        <v>0.0023542396228754</v>
+        <v>0.00235</v>
       </c>
       <c r="U57" s="8" t="n">
-        <v>3.123866457829999</v>
+        <v>3.12183</v>
       </c>
     </row>
     <row r="58">
@@ -5039,13 +4847,9 @@
           <t>PHI</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Ace (SP1)</t>
-        </is>
-      </c>
+      <c r="C58" s="2" t="n"/>
       <c r="D58" s="5" t="n">
-        <v>167.2</v>
+        <v>167.3</v>
       </c>
       <c r="E58" s="6">
         <f>D58*N58</f>
@@ -5087,45 +4891,41 @@
         <v>4.103</v>
       </c>
       <c r="O58" s="8" t="n">
-        <v>0.2743051862349057</v>
+        <v>0.27456</v>
       </c>
       <c r="P58" s="8" t="n">
-        <v>0.0772785564263804</v>
+        <v>0.07732</v>
       </c>
       <c r="Q58" s="8" t="n">
-        <v>0.0234131573332943</v>
+        <v>0.02344</v>
       </c>
       <c r="R58" s="8" t="n">
-        <v>0.1429775844255564</v>
+        <v>0.14286</v>
       </c>
       <c r="S58" s="8" t="n">
-        <v>0.0352897377769046</v>
+        <v>0.03526</v>
       </c>
       <c r="T58" s="8" t="n">
-        <v>0.0025846917636468</v>
+        <v>0.00258</v>
       </c>
       <c r="U58" s="8" t="n">
-        <v>3.360425317142117</v>
+        <v>3.35839</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Braxton Ashcraft</t>
+          <t>Freddy Peralta</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>PIT</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
-        </is>
-      </c>
+          <t>TB</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n"/>
       <c r="D59" s="5" t="n">
-        <v>166.2</v>
+        <v>166.5</v>
       </c>
       <c r="E59" s="6">
         <f>D59*N59</f>
@@ -5164,28 +4964,28 @@
         <v/>
       </c>
       <c r="N59" s="8" t="n">
-        <v>4.083</v>
+        <v>4.173</v>
       </c>
       <c r="O59" s="8" t="n">
-        <v>0.2445322918197399</v>
+        <v>0.25592</v>
       </c>
       <c r="P59" s="8" t="n">
-        <v>0.0653794887116486</v>
+        <v>0.08917</v>
       </c>
       <c r="Q59" s="8" t="n">
-        <v>0.0229376580344182</v>
+        <v>0.02861</v>
       </c>
       <c r="R59" s="8" t="n">
-        <v>0.1509270229731849</v>
+        <v>0.13056</v>
       </c>
       <c r="S59" s="8" t="n">
-        <v>0.034666568132282</v>
+        <v>0.03836</v>
       </c>
       <c r="T59" s="8" t="n">
-        <v>0.0029624927715945</v>
+        <v>0.00359</v>
       </c>
       <c r="U59" s="8" t="n">
-        <v>3.363615621166775</v>
+        <v>3.77381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild 2027 projections (run 36904153833)
Verification PASSED.

Regenerated by .github/workflows/refresh-projections.yml.
Verification and the full baseline audit are in the run summary:
https://github.com/pmammino/DFSSimsFull/actions/runs/36904153833
</commit_message>
<xml_diff>
--- a/out/mlb_2027_what_if.xlsx
+++ b/out/mlb_2027_what_if.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="What-If" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What-If" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -713,10 +713,10 @@
         <v/>
       </c>
       <c r="P6" s="8" t="n">
-        <v>0.11543</v>
+        <v>0.11547</v>
       </c>
       <c r="Q6" s="8" t="n">
-        <v>0.04624</v>
+        <v>0.04625</v>
       </c>
       <c r="R6" s="8" t="n">
         <v>0.00263</v>
@@ -725,25 +725,25 @@
         <v>0.05016</v>
       </c>
       <c r="T6" s="8" t="n">
-        <v>0.11114</v>
+        <v>0.11112</v>
       </c>
       <c r="U6" s="8" t="n">
         <v>0.008489999999999999</v>
       </c>
       <c r="V6" s="8" t="n">
-        <v>0.0061</v>
+        <v>0.00609</v>
       </c>
       <c r="W6" s="8" t="n">
-        <v>0.2395</v>
+        <v>0.23936</v>
       </c>
       <c r="X6" s="8" t="n">
         <v>0.00351</v>
       </c>
       <c r="Y6" s="8" t="n">
-        <v>0.1311061514120952</v>
+        <v>0.1311443884698552</v>
       </c>
       <c r="Z6" s="8" t="n">
-        <v>0.139598019039103</v>
+        <v>0.1396361774803498</v>
       </c>
     </row>
     <row r="7">
@@ -810,10 +810,10 @@
         <v/>
       </c>
       <c r="P7" s="8" t="n">
-        <v>0.11267</v>
+        <v>0.11271</v>
       </c>
       <c r="Q7" s="8" t="n">
-        <v>0.05133</v>
+        <v>0.05135</v>
       </c>
       <c r="R7" s="8" t="n">
         <v>0.0034</v>
@@ -822,25 +822,25 @@
         <v>0.04693</v>
       </c>
       <c r="T7" s="8" t="n">
-        <v>0.07531</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="U7" s="8" t="n">
-        <v>0.02609</v>
+        <v>0.0261</v>
       </c>
       <c r="V7" s="8" t="n">
         <v>0.0037</v>
       </c>
       <c r="W7" s="8" t="n">
-        <v>0.27269</v>
+        <v>0.27253</v>
       </c>
       <c r="X7" s="8" t="n">
         <v>0.03728</v>
       </c>
       <c r="Y7" s="8" t="n">
-        <v>0.1306641264207448</v>
+        <v>0.1307057166175846</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>0.1112787569560603</v>
+        <v>0.1113103729849251</v>
       </c>
     </row>
     <row r="8">
@@ -907,19 +907,19 @@
         <v/>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0.11983</v>
+        <v>0.11988</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>0.04589</v>
+        <v>0.04591</v>
       </c>
       <c r="R8" s="8" t="n">
         <v>0.00315</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>0.04511</v>
+        <v>0.04512</v>
       </c>
       <c r="T8" s="8" t="n">
-        <v>0.13247</v>
+        <v>0.13246</v>
       </c>
       <c r="U8" s="8" t="n">
         <v>0.00557</v>
@@ -928,16 +928,16 @@
         <v>0.00429</v>
       </c>
       <c r="W8" s="8" t="n">
-        <v>0.30078</v>
+        <v>0.30062</v>
       </c>
       <c r="X8" s="8" t="n">
         <v>0.02916</v>
       </c>
       <c r="Y8" s="8" t="n">
-        <v>0.1315287659536379</v>
+        <v>0.1315714761985192</v>
       </c>
       <c r="Z8" s="8" t="n">
-        <v>0.1190261816289879</v>
+        <v>0.1190587159930348</v>
       </c>
     </row>
     <row r="9">
@@ -1004,10 +1004,10 @@
         <v/>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0.17322</v>
+        <v>0.17326</v>
       </c>
       <c r="Q9" s="8" t="n">
-        <v>0.04149</v>
+        <v>0.0415</v>
       </c>
       <c r="R9" s="8" t="n">
         <v>0.00515</v>
@@ -1016,25 +1016,25 @@
         <v>0.02082</v>
       </c>
       <c r="T9" s="8" t="n">
-        <v>0.06383</v>
+        <v>0.06381000000000001</v>
       </c>
       <c r="U9" s="8" t="n">
         <v>0.0075</v>
       </c>
       <c r="V9" s="8" t="n">
-        <v>0.00903</v>
+        <v>0.00902</v>
       </c>
       <c r="W9" s="8" t="n">
-        <v>0.15031</v>
+        <v>0.1502</v>
       </c>
       <c r="X9" s="8" t="n">
         <v>0.03639</v>
       </c>
       <c r="Y9" s="8" t="n">
-        <v>0.115997811533935</v>
+        <v>0.1160265509827313</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>0.1038145250857534</v>
+        <v>0.1038432404446151</v>
       </c>
     </row>
     <row r="10">
@@ -1101,10 +1101,10 @@
         <v/>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0.1134</v>
+        <v>0.11344</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>0.04217</v>
+        <v>0.04218</v>
       </c>
       <c r="R10" s="8" t="n">
         <v>0.00305</v>
@@ -1113,25 +1113,25 @@
         <v>0.04047</v>
       </c>
       <c r="T10" s="8" t="n">
-        <v>0.09624000000000001</v>
+        <v>0.09622</v>
       </c>
       <c r="U10" s="8" t="n">
         <v>0.00481</v>
       </c>
       <c r="V10" s="8" t="n">
-        <v>0.0072</v>
+        <v>0.00719</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>0.26582</v>
+        <v>0.26566</v>
       </c>
       <c r="X10" s="8" t="n">
         <v>0.01709</v>
       </c>
       <c r="Y10" s="8" t="n">
-        <v>0.1225649698035137</v>
+        <v>0.1225934232293224</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>0.1245671174554098</v>
+        <v>0.1245955523456179</v>
       </c>
     </row>
     <row r="11">
@@ -1198,10 +1198,10 @@
         <v/>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0.14399</v>
+        <v>0.14403</v>
       </c>
       <c r="Q11" s="8" t="n">
-        <v>0.04791</v>
+        <v>0.04792</v>
       </c>
       <c r="R11" s="8" t="n">
         <v>0.01378</v>
@@ -1210,25 +1210,25 @@
         <v>0.03033</v>
       </c>
       <c r="T11" s="8" t="n">
-        <v>0.06206</v>
+        <v>0.06204</v>
       </c>
       <c r="U11" s="8" t="n">
         <v>0.009769999999999999</v>
       </c>
       <c r="V11" s="8" t="n">
-        <v>0.009560000000000001</v>
+        <v>0.009549999999999999</v>
       </c>
       <c r="W11" s="8" t="n">
-        <v>0.19136</v>
+        <v>0.19123</v>
       </c>
       <c r="X11" s="8" t="n">
         <v>0.02656</v>
       </c>
       <c r="Y11" s="8" t="n">
-        <v>0.1162631795682918</v>
+        <v>0.116295645916114</v>
       </c>
       <c r="Z11" s="8" t="n">
-        <v>0.1138554206296852</v>
+        <v>0.1138878277062259</v>
       </c>
     </row>
     <row r="12">
@@ -1295,10 +1295,10 @@
         <v/>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0.13318</v>
+        <v>0.13322</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>0.0448</v>
+        <v>0.04481</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>0.00755</v>
@@ -1307,25 +1307,25 @@
         <v>0.03722</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>0.06425</v>
+        <v>0.06424000000000001</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>0.02187</v>
+        <v>0.02188</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>0.00632</v>
+        <v>0.00631</v>
       </c>
       <c r="W12" s="8" t="n">
-        <v>0.21535</v>
+        <v>0.21522</v>
       </c>
       <c r="X12" s="8" t="n">
         <v>0.04791</v>
       </c>
       <c r="Y12" s="8" t="n">
-        <v>0.1303840936713495</v>
+        <v>0.1304267757380806</v>
       </c>
       <c r="Z12" s="8" t="n">
-        <v>0.1109838720594617</v>
+        <v>0.1110162084477117</v>
       </c>
     </row>
     <row r="13">
@@ -1392,10 +1392,10 @@
         <v/>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0.1288</v>
+        <v>0.12884</v>
       </c>
       <c r="Q13" s="8" t="n">
-        <v>0.04535</v>
+        <v>0.04536</v>
       </c>
       <c r="R13" s="8" t="n">
         <v>0.00096</v>
@@ -1404,25 +1404,25 @@
         <v>0.05815</v>
       </c>
       <c r="T13" s="8" t="n">
-        <v>0.09795</v>
+        <v>0.09793</v>
       </c>
       <c r="U13" s="8" t="n">
-        <v>0.02039</v>
+        <v>0.0204</v>
       </c>
       <c r="V13" s="8" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.008789999999999999</v>
       </c>
       <c r="W13" s="8" t="n">
-        <v>0.23444</v>
+        <v>0.2343</v>
       </c>
       <c r="X13" s="8" t="n">
         <v>0.00442</v>
       </c>
       <c r="Y13" s="8" t="n">
-        <v>0.123350145244416</v>
+        <v>0.1233803607544251</v>
       </c>
       <c r="Z13" s="8" t="n">
-        <v>0.1487504071531462</v>
+        <v>0.1487906166084317</v>
       </c>
     </row>
     <row r="14">
@@ -1489,10 +1489,10 @@
         <v/>
       </c>
       <c r="P14" s="8" t="n">
-        <v>0.14566</v>
+        <v>0.1457</v>
       </c>
       <c r="Q14" s="8" t="n">
-        <v>0.04705</v>
+        <v>0.04706</v>
       </c>
       <c r="R14" s="8" t="n">
         <v>0.00604</v>
@@ -1501,25 +1501,25 @@
         <v>0.02937</v>
       </c>
       <c r="T14" s="8" t="n">
-        <v>0.09564</v>
+        <v>0.09562</v>
       </c>
       <c r="U14" s="8" t="n">
         <v>0.009339999999999999</v>
       </c>
       <c r="V14" s="8" t="n">
-        <v>0.00493</v>
+        <v>0.00492</v>
       </c>
       <c r="W14" s="8" t="n">
-        <v>0.23024</v>
+        <v>0.2301</v>
       </c>
       <c r="X14" s="8" t="n">
         <v>0.02686</v>
       </c>
       <c r="Y14" s="8" t="n">
-        <v>0.1293301602858653</v>
+        <v>0.1293702734936025</v>
       </c>
       <c r="Z14" s="8" t="n">
-        <v>0.1023115444715284</v>
+        <v>0.1023416557133602</v>
       </c>
     </row>
     <row r="15">
@@ -1586,10 +1586,10 @@
         <v/>
       </c>
       <c r="P15" s="8" t="n">
-        <v>0.13786</v>
+        <v>0.1379</v>
       </c>
       <c r="Q15" s="8" t="n">
-        <v>0.04268</v>
+        <v>0.04269</v>
       </c>
       <c r="R15" s="8" t="n">
         <v>0.0013</v>
@@ -1598,25 +1598,25 @@
         <v>0.05437</v>
       </c>
       <c r="T15" s="8" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.08548</v>
       </c>
       <c r="U15" s="8" t="n">
         <v>0.00526</v>
       </c>
       <c r="V15" s="8" t="n">
-        <v>0.0063</v>
+        <v>0.00629</v>
       </c>
       <c r="W15" s="8" t="n">
-        <v>0.19668</v>
+        <v>0.19656</v>
       </c>
       <c r="X15" s="8" t="n">
         <v>0.009010000000000001</v>
       </c>
       <c r="Y15" s="8" t="n">
-        <v>0.1255049333383372</v>
+        <v>0.1255411479114942</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>0.1360360065829556</v>
+        <v>0.1360720231242267</v>
       </c>
     </row>
     <row r="16">
@@ -1683,37 +1683,37 @@
         <v/>
       </c>
       <c r="P16" s="8" t="n">
-        <v>0.11163</v>
+        <v>0.11167</v>
       </c>
       <c r="Q16" s="8" t="n">
-        <v>0.03637</v>
+        <v>0.03638</v>
       </c>
       <c r="R16" s="8" t="n">
         <v>0.00316</v>
       </c>
       <c r="S16" s="8" t="n">
-        <v>0.04596</v>
+        <v>0.04597</v>
       </c>
       <c r="T16" s="8" t="n">
-        <v>0.1407</v>
+        <v>0.14068</v>
       </c>
       <c r="U16" s="8" t="n">
-        <v>0.01374</v>
+        <v>0.01375</v>
       </c>
       <c r="V16" s="8" t="n">
-        <v>0.00504</v>
+        <v>0.00503</v>
       </c>
       <c r="W16" s="8" t="n">
-        <v>0.28268</v>
+        <v>0.28253</v>
       </c>
       <c r="X16" s="8" t="n">
         <v>0.0123</v>
       </c>
       <c r="Y16" s="8" t="n">
-        <v>0.1351549456017528</v>
+        <v>0.1351966789637865</v>
       </c>
       <c r="Z16" s="8" t="n">
-        <v>0.1085374860809867</v>
+        <v>0.108569014719431</v>
       </c>
     </row>
     <row r="17">
@@ -1780,10 +1780,10 @@
         <v/>
       </c>
       <c r="P17" s="8" t="n">
-        <v>0.13818</v>
+        <v>0.13822</v>
       </c>
       <c r="Q17" s="8" t="n">
-        <v>0.04945</v>
+        <v>0.04947</v>
       </c>
       <c r="R17" s="8" t="n">
         <v>0.00573</v>
@@ -1792,25 +1792,25 @@
         <v>0.03481</v>
       </c>
       <c r="T17" s="8" t="n">
-        <v>0.09485</v>
+        <v>0.09483</v>
       </c>
       <c r="U17" s="8" t="n">
-        <v>0.01436</v>
+        <v>0.01437</v>
       </c>
       <c r="V17" s="8" t="n">
-        <v>0.00511</v>
+        <v>0.0051</v>
       </c>
       <c r="W17" s="8" t="n">
-        <v>0.23914</v>
+        <v>0.239</v>
       </c>
       <c r="X17" s="8" t="n">
         <v>0.01286</v>
       </c>
       <c r="Y17" s="8" t="n">
-        <v>0.1229915969489033</v>
+        <v>0.1230230418459303</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>0.1157813761275328</v>
+        <v>0.1158126866287359</v>
       </c>
     </row>
     <row r="18">
@@ -1877,10 +1877,10 @@
         <v/>
       </c>
       <c r="P18" s="8" t="n">
-        <v>0.15895</v>
+        <v>0.15899</v>
       </c>
       <c r="Q18" s="8" t="n">
-        <v>0.04708</v>
+        <v>0.04709</v>
       </c>
       <c r="R18" s="8" t="n">
         <v>0.00192</v>
@@ -1889,25 +1889,25 @@
         <v>0.03974</v>
       </c>
       <c r="T18" s="8" t="n">
-        <v>0.07149999999999999</v>
+        <v>0.07148</v>
       </c>
       <c r="U18" s="8" t="n">
         <v>0.00718</v>
       </c>
       <c r="V18" s="8" t="n">
-        <v>0.00711</v>
+        <v>0.0071</v>
       </c>
       <c r="W18" s="8" t="n">
-        <v>0.16022</v>
+        <v>0.16011</v>
       </c>
       <c r="X18" s="8" t="n">
         <v>0.008869999999999999</v>
       </c>
       <c r="Y18" s="8" t="n">
-        <v>0.1081387284944334</v>
+        <v>0.1081688846180165</v>
       </c>
       <c r="Z18" s="8" t="n">
-        <v>0.128367869972501</v>
+        <v>0.1284077807000251</v>
       </c>
     </row>
     <row r="19">
@@ -1974,10 +1974,10 @@
         <v/>
       </c>
       <c r="P19" s="8" t="n">
-        <v>0.18566</v>
+        <v>0.1857</v>
       </c>
       <c r="Q19" s="8" t="n">
-        <v>0.03121</v>
+        <v>0.03122</v>
       </c>
       <c r="R19" s="8" t="n">
         <v>0.00534</v>
@@ -1986,25 +1986,25 @@
         <v>0.00733</v>
       </c>
       <c r="T19" s="8" t="n">
-        <v>0.09446</v>
+        <v>0.09444</v>
       </c>
       <c r="U19" s="8" t="n">
         <v>0.00284</v>
       </c>
       <c r="V19" s="8" t="n">
-        <v>0.007939999999999999</v>
+        <v>0.00793</v>
       </c>
       <c r="W19" s="8" t="n">
-        <v>0.15582</v>
+        <v>0.15571</v>
       </c>
       <c r="X19" s="8" t="n">
         <v>0.04288</v>
       </c>
       <c r="Y19" s="8" t="n">
-        <v>0.109697094751451</v>
+        <v>0.1097258217418803</v>
       </c>
       <c r="Z19" s="8" t="n">
-        <v>0.0788397382013374</v>
+        <v>0.0788589008153579</v>
       </c>
     </row>
     <row r="20">
@@ -2071,10 +2071,10 @@
         <v/>
       </c>
       <c r="P20" s="8" t="n">
-        <v>0.13679</v>
+        <v>0.13683</v>
       </c>
       <c r="Q20" s="8" t="n">
-        <v>0.04443</v>
+        <v>0.04444</v>
       </c>
       <c r="R20" s="8" t="n">
         <v>0.00356</v>
@@ -2083,25 +2083,25 @@
         <v>0.03164</v>
       </c>
       <c r="T20" s="8" t="n">
-        <v>0.073</v>
+        <v>0.07299</v>
       </c>
       <c r="U20" s="8" t="n">
         <v>0.00865</v>
       </c>
       <c r="V20" s="8" t="n">
-        <v>0.00526</v>
+        <v>0.00525</v>
       </c>
       <c r="W20" s="8" t="n">
-        <v>0.27024</v>
+        <v>0.27008</v>
       </c>
       <c r="X20" s="8" t="n">
         <v>0.02463</v>
       </c>
       <c r="Y20" s="8" t="n">
-        <v>0.1129101061646542</v>
+        <v>0.1129403520129875</v>
       </c>
       <c r="Z20" s="8" t="n">
-        <v>0.1171940346426323</v>
+        <v>0.1172243610493367</v>
       </c>
     </row>
     <row r="21">
@@ -2168,10 +2168,10 @@
         <v/>
       </c>
       <c r="P21" s="8" t="n">
-        <v>0.1446</v>
+        <v>0.14464</v>
       </c>
       <c r="Q21" s="8" t="n">
-        <v>0.03967</v>
+        <v>0.03968</v>
       </c>
       <c r="R21" s="8" t="n">
         <v>0.00765</v>
@@ -2180,25 +2180,25 @@
         <v>0.01771</v>
       </c>
       <c r="T21" s="8" t="n">
-        <v>0.11217</v>
+        <v>0.11214</v>
       </c>
       <c r="U21" s="8" t="n">
-        <v>0.01873</v>
+        <v>0.01874</v>
       </c>
       <c r="V21" s="8" t="n">
         <v>0.0027</v>
       </c>
       <c r="W21" s="8" t="n">
-        <v>0.21134</v>
+        <v>0.2112</v>
       </c>
       <c r="X21" s="8" t="n">
         <v>0.04402</v>
       </c>
       <c r="Y21" s="8" t="n">
-        <v>0.1191814316276485</v>
+        <v>0.1192101773713967</v>
       </c>
       <c r="Z21" s="8" t="n">
-        <v>0.0846367777749651</v>
+        <v>0.0846559518514351</v>
       </c>
     </row>
     <row r="22">
@@ -2265,10 +2265,10 @@
         <v/>
       </c>
       <c r="P22" s="8" t="n">
-        <v>0.18452</v>
+        <v>0.18455</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>0.04556</v>
+        <v>0.04557</v>
       </c>
       <c r="R22" s="8" t="n">
         <v>0.00671</v>
@@ -2277,25 +2277,25 @@
         <v>0.01458</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>0.06333</v>
+        <v>0.06331000000000001</v>
       </c>
       <c r="U22" s="8" t="n">
         <v>0.01013</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>0.00725</v>
+        <v>0.00724</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>0.11711</v>
+        <v>0.11702</v>
       </c>
       <c r="X22" s="8" t="n">
         <v>0.01942</v>
       </c>
       <c r="Y22" s="8" t="n">
-        <v>0.1134418832123613</v>
+        <v>0.1134704210984195</v>
       </c>
       <c r="Z22" s="8" t="n">
-        <v>0.0933020531376229</v>
+        <v>0.0933307774753884</v>
       </c>
     </row>
     <row r="23">
@@ -2362,10 +2362,10 @@
         <v/>
       </c>
       <c r="P23" s="8" t="n">
-        <v>0.17705</v>
+        <v>0.17709</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>0.03649</v>
+        <v>0.0365</v>
       </c>
       <c r="R23" s="8" t="n">
         <v>0.00173</v>
@@ -2374,25 +2374,25 @@
         <v>0.02963</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>0.09204</v>
+        <v>0.09200999999999999</v>
       </c>
       <c r="U23" s="8" t="n">
         <v>0.01064</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>0.00572</v>
+        <v>0.00571</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>0.14926</v>
+        <v>0.14916</v>
       </c>
       <c r="X23" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="Y23" s="8" t="n">
-        <v>0.1167386828077894</v>
+        <v>0.1167654185675505</v>
       </c>
       <c r="Z23" s="8" t="n">
-        <v>0.1117624613845082</v>
+        <v>0.1117892907197758</v>
       </c>
     </row>
     <row r="24">
@@ -2459,10 +2459,10 @@
         <v/>
       </c>
       <c r="P24" s="8" t="n">
-        <v>0.11651</v>
+        <v>0.11655</v>
       </c>
       <c r="Q24" s="8" t="n">
-        <v>0.04933</v>
+        <v>0.04935</v>
       </c>
       <c r="R24" s="8" t="n">
         <v>0.00157</v>
@@ -2471,25 +2471,25 @@
         <v>0.0472</v>
       </c>
       <c r="T24" s="8" t="n">
-        <v>0.10954</v>
+        <v>0.10952</v>
       </c>
       <c r="U24" s="8" t="n">
         <v>0.00672</v>
       </c>
       <c r="V24" s="8" t="n">
-        <v>0.0067</v>
+        <v>0.00669</v>
       </c>
       <c r="W24" s="8" t="n">
-        <v>0.24663</v>
+        <v>0.24649</v>
       </c>
       <c r="X24" s="8" t="n">
         <v>0.00144</v>
       </c>
       <c r="Y24" s="8" t="n">
-        <v>0.1267111927789676</v>
+        <v>0.1267409005075677</v>
       </c>
       <c r="Z24" s="8" t="n">
-        <v>0.133170417963377</v>
+        <v>0.1332102973321215</v>
       </c>
     </row>
     <row r="25">
@@ -2556,10 +2556,10 @@
         <v/>
       </c>
       <c r="P25" s="8" t="n">
-        <v>0.11356</v>
+        <v>0.1136</v>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>0.04871</v>
+        <v>0.04873</v>
       </c>
       <c r="R25" s="8" t="n">
         <v>0.00231</v>
@@ -2568,25 +2568,25 @@
         <v>0.04961</v>
       </c>
       <c r="T25" s="8" t="n">
-        <v>0.09122</v>
+        <v>0.09121</v>
       </c>
       <c r="U25" s="8" t="n">
-        <v>0.01075</v>
+        <v>0.01076</v>
       </c>
       <c r="V25" s="8" t="n">
-        <v>0.00572</v>
+        <v>0.00571</v>
       </c>
       <c r="W25" s="8" t="n">
-        <v>0.277</v>
+        <v>0.27684</v>
       </c>
       <c r="X25" s="8" t="n">
         <v>0.01097</v>
       </c>
       <c r="Y25" s="8" t="n">
-        <v>0.1275988435967263</v>
+        <v>0.1276311387344904</v>
       </c>
       <c r="Z25" s="8" t="n">
-        <v>0.147048298239513</v>
+        <v>0.1470909543443185</v>
       </c>
     </row>
     <row r="26">
@@ -2653,10 +2653,10 @@
         <v/>
       </c>
       <c r="P26" s="8" t="n">
-        <v>0.14496</v>
+        <v>0.145</v>
       </c>
       <c r="Q26" s="8" t="n">
-        <v>0.03891</v>
+        <v>0.03892</v>
       </c>
       <c r="R26" s="8" t="n">
         <v>0.00152</v>
@@ -2665,25 +2665,25 @@
         <v>0.03139</v>
       </c>
       <c r="T26" s="8" t="n">
-        <v>0.09826</v>
+        <v>0.09823999999999999</v>
       </c>
       <c r="U26" s="8" t="n">
-        <v>0.0315</v>
+        <v>0.03151</v>
       </c>
       <c r="V26" s="8" t="n">
-        <v>0.007849999999999999</v>
+        <v>0.00784</v>
       </c>
       <c r="W26" s="8" t="n">
-        <v>0.20141</v>
+        <v>0.20128</v>
       </c>
       <c r="X26" s="8" t="n">
         <v>0.01169</v>
       </c>
       <c r="Y26" s="8" t="n">
-        <v>0.1208124074927408</v>
+        <v>0.1208521761413874</v>
       </c>
       <c r="Z26" s="8" t="n">
-        <v>0.1040610285208656</v>
+        <v>0.1040911079641611</v>
       </c>
     </row>
     <row r="27">
@@ -2750,10 +2750,10 @@
         <v/>
       </c>
       <c r="P27" s="8" t="n">
-        <v>0.14138</v>
+        <v>0.14142</v>
       </c>
       <c r="Q27" s="8" t="n">
-        <v>0.04342</v>
+        <v>0.04343</v>
       </c>
       <c r="R27" s="8" t="n">
         <v>0.00915</v>
@@ -2762,25 +2762,25 @@
         <v>0.02754</v>
       </c>
       <c r="T27" s="8" t="n">
-        <v>0.07296999999999999</v>
+        <v>0.07296</v>
       </c>
       <c r="U27" s="8" t="n">
-        <v>0.01146</v>
+        <v>0.01147</v>
       </c>
       <c r="V27" s="8" t="n">
-        <v>0.00602</v>
+        <v>0.00601</v>
       </c>
       <c r="W27" s="8" t="n">
-        <v>0.25103</v>
+        <v>0.25088</v>
       </c>
       <c r="X27" s="8" t="n">
         <v>0.0397</v>
       </c>
       <c r="Y27" s="8" t="n">
-        <v>0.1154204542066042</v>
+        <v>0.1154503661598059</v>
       </c>
       <c r="Z27" s="8" t="n">
-        <v>0.1027000453277901</v>
+        <v>0.102729920964542</v>
       </c>
     </row>
     <row r="28">
@@ -2847,10 +2847,10 @@
         <v/>
       </c>
       <c r="P28" s="8" t="n">
-        <v>0.14584</v>
+        <v>0.14589</v>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>0.04295</v>
+        <v>0.04296</v>
       </c>
       <c r="R28" s="8" t="n">
         <v>0.00178</v>
@@ -2859,25 +2859,25 @@
         <v>0.03658</v>
       </c>
       <c r="T28" s="8" t="n">
-        <v>0.09723999999999999</v>
+        <v>0.09722</v>
       </c>
       <c r="U28" s="8" t="n">
-        <v>0.01611</v>
+        <v>0.01612</v>
       </c>
       <c r="V28" s="8" t="n">
-        <v>0.00886</v>
+        <v>0.00885</v>
       </c>
       <c r="W28" s="8" t="n">
-        <v>0.25138</v>
+        <v>0.25123</v>
       </c>
       <c r="X28" s="8" t="n">
         <v>0.00285</v>
       </c>
       <c r="Y28" s="8" t="n">
-        <v>0.1131704620197777</v>
+        <v>0.1131972648782547</v>
       </c>
       <c r="Z28" s="8" t="n">
-        <v>0.120239396716028</v>
+        <v>0.1202660666465083</v>
       </c>
     </row>
     <row r="29">
@@ -2944,37 +2944,37 @@
         <v/>
       </c>
       <c r="P29" s="8" t="n">
-        <v>0.09571</v>
+        <v>0.09575</v>
       </c>
       <c r="Q29" s="8" t="n">
-        <v>0.03736</v>
+        <v>0.03737</v>
       </c>
       <c r="R29" s="8" t="n">
         <v>0.00154</v>
       </c>
       <c r="S29" s="8" t="n">
-        <v>0.06152</v>
+        <v>0.06153</v>
       </c>
       <c r="T29" s="8" t="n">
-        <v>0.14571</v>
+        <v>0.1457</v>
       </c>
       <c r="U29" s="8" t="n">
-        <v>0.00946</v>
+        <v>0.009469999999999999</v>
       </c>
       <c r="V29" s="8" t="n">
-        <v>0.00564</v>
+        <v>0.00563</v>
       </c>
       <c r="W29" s="8" t="n">
-        <v>0.29639</v>
+        <v>0.29624</v>
       </c>
       <c r="X29" s="8" t="n">
         <v>0.00756</v>
       </c>
       <c r="Y29" s="8" t="n">
-        <v>0.1376809194020578</v>
+        <v>0.1377218230785208</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>0.1405627323146818</v>
+        <v>0.1406036335100544</v>
       </c>
     </row>
     <row r="30">
@@ -3041,10 +3041,10 @@
         <v/>
       </c>
       <c r="P30" s="8" t="n">
-        <v>0.13893</v>
+        <v>0.13896</v>
       </c>
       <c r="Q30" s="8" t="n">
-        <v>0.04323</v>
+        <v>0.04324</v>
       </c>
       <c r="R30" s="8" t="n">
         <v>0.007889999999999999</v>
@@ -3053,25 +3053,25 @@
         <v>0.02952</v>
       </c>
       <c r="T30" s="8" t="n">
-        <v>0.12496</v>
+        <v>0.12493</v>
       </c>
       <c r="U30" s="8" t="n">
         <v>0.00483</v>
       </c>
       <c r="V30" s="8" t="n">
-        <v>0.0057</v>
+        <v>0.00569</v>
       </c>
       <c r="W30" s="8" t="n">
-        <v>0.15647</v>
+        <v>0.15636</v>
       </c>
       <c r="X30" s="8" t="n">
         <v>0.01801</v>
       </c>
       <c r="Y30" s="8" t="n">
-        <v>0.1299404821594245</v>
+        <v>0.1299821007704813</v>
       </c>
       <c r="Z30" s="8" t="n">
-        <v>0.1026713963924373</v>
+        <v>0.1027026562992671</v>
       </c>
     </row>
     <row r="33">
@@ -3205,7 +3205,7 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>228.2</v>
+        <v>228.4</v>
       </c>
       <c r="E35" s="6">
         <f>D35*N35</f>
@@ -3247,25 +3247,25 @@
         <v>4.174</v>
       </c>
       <c r="O35" s="8" t="n">
-        <v>0.21729</v>
+        <v>0.21751</v>
       </c>
       <c r="P35" s="8" t="n">
-        <v>0.05734</v>
+        <v>0.05737</v>
       </c>
       <c r="Q35" s="8" t="n">
-        <v>0.02094</v>
+        <v>0.02097</v>
       </c>
       <c r="R35" s="8" t="n">
-        <v>0.17105</v>
+        <v>0.17092</v>
       </c>
       <c r="S35" s="8" t="n">
-        <v>0.03989</v>
+        <v>0.03986</v>
       </c>
       <c r="T35" s="8" t="n">
         <v>0.00497</v>
       </c>
       <c r="U35" s="8" t="n">
-        <v>3.79891</v>
+        <v>3.79741</v>
       </c>
     </row>
     <row r="36">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>215.4</v>
+        <v>215.5</v>
       </c>
       <c r="E36" s="6">
         <f>D36*N36</f>
@@ -3327,25 +3327,25 @@
         <v>4.221</v>
       </c>
       <c r="O36" s="8" t="n">
-        <v>0.19046</v>
+        <v>0.19066</v>
       </c>
       <c r="P36" s="8" t="n">
-        <v>0.06854</v>
+        <v>0.06858</v>
       </c>
       <c r="Q36" s="8" t="n">
-        <v>0.02662</v>
+        <v>0.02666</v>
       </c>
       <c r="R36" s="8" t="n">
-        <v>0.15459</v>
+        <v>0.15448</v>
       </c>
       <c r="S36" s="8" t="n">
-        <v>0.04576</v>
+        <v>0.04573</v>
       </c>
       <c r="T36" s="8" t="n">
         <v>0.00441</v>
       </c>
       <c r="U36" s="8" t="n">
-        <v>4.16804</v>
+        <v>4.16652</v>
       </c>
     </row>
     <row r="37">
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>210.2</v>
+        <v>210.5</v>
       </c>
       <c r="E37" s="6">
         <f>D37*N37</f>
@@ -3407,25 +3407,25 @@
         <v>4.207</v>
       </c>
       <c r="O37" s="8" t="n">
-        <v>0.2546</v>
+        <v>0.25484</v>
       </c>
       <c r="P37" s="8" t="n">
-        <v>0.09235</v>
+        <v>0.0924</v>
       </c>
       <c r="Q37" s="8" t="n">
-        <v>0.02139</v>
+        <v>0.02142</v>
       </c>
       <c r="R37" s="8" t="n">
-        <v>0.13535</v>
+        <v>0.13523</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>0.03727</v>
+        <v>0.03724</v>
       </c>
       <c r="T37" s="8" t="n">
         <v>0.00316</v>
       </c>
       <c r="U37" s="8" t="n">
-        <v>3.59592</v>
+        <v>3.59469</v>
       </c>
     </row>
     <row r="38">
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>201.7</v>
+        <v>202.1</v>
       </c>
       <c r="E38" s="6">
         <f>D38*N38</f>
@@ -3484,28 +3484,28 @@
         <v/>
       </c>
       <c r="N38" s="8" t="n">
-        <v>4.333</v>
+        <v>4.332</v>
       </c>
       <c r="O38" s="8" t="n">
-        <v>0.16276</v>
+        <v>0.16294</v>
       </c>
       <c r="P38" s="8" t="n">
-        <v>0.08613</v>
+        <v>0.08619</v>
       </c>
       <c r="Q38" s="8" t="n">
-        <v>0.02064</v>
+        <v>0.02067</v>
       </c>
       <c r="R38" s="8" t="n">
-        <v>0.1733</v>
+        <v>0.17318</v>
       </c>
       <c r="S38" s="8" t="n">
-        <v>0.03684</v>
+        <v>0.03682</v>
       </c>
       <c r="T38" s="8" t="n">
         <v>0.00408</v>
       </c>
       <c r="U38" s="8" t="n">
-        <v>4.20236</v>
+        <v>4.20085</v>
       </c>
     </row>
     <row r="39">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>200.9</v>
+        <v>201.2</v>
       </c>
       <c r="E39" s="6">
         <f>D39*N39</f>
@@ -3567,25 +3567,25 @@
         <v>4.272</v>
       </c>
       <c r="O39" s="8" t="n">
-        <v>0.16528</v>
+        <v>0.16546</v>
       </c>
       <c r="P39" s="8" t="n">
-        <v>0.06435</v>
+        <v>0.06439</v>
       </c>
       <c r="Q39" s="8" t="n">
-        <v>0.03331</v>
+        <v>0.03336</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>0.16407</v>
+        <v>0.16395</v>
       </c>
       <c r="S39" s="8" t="n">
-        <v>0.04724</v>
+        <v>0.04721</v>
       </c>
       <c r="T39" s="8" t="n">
         <v>0.0044</v>
       </c>
       <c r="U39" s="8" t="n">
-        <v>4.66116</v>
+        <v>4.66031</v>
       </c>
     </row>
     <row r="40">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>190.7</v>
+        <v>191.1</v>
       </c>
       <c r="E40" s="6">
         <f>D40*N40</f>
@@ -3644,28 +3644,28 @@
         <v/>
       </c>
       <c r="N40" s="8" t="n">
-        <v>4.321</v>
+        <v>4.32</v>
       </c>
       <c r="O40" s="8" t="n">
-        <v>0.20161</v>
+        <v>0.20181</v>
       </c>
       <c r="P40" s="8" t="n">
-        <v>0.07896</v>
+        <v>0.07901</v>
       </c>
       <c r="Q40" s="8" t="n">
-        <v>0.03674</v>
+        <v>0.03679</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>0.15011</v>
+        <v>0.14999</v>
       </c>
       <c r="S40" s="8" t="n">
-        <v>0.04817</v>
+        <v>0.04814</v>
       </c>
       <c r="T40" s="8" t="n">
         <v>0.00347</v>
       </c>
       <c r="U40" s="8" t="n">
-        <v>4.81222</v>
+        <v>4.81132</v>
       </c>
     </row>
     <row r="41">
@@ -3727,25 +3727,25 @@
         <v>4.106</v>
       </c>
       <c r="O41" s="8" t="n">
-        <v>0.24011</v>
+        <v>0.24035</v>
       </c>
       <c r="P41" s="8" t="n">
-        <v>0.05777</v>
+        <v>0.0578</v>
       </c>
       <c r="Q41" s="8" t="n">
-        <v>0.02026</v>
+        <v>0.02029</v>
       </c>
       <c r="R41" s="8" t="n">
-        <v>0.16371</v>
+        <v>0.16358</v>
       </c>
       <c r="S41" s="8" t="n">
-        <v>0.03965</v>
+        <v>0.03962</v>
       </c>
       <c r="T41" s="8" t="n">
         <v>0.00258</v>
       </c>
       <c r="U41" s="8" t="n">
-        <v>3.46143</v>
+        <v>3.46002</v>
       </c>
     </row>
     <row r="42">
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>188.3</v>
+        <v>188.5</v>
       </c>
       <c r="E42" s="6">
         <f>D42*N42</f>
@@ -3807,25 +3807,25 @@
         <v>4.167</v>
       </c>
       <c r="O42" s="8" t="n">
-        <v>0.19514</v>
+        <v>0.19534</v>
       </c>
       <c r="P42" s="8" t="n">
-        <v>0.06849</v>
+        <v>0.06852999999999999</v>
       </c>
       <c r="Q42" s="8" t="n">
-        <v>0.03138</v>
+        <v>0.03142</v>
       </c>
       <c r="R42" s="8" t="n">
-        <v>0.13919</v>
+        <v>0.13908</v>
       </c>
       <c r="S42" s="8" t="n">
-        <v>0.04856</v>
+        <v>0.04853</v>
       </c>
       <c r="T42" s="8" t="n">
         <v>0.00603</v>
       </c>
       <c r="U42" s="8" t="n">
-        <v>4.19931</v>
+        <v>4.19852</v>
       </c>
     </row>
     <row r="43">
@@ -3845,7 +3845,7 @@
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>186.2</v>
+        <v>186.4</v>
       </c>
       <c r="E43" s="6">
         <f>D43*N43</f>
@@ -3884,28 +3884,28 @@
         <v/>
       </c>
       <c r="N43" s="8" t="n">
-        <v>4.006</v>
+        <v>4.005</v>
       </c>
       <c r="O43" s="8" t="n">
-        <v>0.28382</v>
+        <v>0.28408</v>
       </c>
       <c r="P43" s="8" t="n">
-        <v>0.0663</v>
+        <v>0.06633</v>
       </c>
       <c r="Q43" s="8" t="n">
-        <v>0.02319</v>
+        <v>0.02322</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>0.12969</v>
+        <v>0.12957</v>
       </c>
       <c r="S43" s="8" t="n">
-        <v>0.03776</v>
+        <v>0.03773</v>
       </c>
       <c r="T43" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="U43" s="8" t="n">
-        <v>3.09759</v>
+        <v>3.09649</v>
       </c>
     </row>
     <row r="44">
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>182.5</v>
+        <v>182.6</v>
       </c>
       <c r="E44" s="6">
         <f>D44*N44</f>
@@ -3967,25 +3967,25 @@
         <v>4.237</v>
       </c>
       <c r="O44" s="8" t="n">
-        <v>0.23535</v>
+        <v>0.23557</v>
       </c>
       <c r="P44" s="8" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.07543999999999999</v>
       </c>
       <c r="Q44" s="8" t="n">
-        <v>0.03878</v>
+        <v>0.03883</v>
       </c>
       <c r="R44" s="8" t="n">
-        <v>0.13145</v>
+        <v>0.13134</v>
       </c>
       <c r="S44" s="8" t="n">
-        <v>0.04773</v>
+        <v>0.04769</v>
       </c>
       <c r="T44" s="8" t="n">
         <v>0.0037</v>
       </c>
       <c r="U44" s="8" t="n">
-        <v>4.5295</v>
+        <v>4.52874</v>
       </c>
     </row>
     <row r="45">
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>178.8</v>
+        <v>179.2</v>
       </c>
       <c r="E45" s="6">
         <f>D45*N45</f>
@@ -4047,25 +4047,25 @@
         <v>4.248</v>
       </c>
       <c r="O45" s="8" t="n">
-        <v>0.21747</v>
+        <v>0.21769</v>
       </c>
       <c r="P45" s="8" t="n">
-        <v>0.08298999999999999</v>
+        <v>0.08304</v>
       </c>
       <c r="Q45" s="8" t="n">
-        <v>0.01963</v>
+        <v>0.01966</v>
       </c>
       <c r="R45" s="8" t="n">
-        <v>0.15444</v>
+        <v>0.15432</v>
       </c>
       <c r="S45" s="8" t="n">
-        <v>0.04099</v>
+        <v>0.04096</v>
       </c>
       <c r="T45" s="8" t="n">
         <v>0.00366</v>
       </c>
       <c r="U45" s="8" t="n">
-        <v>3.84543</v>
+        <v>3.84354</v>
       </c>
     </row>
     <row r="46">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>178.6</v>
+        <v>178.9</v>
       </c>
       <c r="E46" s="6">
         <f>D46*N46</f>
@@ -4124,28 +4124,28 @@
         <v/>
       </c>
       <c r="N46" s="8" t="n">
-        <v>4.13</v>
+        <v>4.129</v>
       </c>
       <c r="O46" s="8" t="n">
-        <v>0.26032</v>
+        <v>0.26056</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>0.09154</v>
+        <v>0.09159</v>
       </c>
       <c r="Q46" s="8" t="n">
-        <v>0.02041</v>
+        <v>0.02044</v>
       </c>
       <c r="R46" s="8" t="n">
-        <v>0.14146</v>
+        <v>0.14134</v>
       </c>
       <c r="S46" s="8" t="n">
-        <v>0.02817</v>
+        <v>0.02815</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0.00328</v>
       </c>
       <c r="U46" s="8" t="n">
-        <v>3.22753</v>
+        <v>3.22594</v>
       </c>
     </row>
     <row r="47">
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>178.5</v>
+        <v>178.8</v>
       </c>
       <c r="E47" s="6">
         <f>D47*N47</f>
@@ -4207,25 +4207,25 @@
         <v>4.047</v>
       </c>
       <c r="O47" s="8" t="n">
-        <v>0.29977</v>
+        <v>0.30004</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>0.06676</v>
+        <v>0.06679</v>
       </c>
       <c r="Q47" s="8" t="n">
-        <v>0.02928</v>
+        <v>0.02932</v>
       </c>
       <c r="R47" s="8" t="n">
-        <v>0.1335</v>
+        <v>0.13338</v>
       </c>
       <c r="S47" s="8" t="n">
-        <v>0.03956</v>
+        <v>0.03953</v>
       </c>
       <c r="T47" s="8" t="n">
         <v>0.00272</v>
       </c>
       <c r="U47" s="8" t="n">
-        <v>3.42705</v>
+        <v>3.42538</v>
       </c>
     </row>
     <row r="48">
@@ -4245,7 +4245,7 @@
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>175.5</v>
+        <v>175.8</v>
       </c>
       <c r="E48" s="6">
         <f>D48*N48</f>
@@ -4287,25 +4287,25 @@
         <v>4.342</v>
       </c>
       <c r="O48" s="8" t="n">
-        <v>0.20555</v>
+        <v>0.20576</v>
       </c>
       <c r="P48" s="8" t="n">
-        <v>0.07463</v>
+        <v>0.07467</v>
       </c>
       <c r="Q48" s="8" t="n">
-        <v>0.02953</v>
+        <v>0.02957</v>
       </c>
       <c r="R48" s="8" t="n">
-        <v>0.15527</v>
+        <v>0.15515</v>
       </c>
       <c r="S48" s="8" t="n">
-        <v>0.04904</v>
+        <v>0.04901</v>
       </c>
       <c r="T48" s="8" t="n">
         <v>0.0043</v>
       </c>
       <c r="U48" s="8" t="n">
-        <v>4.66242</v>
+        <v>4.66145</v>
       </c>
     </row>
     <row r="49">
@@ -4325,7 +4325,7 @@
         </is>
       </c>
       <c r="D49" s="5" t="n">
-        <v>174.9</v>
+        <v>175</v>
       </c>
       <c r="E49" s="6">
         <f>D49*N49</f>
@@ -4367,25 +4367,25 @@
         <v>4.031</v>
       </c>
       <c r="O49" s="8" t="n">
-        <v>0.26141</v>
+        <v>0.26166</v>
       </c>
       <c r="P49" s="8" t="n">
-        <v>0.05909</v>
+        <v>0.05912</v>
       </c>
       <c r="Q49" s="8" t="n">
-        <v>0.03671</v>
+        <v>0.03676</v>
       </c>
       <c r="R49" s="8" t="n">
-        <v>0.13074</v>
+        <v>0.13063</v>
       </c>
       <c r="S49" s="8" t="n">
-        <v>0.04067</v>
+        <v>0.04064</v>
       </c>
       <c r="T49" s="8" t="n">
         <v>0.00277</v>
       </c>
       <c r="U49" s="8" t="n">
-        <v>3.69946</v>
+        <v>3.69867</v>
       </c>
     </row>
     <row r="50">
@@ -4405,7 +4405,7 @@
         </is>
       </c>
       <c r="D50" s="5" t="n">
-        <v>173.7</v>
+        <v>174</v>
       </c>
       <c r="E50" s="6">
         <f>D50*N50</f>
@@ -4444,28 +4444,28 @@
         <v/>
       </c>
       <c r="N50" s="8" t="n">
-        <v>4.337</v>
+        <v>4.336</v>
       </c>
       <c r="O50" s="8" t="n">
-        <v>0.19035</v>
+        <v>0.19054</v>
       </c>
       <c r="P50" s="8" t="n">
-        <v>0.08605</v>
+        <v>0.0861</v>
       </c>
       <c r="Q50" s="8" t="n">
-        <v>0.0431</v>
+        <v>0.04316</v>
       </c>
       <c r="R50" s="8" t="n">
-        <v>0.1397</v>
+        <v>0.13959</v>
       </c>
       <c r="S50" s="8" t="n">
-        <v>0.04403</v>
+        <v>0.044</v>
       </c>
       <c r="T50" s="8" t="n">
         <v>0.00459</v>
       </c>
       <c r="U50" s="8" t="n">
-        <v>5.02712</v>
+        <v>5.0275</v>
       </c>
     </row>
     <row r="51">
@@ -4485,7 +4485,7 @@
         </is>
       </c>
       <c r="D51" s="5" t="n">
-        <v>172.2</v>
+        <v>172.4</v>
       </c>
       <c r="E51" s="6">
         <f>D51*N51</f>
@@ -4524,28 +4524,28 @@
         <v/>
       </c>
       <c r="N51" s="8" t="n">
-        <v>4.187</v>
+        <v>4.186</v>
       </c>
       <c r="O51" s="8" t="n">
-        <v>0.20619</v>
+        <v>0.2064</v>
       </c>
       <c r="P51" s="8" t="n">
-        <v>0.07961</v>
+        <v>0.07965999999999999</v>
       </c>
       <c r="Q51" s="8" t="n">
-        <v>0.03036</v>
+        <v>0.0304</v>
       </c>
       <c r="R51" s="8" t="n">
-        <v>0.1421</v>
+        <v>0.14199</v>
       </c>
       <c r="S51" s="8" t="n">
-        <v>0.04202</v>
+        <v>0.04199</v>
       </c>
       <c r="T51" s="8" t="n">
         <v>0.00353</v>
       </c>
       <c r="U51" s="8" t="n">
-        <v>4.04272</v>
+        <v>4.04163</v>
       </c>
     </row>
     <row r="52">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>171.1</v>
+        <v>171.3</v>
       </c>
       <c r="E52" s="6">
         <f>D52*N52</f>
@@ -4607,25 +4607,25 @@
         <v>4.231</v>
       </c>
       <c r="O52" s="8" t="n">
-        <v>0.20511</v>
+        <v>0.20531</v>
       </c>
       <c r="P52" s="8" t="n">
-        <v>0.07983</v>
+        <v>0.07988000000000001</v>
       </c>
       <c r="Q52" s="8" t="n">
-        <v>0.03961</v>
+        <v>0.03966</v>
       </c>
       <c r="R52" s="8" t="n">
-        <v>0.13805</v>
+        <v>0.13794</v>
       </c>
       <c r="S52" s="8" t="n">
-        <v>0.04577</v>
+        <v>0.04574</v>
       </c>
       <c r="T52" s="8" t="n">
         <v>0.00309</v>
       </c>
       <c r="U52" s="8" t="n">
-        <v>4.54682</v>
+        <v>4.54668</v>
       </c>
     </row>
     <row r="53">
@@ -4645,7 +4645,7 @@
         </is>
       </c>
       <c r="D53" s="5" t="n">
-        <v>170.2</v>
+        <v>170.3</v>
       </c>
       <c r="E53" s="6">
         <f>D53*N53</f>
@@ -4684,28 +4684,28 @@
         <v/>
       </c>
       <c r="N53" s="8" t="n">
-        <v>4.039</v>
+        <v>4.038</v>
       </c>
       <c r="O53" s="8" t="n">
-        <v>0.24151</v>
+        <v>0.24175</v>
       </c>
       <c r="P53" s="8" t="n">
-        <v>0.05525</v>
+        <v>0.05528</v>
       </c>
       <c r="Q53" s="8" t="n">
-        <v>0.02801</v>
+        <v>0.02805</v>
       </c>
       <c r="R53" s="8" t="n">
-        <v>0.14148</v>
+        <v>0.14136</v>
       </c>
       <c r="S53" s="8" t="n">
-        <v>0.04106</v>
+        <v>0.04103</v>
       </c>
       <c r="T53" s="8" t="n">
         <v>0.00299</v>
       </c>
       <c r="U53" s="8" t="n">
-        <v>3.49029</v>
+        <v>3.48925</v>
       </c>
     </row>
     <row r="54">
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>169.8</v>
+        <v>170.1</v>
       </c>
       <c r="E54" s="6">
         <f>D54*N54</f>
@@ -4767,25 +4767,25 @@
         <v>4.305</v>
       </c>
       <c r="O54" s="8" t="n">
-        <v>0.21232</v>
+        <v>0.21253</v>
       </c>
       <c r="P54" s="8" t="n">
-        <v>0.1069</v>
+        <v>0.10696</v>
       </c>
       <c r="Q54" s="8" t="n">
-        <v>0.0193</v>
+        <v>0.01933</v>
       </c>
       <c r="R54" s="8" t="n">
-        <v>0.14244</v>
+        <v>0.14232</v>
       </c>
       <c r="S54" s="8" t="n">
-        <v>0.04333</v>
+        <v>0.0433</v>
       </c>
       <c r="T54" s="8" t="n">
         <v>0.0043</v>
       </c>
       <c r="U54" s="8" t="n">
-        <v>3.97224</v>
+        <v>3.9709</v>
       </c>
     </row>
     <row r="55">
@@ -4805,7 +4805,7 @@
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>169.5</v>
+        <v>169.7</v>
       </c>
       <c r="E55" s="6">
         <f>D55*N55</f>
@@ -4847,25 +4847,25 @@
         <v>4.282</v>
       </c>
       <c r="O55" s="8" t="n">
-        <v>0.20278</v>
+        <v>0.20298</v>
       </c>
       <c r="P55" s="8" t="n">
-        <v>0.07198</v>
+        <v>0.07202</v>
       </c>
       <c r="Q55" s="8" t="n">
-        <v>0.03632</v>
+        <v>0.03637</v>
       </c>
       <c r="R55" s="8" t="n">
-        <v>0.14842</v>
+        <v>0.1483</v>
       </c>
       <c r="S55" s="8" t="n">
-        <v>0.04769</v>
+        <v>0.04766</v>
       </c>
       <c r="T55" s="8" t="n">
         <v>0.00532</v>
       </c>
       <c r="U55" s="8" t="n">
-        <v>4.72255</v>
+        <v>4.72189</v>
       </c>
     </row>
     <row r="56">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>168.8</v>
+        <v>168.9</v>
       </c>
       <c r="E56" s="6">
         <f>D56*N56</f>
@@ -4924,28 +4924,28 @@
         <v/>
       </c>
       <c r="N56" s="8" t="n">
-        <v>4.127</v>
+        <v>4.126</v>
       </c>
       <c r="O56" s="8" t="n">
-        <v>0.22239</v>
+        <v>0.22262</v>
       </c>
       <c r="P56" s="8" t="n">
-        <v>0.04799</v>
+        <v>0.04802</v>
       </c>
       <c r="Q56" s="8" t="n">
-        <v>0.02637</v>
+        <v>0.02641</v>
       </c>
       <c r="R56" s="8" t="n">
-        <v>0.1637</v>
+        <v>0.16357</v>
       </c>
       <c r="S56" s="8" t="n">
-        <v>0.04367</v>
+        <v>0.04364</v>
       </c>
       <c r="T56" s="8" t="n">
         <v>0.00373</v>
       </c>
       <c r="U56" s="8" t="n">
-        <v>3.86109</v>
+        <v>3.85976</v>
       </c>
     </row>
     <row r="57">
@@ -4965,7 +4965,7 @@
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>167.6</v>
+        <v>167.8</v>
       </c>
       <c r="E57" s="6">
         <f>D57*N57</f>
@@ -5004,28 +5004,28 @@
         <v/>
       </c>
       <c r="N57" s="8" t="n">
-        <v>4.065</v>
+        <v>4.064</v>
       </c>
       <c r="O57" s="8" t="n">
-        <v>0.23073</v>
+        <v>0.23096</v>
       </c>
       <c r="P57" s="8" t="n">
-        <v>0.06836</v>
+        <v>0.0684</v>
       </c>
       <c r="Q57" s="8" t="n">
-        <v>0.01729</v>
+        <v>0.01731</v>
       </c>
       <c r="R57" s="8" t="n">
-        <v>0.15074</v>
+        <v>0.15062</v>
       </c>
       <c r="S57" s="8" t="n">
-        <v>0.03599</v>
+        <v>0.03596</v>
       </c>
       <c r="T57" s="8" t="n">
         <v>0.00235</v>
       </c>
       <c r="U57" s="8" t="n">
-        <v>3.12335</v>
+        <v>3.12183</v>
       </c>
     </row>
     <row r="58">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>167.2</v>
+        <v>167.3</v>
       </c>
       <c r="E58" s="6">
         <f>D58*N58</f>
@@ -5087,36 +5087,36 @@
         <v>4.103</v>
       </c>
       <c r="O58" s="8" t="n">
-        <v>0.2743</v>
+        <v>0.27456</v>
       </c>
       <c r="P58" s="8" t="n">
-        <v>0.07728</v>
+        <v>0.07732</v>
       </c>
       <c r="Q58" s="8" t="n">
-        <v>0.02341</v>
+        <v>0.02344</v>
       </c>
       <c r="R58" s="8" t="n">
-        <v>0.14298</v>
+        <v>0.14286</v>
       </c>
       <c r="S58" s="8" t="n">
-        <v>0.03529</v>
+        <v>0.03526</v>
       </c>
       <c r="T58" s="8" t="n">
         <v>0.00258</v>
       </c>
       <c r="U58" s="8" t="n">
-        <v>3.36023</v>
+        <v>3.35839</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Braxton Ashcraft</t>
+          <t>Freddy Peralta</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="D59" s="5" t="n">
-        <v>166.2</v>
+        <v>166.5</v>
       </c>
       <c r="E59" s="6">
         <f>D59*N59</f>
@@ -5164,28 +5164,28 @@
         <v/>
       </c>
       <c r="N59" s="8" t="n">
-        <v>4.083</v>
+        <v>4.173</v>
       </c>
       <c r="O59" s="8" t="n">
-        <v>0.24452</v>
+        <v>0.25592</v>
       </c>
       <c r="P59" s="8" t="n">
-        <v>0.06537999999999999</v>
+        <v>0.08917</v>
       </c>
       <c r="Q59" s="8" t="n">
-        <v>0.02293</v>
+        <v>0.02861</v>
       </c>
       <c r="R59" s="8" t="n">
-        <v>0.15093</v>
+        <v>0.13056</v>
       </c>
       <c r="S59" s="8" t="n">
-        <v>0.03467</v>
+        <v>0.03836</v>
       </c>
       <c r="T59" s="8" t="n">
-        <v>0.00296</v>
+        <v>0.00359</v>
       </c>
       <c r="U59" s="8" t="n">
-        <v>3.36338</v>
+        <v>3.77381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild 2027 projections (run 36906744278)
Verification PASSED.

Regenerated by .github/workflows/refresh-projections.yml.
Verification and the full baseline audit are in the run summary:
https://github.com/pmammino/DFSSimsFull/actions/runs/36906744278
</commit_message>
<xml_diff>
--- a/out/mlb_2027_what_if.xlsx
+++ b/out/mlb_2027_what_if.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="What-If" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What-If" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -713,37 +713,37 @@
         <v/>
       </c>
       <c r="P6" s="8" t="n">
-        <v>0.11537</v>
+        <v>0.11544</v>
       </c>
       <c r="Q6" s="8" t="n">
-        <v>0.04621</v>
+        <v>0.04624</v>
       </c>
       <c r="R6" s="8" t="n">
         <v>0.00263</v>
       </c>
       <c r="S6" s="8" t="n">
-        <v>0.05012</v>
+        <v>0.05014</v>
       </c>
       <c r="T6" s="8" t="n">
-        <v>0.11085</v>
+        <v>0.11081</v>
       </c>
       <c r="U6" s="8" t="n">
-        <v>0.008449999999999999</v>
+        <v>0.00844</v>
       </c>
       <c r="V6" s="8" t="n">
         <v>0.00606</v>
       </c>
       <c r="W6" s="8" t="n">
-        <v>0.24022</v>
+        <v>0.23989</v>
       </c>
       <c r="X6" s="8" t="n">
         <v>0.00351</v>
       </c>
       <c r="Y6" s="8" t="n">
-        <v>0.1308769253759874</v>
+        <v>0.1309504323723552</v>
       </c>
       <c r="Z6" s="8" t="n">
-        <v>0.1393581367257989</v>
+        <v>0.1394319334900104</v>
       </c>
     </row>
     <row r="7">
@@ -810,37 +810,37 @@
         <v/>
       </c>
       <c r="P7" s="8" t="n">
-        <v>0.1126</v>
+        <v>0.11268</v>
       </c>
       <c r="Q7" s="8" t="n">
-        <v>0.05129</v>
+        <v>0.05133</v>
       </c>
       <c r="R7" s="8" t="n">
         <v>0.0034</v>
       </c>
       <c r="S7" s="8" t="n">
-        <v>0.04689</v>
+        <v>0.04691</v>
       </c>
       <c r="T7" s="8" t="n">
-        <v>0.07511</v>
+        <v>0.07509</v>
       </c>
       <c r="U7" s="8" t="n">
-        <v>0.02598</v>
+        <v>0.02595</v>
       </c>
       <c r="V7" s="8" t="n">
         <v>0.00368</v>
       </c>
       <c r="W7" s="8" t="n">
-        <v>0.27348</v>
+        <v>0.27311</v>
       </c>
       <c r="X7" s="8" t="n">
         <v>0.03728</v>
       </c>
       <c r="Y7" s="8" t="n">
-        <v>0.1305117444263506</v>
+        <v>0.1305842564423994</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>0.1111451232387927</v>
+        <v>0.1112072377444949</v>
       </c>
     </row>
     <row r="8">
@@ -907,37 +907,37 @@
         <v/>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0.11974</v>
+        <v>0.11984</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>0.04585</v>
+        <v>0.04589</v>
       </c>
       <c r="R8" s="8" t="n">
         <v>0.00315</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>0.04506</v>
+        <v>0.04509</v>
       </c>
       <c r="T8" s="8" t="n">
-        <v>0.13211</v>
+        <v>0.13208</v>
       </c>
       <c r="U8" s="8" t="n">
-        <v>0.00555</v>
+        <v>0.00554</v>
       </c>
       <c r="V8" s="8" t="n">
         <v>0.00426</v>
       </c>
       <c r="W8" s="8" t="n">
-        <v>0.30163</v>
+        <v>0.30125</v>
       </c>
       <c r="X8" s="8" t="n">
         <v>0.02916</v>
       </c>
       <c r="Y8" s="8" t="n">
-        <v>0.1313272675270353</v>
+        <v>0.1313971805106357</v>
       </c>
       <c r="Z8" s="8" t="n">
-        <v>0.1188429364665634</v>
+        <v>0.1189029015166095</v>
       </c>
     </row>
     <row r="9">
@@ -1004,37 +1004,37 @@
         <v/>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0.17317</v>
+        <v>0.17324</v>
       </c>
       <c r="Q9" s="8" t="n">
-        <v>0.04147</v>
+        <v>0.04149</v>
       </c>
       <c r="R9" s="8" t="n">
         <v>0.00515</v>
       </c>
       <c r="S9" s="8" t="n">
-        <v>0.02081</v>
+        <v>0.02082</v>
       </c>
       <c r="T9" s="8" t="n">
-        <v>0.06368</v>
+        <v>0.06364</v>
       </c>
       <c r="U9" s="8" t="n">
-        <v>0.00747</v>
+        <v>0.00746</v>
       </c>
       <c r="V9" s="8" t="n">
         <v>0.008970000000000001</v>
       </c>
       <c r="W9" s="8" t="n">
-        <v>0.1508</v>
+        <v>0.15055</v>
       </c>
       <c r="X9" s="8" t="n">
         <v>0.03639</v>
       </c>
       <c r="Y9" s="8" t="n">
-        <v>0.1158223561605789</v>
+        <v>0.1158800774371023</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>0.1036565416286947</v>
+        <v>0.1037046854426036</v>
       </c>
     </row>
     <row r="10">
@@ -1101,37 +1101,37 @@
         <v/>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0.11332</v>
+        <v>0.11341</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>0.04214</v>
+        <v>0.04217</v>
       </c>
       <c r="R10" s="8" t="n">
         <v>0.00305</v>
       </c>
       <c r="S10" s="8" t="n">
-        <v>0.04043</v>
+        <v>0.04045</v>
       </c>
       <c r="T10" s="8" t="n">
-        <v>0.09598</v>
+        <v>0.09594</v>
       </c>
       <c r="U10" s="8" t="n">
-        <v>0.00479</v>
+        <v>0.00478</v>
       </c>
       <c r="V10" s="8" t="n">
         <v>0.00715</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>0.26658</v>
+        <v>0.26622</v>
       </c>
       <c r="X10" s="8" t="n">
         <v>0.01709</v>
       </c>
       <c r="Y10" s="8" t="n">
-        <v>0.122346404657863</v>
+        <v>0.1224196202016904</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>0.124348365011365</v>
+        <v>0.1244117867432792</v>
       </c>
     </row>
     <row r="11">
@@ -1198,37 +1198,37 @@
         <v/>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0.14392</v>
+        <v>0.144</v>
       </c>
       <c r="Q11" s="8" t="n">
-        <v>0.04788</v>
+        <v>0.04791</v>
       </c>
       <c r="R11" s="8" t="n">
-        <v>0.01377</v>
+        <v>0.01378</v>
       </c>
       <c r="S11" s="8" t="n">
-        <v>0.03031</v>
+        <v>0.03032</v>
       </c>
       <c r="T11" s="8" t="n">
-        <v>0.06191</v>
+        <v>0.06187</v>
       </c>
       <c r="U11" s="8" t="n">
-        <v>0.009730000000000001</v>
+        <v>0.00971</v>
       </c>
       <c r="V11" s="8" t="n">
-        <v>0.0095</v>
+        <v>0.00949</v>
       </c>
       <c r="W11" s="8" t="n">
-        <v>0.19195</v>
+        <v>0.19166</v>
       </c>
       <c r="X11" s="8" t="n">
         <v>0.02656</v>
       </c>
       <c r="Y11" s="8" t="n">
-        <v>0.1160796062713601</v>
+        <v>0.1161494229705326</v>
       </c>
       <c r="Z11" s="8" t="n">
-        <v>0.1136814304233801</v>
+        <v>0.1137314937813253</v>
       </c>
     </row>
     <row r="12">
@@ -1295,37 +1295,37 @@
         <v/>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0.13311</v>
+        <v>0.13319</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>0.04477</v>
+        <v>0.04479</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>0.00755</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>0.03719</v>
+        <v>0.0372</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>0.06408999999999999</v>
+        <v>0.06406000000000001</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>0.02178</v>
+        <v>0.02176</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>0.00628</v>
       </c>
       <c r="W12" s="8" t="n">
-        <v>0.21601</v>
+        <v>0.2157</v>
       </c>
       <c r="X12" s="8" t="n">
         <v>0.04791</v>
       </c>
       <c r="Y12" s="8" t="n">
-        <v>0.1301824593033082</v>
+        <v>0.1302523650577865</v>
       </c>
       <c r="Z12" s="8" t="n">
-        <v>0.110809540827651</v>
+        <v>0.1108793242479339</v>
       </c>
     </row>
     <row r="13">
@@ -1392,37 +1392,37 @@
         <v/>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0.12874</v>
+        <v>0.12882</v>
       </c>
       <c r="Q13" s="8" t="n">
-        <v>0.04532</v>
+        <v>0.04535</v>
       </c>
       <c r="R13" s="8" t="n">
         <v>0.00096</v>
       </c>
       <c r="S13" s="8" t="n">
-        <v>0.0581</v>
+        <v>0.05813</v>
       </c>
       <c r="T13" s="8" t="n">
-        <v>0.0977</v>
+        <v>0.09767000000000001</v>
       </c>
       <c r="U13" s="8" t="n">
-        <v>0.0203</v>
+        <v>0.02029</v>
       </c>
       <c r="V13" s="8" t="n">
         <v>0.00874</v>
       </c>
       <c r="W13" s="8" t="n">
-        <v>0.23516</v>
+        <v>0.23484</v>
       </c>
       <c r="X13" s="8" t="n">
         <v>0.00442</v>
       </c>
       <c r="Y13" s="8" t="n">
-        <v>0.1231540847191711</v>
+        <v>0.1232192330356798</v>
       </c>
       <c r="Z13" s="8" t="n">
-        <v>0.1485171745283121</v>
+        <v>0.148603283285401</v>
       </c>
     </row>
     <row r="14">
@@ -1489,10 +1489,10 @@
         <v/>
       </c>
       <c r="P14" s="8" t="n">
-        <v>0.14558</v>
+        <v>0.14566</v>
       </c>
       <c r="Q14" s="8" t="n">
-        <v>0.04702</v>
+        <v>0.04705</v>
       </c>
       <c r="R14" s="8" t="n">
         <v>0.00604</v>
@@ -1501,25 +1501,25 @@
         <v>0.02935</v>
       </c>
       <c r="T14" s="8" t="n">
-        <v>0.09539</v>
+        <v>0.09536</v>
       </c>
       <c r="U14" s="8" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.00929</v>
       </c>
       <c r="V14" s="8" t="n">
-        <v>0.0049</v>
+        <v>0.00489</v>
       </c>
       <c r="W14" s="8" t="n">
-        <v>0.23093</v>
+        <v>0.23061</v>
       </c>
       <c r="X14" s="8" t="n">
         <v>0.02686</v>
       </c>
       <c r="Y14" s="8" t="n">
-        <v>0.1291247731761868</v>
+        <v>0.1292099478496693</v>
       </c>
       <c r="Z14" s="8" t="n">
-        <v>0.1021530516009408</v>
+        <v>0.1022073189681618</v>
       </c>
     </row>
     <row r="15">
@@ -1586,10 +1586,10 @@
         <v/>
       </c>
       <c r="P15" s="8" t="n">
-        <v>0.1589</v>
+        <v>0.15897</v>
       </c>
       <c r="Q15" s="8" t="n">
-        <v>0.04706</v>
+        <v>0.04708</v>
       </c>
       <c r="R15" s="8" t="n">
         <v>0.00192</v>
@@ -1598,25 +1598,25 @@
         <v>0.03972</v>
       </c>
       <c r="T15" s="8" t="n">
-        <v>0.07133</v>
+        <v>0.07129000000000001</v>
       </c>
       <c r="U15" s="8" t="n">
         <v>0.00715</v>
       </c>
       <c r="V15" s="8" t="n">
-        <v>0.00707</v>
+        <v>0.00706</v>
       </c>
       <c r="W15" s="8" t="n">
-        <v>0.16073</v>
+        <v>0.16048</v>
       </c>
       <c r="X15" s="8" t="n">
         <v>0.008869999999999999</v>
       </c>
       <c r="Y15" s="8" t="n">
-        <v>0.1078631898841976</v>
+        <v>0.1079168715572707</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>0.1280366127382883</v>
+        <v>0.1281085555872521</v>
       </c>
     </row>
     <row r="16">
@@ -1683,37 +1683,37 @@
         <v/>
       </c>
       <c r="P16" s="8" t="n">
-        <v>0.11156</v>
+        <v>0.11165</v>
       </c>
       <c r="Q16" s="8" t="n">
-        <v>0.03634</v>
+        <v>0.03637</v>
       </c>
       <c r="R16" s="8" t="n">
-        <v>0.00316</v>
+        <v>0.00315</v>
       </c>
       <c r="S16" s="8" t="n">
-        <v>0.04592</v>
+        <v>0.04595</v>
       </c>
       <c r="T16" s="8" t="n">
-        <v>0.14033</v>
+        <v>0.14029</v>
       </c>
       <c r="U16" s="8" t="n">
         <v>0.01368</v>
       </c>
       <c r="V16" s="8" t="n">
-        <v>0.00501</v>
+        <v>0.005</v>
       </c>
       <c r="W16" s="8" t="n">
-        <v>0.28351</v>
+        <v>0.28316</v>
       </c>
       <c r="X16" s="8" t="n">
         <v>0.0123</v>
       </c>
       <c r="Y16" s="8" t="n">
-        <v>0.1349953652812758</v>
+        <v>0.1350774781694497</v>
       </c>
       <c r="Z16" s="8" t="n">
-        <v>0.1084118929890262</v>
+        <v>0.1084738611938727</v>
       </c>
     </row>
     <row r="17">
@@ -1780,37 +1780,37 @@
         <v/>
       </c>
       <c r="P17" s="8" t="n">
-        <v>0.1378</v>
+        <v>0.13788</v>
       </c>
       <c r="Q17" s="8" t="n">
-        <v>0.04265</v>
+        <v>0.04268</v>
       </c>
       <c r="R17" s="8" t="n">
         <v>0.0013</v>
       </c>
       <c r="S17" s="8" t="n">
-        <v>0.05433</v>
+        <v>0.05434</v>
       </c>
       <c r="T17" s="8" t="n">
-        <v>0.08529</v>
+        <v>0.08524</v>
       </c>
       <c r="U17" s="8" t="n">
-        <v>0.00524</v>
+        <v>0.00523</v>
       </c>
       <c r="V17" s="8" t="n">
         <v>0.00626</v>
       </c>
       <c r="W17" s="8" t="n">
-        <v>0.19729</v>
+        <v>0.197</v>
       </c>
       <c r="X17" s="8" t="n">
         <v>0.009010000000000001</v>
       </c>
       <c r="Y17" s="8" t="n">
-        <v>0.1253298922297539</v>
+        <v>0.1253889592414693</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>0.1358544390603159</v>
+        <v>0.1359224420856638</v>
       </c>
     </row>
     <row r="18">
@@ -1877,37 +1877,37 @@
         <v/>
       </c>
       <c r="P18" s="8" t="n">
-        <v>0.13669</v>
+        <v>0.13678</v>
       </c>
       <c r="Q18" s="8" t="n">
-        <v>0.04439</v>
+        <v>0.04442</v>
       </c>
       <c r="R18" s="8" t="n">
         <v>0.00356</v>
       </c>
       <c r="S18" s="8" t="n">
-        <v>0.03161</v>
+        <v>0.03162</v>
       </c>
       <c r="T18" s="8" t="n">
-        <v>0.0728</v>
+        <v>0.07277</v>
       </c>
       <c r="U18" s="8" t="n">
-        <v>0.00861</v>
+        <v>0.0086</v>
       </c>
       <c r="V18" s="8" t="n">
-        <v>0.00523</v>
+        <v>0.00522</v>
       </c>
       <c r="W18" s="8" t="n">
-        <v>0.271</v>
+        <v>0.27063</v>
       </c>
       <c r="X18" s="8" t="n">
         <v>0.02463</v>
       </c>
       <c r="Y18" s="8" t="n">
-        <v>0.1126208959240667</v>
+        <v>0.1126744668667468</v>
       </c>
       <c r="Z18" s="8" t="n">
-        <v>0.1168915926842642</v>
+        <v>0.1169544295762559</v>
       </c>
     </row>
     <row r="19">
@@ -1974,37 +1974,37 @@
         <v/>
       </c>
       <c r="P19" s="8" t="n">
-        <v>0.1381</v>
+        <v>0.13819</v>
       </c>
       <c r="Q19" s="8" t="n">
-        <v>0.04941</v>
+        <v>0.04945</v>
       </c>
       <c r="R19" s="8" t="n">
         <v>0.00573</v>
       </c>
       <c r="S19" s="8" t="n">
-        <v>0.03478</v>
+        <v>0.03479</v>
       </c>
       <c r="T19" s="8" t="n">
-        <v>0.0946</v>
+        <v>0.09456000000000001</v>
       </c>
       <c r="U19" s="8" t="n">
-        <v>0.0143</v>
+        <v>0.01429</v>
       </c>
       <c r="V19" s="8" t="n">
-        <v>0.00508</v>
+        <v>0.00507</v>
       </c>
       <c r="W19" s="8" t="n">
-        <v>0.23985</v>
+        <v>0.23952</v>
       </c>
       <c r="X19" s="8" t="n">
         <v>0.01286</v>
       </c>
       <c r="Y19" s="8" t="n">
-        <v>0.1228742913512657</v>
+        <v>0.1229411148850543</v>
       </c>
       <c r="Z19" s="8" t="n">
-        <v>0.1156687001917779</v>
+        <v>0.1157447515711056</v>
       </c>
     </row>
     <row r="20">
@@ -2071,37 +2071,37 @@
         <v/>
       </c>
       <c r="P20" s="8" t="n">
-        <v>0.18561</v>
+        <v>0.18568</v>
       </c>
       <c r="Q20" s="8" t="n">
-        <v>0.0312</v>
+        <v>0.03121</v>
       </c>
       <c r="R20" s="8" t="n">
-        <v>0.00534</v>
+        <v>0.00535</v>
       </c>
       <c r="S20" s="8" t="n">
         <v>0.00733</v>
       </c>
       <c r="T20" s="8" t="n">
-        <v>0.09424</v>
+        <v>0.09419</v>
       </c>
       <c r="U20" s="8" t="n">
-        <v>0.00283</v>
+        <v>0.00282</v>
       </c>
       <c r="V20" s="8" t="n">
         <v>0.007889999999999999</v>
       </c>
       <c r="W20" s="8" t="n">
-        <v>0.15633</v>
+        <v>0.15608</v>
       </c>
       <c r="X20" s="8" t="n">
         <v>0.04288</v>
       </c>
       <c r="Y20" s="8" t="n">
-        <v>0.10953034895737</v>
+        <v>0.1095880325500155</v>
       </c>
       <c r="Z20" s="8" t="n">
-        <v>0.078716621838332</v>
+        <v>0.078755111683385</v>
       </c>
     </row>
     <row r="21">
@@ -2168,37 +2168,37 @@
         <v/>
       </c>
       <c r="P21" s="8" t="n">
-        <v>0.18448</v>
+        <v>0.18455</v>
       </c>
       <c r="Q21" s="8" t="n">
-        <v>0.04554</v>
+        <v>0.04557</v>
       </c>
       <c r="R21" s="8" t="n">
         <v>0.00671</v>
       </c>
       <c r="S21" s="8" t="n">
-        <v>0.01457</v>
+        <v>0.01458</v>
       </c>
       <c r="T21" s="8" t="n">
-        <v>0.06319</v>
+        <v>0.06315</v>
       </c>
       <c r="U21" s="8" t="n">
-        <v>0.01009</v>
+        <v>0.01008</v>
       </c>
       <c r="V21" s="8" t="n">
-        <v>0.00721</v>
+        <v>0.0072</v>
       </c>
       <c r="W21" s="8" t="n">
-        <v>0.1175</v>
+        <v>0.1173</v>
       </c>
       <c r="X21" s="8" t="n">
         <v>0.01942</v>
       </c>
       <c r="Y21" s="8" t="n">
-        <v>0.1132438952673094</v>
+        <v>0.113306937605512</v>
       </c>
       <c r="Z21" s="8" t="n">
-        <v>0.09313553486932589</v>
+        <v>0.09319789018818769</v>
       </c>
     </row>
     <row r="22">
@@ -2265,37 +2265,37 @@
         <v/>
       </c>
       <c r="P22" s="8" t="n">
-        <v>0.14454</v>
+        <v>0.14463</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>0.03965</v>
+        <v>0.03967</v>
       </c>
       <c r="R22" s="8" t="n">
         <v>0.00765</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>0.0177</v>
+        <v>0.01771</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>0.11189</v>
+        <v>0.11184</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>0.01865</v>
+        <v>0.01864</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>0.00268</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>0.212</v>
+        <v>0.21169</v>
       </c>
       <c r="X22" s="8" t="n">
         <v>0.04402</v>
       </c>
       <c r="Y22" s="8" t="n">
-        <v>0.1189968733899924</v>
+        <v>0.1190641182787549</v>
       </c>
       <c r="Z22" s="8" t="n">
-        <v>0.0845048882835801</v>
+        <v>0.084552917395051</v>
       </c>
     </row>
     <row r="23">
@@ -2362,37 +2362,37 @@
         <v/>
       </c>
       <c r="P23" s="8" t="n">
-        <v>0.177</v>
+        <v>0.17709</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>0.03647</v>
+        <v>0.03649</v>
       </c>
       <c r="R23" s="8" t="n">
         <v>0.00173</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>0.02961</v>
+        <v>0.02962</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>0.09182999999999999</v>
+        <v>0.09177</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>0.0106</v>
+        <v>0.01059</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>0.00569</v>
+        <v>0.00568</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>0.14975</v>
+        <v>0.14952</v>
       </c>
       <c r="X23" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="Y23" s="8" t="n">
-        <v>0.1165803377152537</v>
+        <v>0.1166303489644284</v>
       </c>
       <c r="Z23" s="8" t="n">
-        <v>0.1116122885697547</v>
+        <v>0.1116529889391497</v>
       </c>
     </row>
     <row r="24">
@@ -2459,37 +2459,37 @@
         <v/>
       </c>
       <c r="P24" s="8" t="n">
-        <v>0.11644</v>
+        <v>0.11652</v>
       </c>
       <c r="Q24" s="8" t="n">
-        <v>0.04929</v>
+        <v>0.04933</v>
       </c>
       <c r="R24" s="8" t="n">
         <v>0.00157</v>
       </c>
       <c r="S24" s="8" t="n">
-        <v>0.04716</v>
+        <v>0.04717</v>
       </c>
       <c r="T24" s="8" t="n">
-        <v>0.10926</v>
+        <v>0.10922</v>
       </c>
       <c r="U24" s="8" t="n">
-        <v>0.00669</v>
+        <v>0.00668</v>
       </c>
       <c r="V24" s="8" t="n">
-        <v>0.00666</v>
+        <v>0.00665</v>
       </c>
       <c r="W24" s="8" t="n">
-        <v>0.24737</v>
+        <v>0.24703</v>
       </c>
       <c r="X24" s="8" t="n">
         <v>0.00144</v>
       </c>
       <c r="Y24" s="8" t="n">
-        <v>0.1267743240113502</v>
+        <v>0.1268448235725187</v>
       </c>
       <c r="Z24" s="8" t="n">
-        <v>0.133237489435214</v>
+        <v>0.133318170511943</v>
       </c>
     </row>
     <row r="25">
@@ -2556,37 +2556,37 @@
         <v/>
       </c>
       <c r="P25" s="8" t="n">
-        <v>0.11348</v>
+        <v>0.11356</v>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>0.04867</v>
+        <v>0.04871</v>
       </c>
       <c r="R25" s="8" t="n">
         <v>0.00231</v>
       </c>
       <c r="S25" s="8" t="n">
-        <v>0.04956</v>
+        <v>0.04958</v>
       </c>
       <c r="T25" s="8" t="n">
-        <v>0.09097</v>
+        <v>0.09095</v>
       </c>
       <c r="U25" s="8" t="n">
         <v>0.0107</v>
       </c>
       <c r="V25" s="8" t="n">
-        <v>0.00568</v>
+        <v>0.00567</v>
       </c>
       <c r="W25" s="8" t="n">
-        <v>0.27779</v>
+        <v>0.27742</v>
       </c>
       <c r="X25" s="8" t="n">
         <v>0.01097</v>
       </c>
       <c r="Y25" s="8" t="n">
-        <v>0.1273954023846647</v>
+        <v>0.1274595313651934</v>
       </c>
       <c r="Z25" s="8" t="n">
-        <v>0.1468158609563221</v>
+        <v>0.1469006423682971</v>
       </c>
     </row>
     <row r="26">
@@ -2653,53 +2653,53 @@
         <v/>
       </c>
       <c r="P26" s="8" t="n">
-        <v>0.14129</v>
+        <v>0.14138</v>
       </c>
       <c r="Q26" s="8" t="n">
-        <v>0.04339</v>
+        <v>0.04341</v>
       </c>
       <c r="R26" s="8" t="n">
-        <v>0.009140000000000001</v>
+        <v>0.00915</v>
       </c>
       <c r="S26" s="8" t="n">
-        <v>0.02751</v>
+        <v>0.02753</v>
       </c>
       <c r="T26" s="8" t="n">
-        <v>0.07277</v>
+        <v>0.07275</v>
       </c>
       <c r="U26" s="8" t="n">
         <v>0.01141</v>
       </c>
       <c r="V26" s="8" t="n">
-        <v>0.00598</v>
+        <v>0.00597</v>
       </c>
       <c r="W26" s="8" t="n">
-        <v>0.25176</v>
+        <v>0.2514</v>
       </c>
       <c r="X26" s="8" t="n">
         <v>0.0397</v>
       </c>
       <c r="Y26" s="8" t="n">
-        <v>0.115240504423424</v>
+        <v>0.1152966838962423</v>
       </c>
       <c r="Z26" s="8" t="n">
-        <v>0.1025390009408491</v>
+        <v>0.1025944232805242</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Everyday DH / 1B-DH</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
@@ -2750,53 +2750,53 @@
         <v/>
       </c>
       <c r="P27" s="8" t="n">
-        <v>0.14576</v>
+        <v>0.13896</v>
       </c>
       <c r="Q27" s="8" t="n">
-        <v>0.04292</v>
+        <v>0.04324</v>
       </c>
       <c r="R27" s="8" t="n">
-        <v>0.00178</v>
+        <v>0.007889999999999999</v>
       </c>
       <c r="S27" s="8" t="n">
-        <v>0.03655</v>
+        <v>0.02951</v>
       </c>
       <c r="T27" s="8" t="n">
-        <v>0.09699000000000001</v>
+        <v>0.12461</v>
       </c>
       <c r="U27" s="8" t="n">
-        <v>0.01604</v>
+        <v>0.0048</v>
       </c>
       <c r="V27" s="8" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.00566</v>
       </c>
       <c r="W27" s="8" t="n">
-        <v>0.25213</v>
+        <v>0.15674</v>
       </c>
       <c r="X27" s="8" t="n">
-        <v>0.00285</v>
+        <v>0.01801</v>
       </c>
       <c r="Y27" s="8" t="n">
-        <v>0.1130207063857602</v>
+        <v>0.1298104529584322</v>
       </c>
       <c r="Z27" s="8" t="n">
-        <v>0.1200724421631578</v>
+        <v>0.1025692821317952</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Full Time</t>
+          <t>Everyday DH / 1B-DH</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
@@ -2847,37 +2847,37 @@
         <v/>
       </c>
       <c r="P28" s="8" t="n">
-        <v>0.1389</v>
+        <v>0.14586</v>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>0.04321</v>
+        <v>0.04295</v>
       </c>
       <c r="R28" s="8" t="n">
-        <v>0.007889999999999999</v>
+        <v>0.00178</v>
       </c>
       <c r="S28" s="8" t="n">
-        <v>0.0295</v>
+        <v>0.03656</v>
       </c>
       <c r="T28" s="8" t="n">
-        <v>0.12468</v>
+        <v>0.09694999999999999</v>
       </c>
       <c r="U28" s="8" t="n">
-        <v>0.00481</v>
+        <v>0.01603</v>
       </c>
       <c r="V28" s="8" t="n">
-        <v>0.00567</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="W28" s="8" t="n">
-        <v>0.15699</v>
+        <v>0.25179</v>
       </c>
       <c r="X28" s="8" t="n">
-        <v>0.01801</v>
+        <v>0.00285</v>
       </c>
       <c r="Y28" s="8" t="n">
-        <v>0.1297388697627141</v>
+        <v>0.1130709577835605</v>
       </c>
       <c r="Z28" s="8" t="n">
-        <v>0.1025079752512514</v>
+        <v>0.120122217819372</v>
       </c>
     </row>
     <row r="29">
@@ -2944,37 +2944,37 @@
         <v/>
       </c>
       <c r="P29" s="8" t="n">
-        <v>0.09565</v>
+        <v>0.09573</v>
       </c>
       <c r="Q29" s="8" t="n">
-        <v>0.03733</v>
+        <v>0.03736</v>
       </c>
       <c r="R29" s="8" t="n">
         <v>0.00154</v>
       </c>
       <c r="S29" s="8" t="n">
-        <v>0.06146</v>
+        <v>0.06149</v>
       </c>
       <c r="T29" s="8" t="n">
-        <v>0.14532</v>
+        <v>0.14529</v>
       </c>
       <c r="U29" s="8" t="n">
-        <v>0.00942</v>
+        <v>0.00941</v>
       </c>
       <c r="V29" s="8" t="n">
-        <v>0.0056</v>
+        <v>0.00559</v>
       </c>
       <c r="W29" s="8" t="n">
-        <v>0.29725</v>
+        <v>0.29689</v>
       </c>
       <c r="X29" s="8" t="n">
         <v>0.00756</v>
       </c>
       <c r="Y29" s="8" t="n">
-        <v>0.1374788509075141</v>
+        <v>0.1375454863523066</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>0.1403509003184</v>
+        <v>0.1404276848359008</v>
       </c>
     </row>
     <row r="30">
@@ -3041,37 +3041,37 @@
         <v/>
       </c>
       <c r="P30" s="8" t="n">
-        <v>0.11346</v>
+        <v>0.11354</v>
       </c>
       <c r="Q30" s="8" t="n">
-        <v>0.04915</v>
+        <v>0.04918</v>
       </c>
       <c r="R30" s="8" t="n">
         <v>0.0066</v>
       </c>
       <c r="S30" s="8" t="n">
-        <v>0.0645</v>
+        <v>0.06453</v>
       </c>
       <c r="T30" s="8" t="n">
-        <v>0.12629</v>
+        <v>0.12625</v>
       </c>
       <c r="U30" s="8" t="n">
         <v>0.00705</v>
       </c>
       <c r="V30" s="8" t="n">
-        <v>0.00531</v>
+        <v>0.0053</v>
       </c>
       <c r="W30" s="8" t="n">
-        <v>0.24667</v>
+        <v>0.24633</v>
       </c>
       <c r="X30" s="8" t="n">
         <v>0.03207</v>
       </c>
       <c r="Y30" s="8" t="n">
-        <v>0.1657201067475644</v>
+        <v>0.1657950155444659</v>
       </c>
       <c r="Z30" s="8" t="n">
-        <v>0.147731752210238</v>
+        <v>0.1478070775708195</v>
       </c>
     </row>
     <row r="33">
@@ -3244,39 +3244,39 @@
         <v/>
       </c>
       <c r="N35" s="8" t="n">
-        <v>4.177</v>
+        <v>4.176</v>
       </c>
       <c r="O35" s="8" t="n">
-        <v>0.21648</v>
+        <v>0.217</v>
       </c>
       <c r="P35" s="8" t="n">
-        <v>0.05744</v>
+        <v>0.05752</v>
       </c>
       <c r="Q35" s="8" t="n">
-        <v>0.02102</v>
+        <v>0.02104</v>
       </c>
       <c r="R35" s="8" t="n">
-        <v>0.17117</v>
+        <v>0.17097</v>
       </c>
       <c r="S35" s="8" t="n">
-        <v>0.03998</v>
+        <v>0.03992</v>
       </c>
       <c r="T35" s="8" t="n">
         <v>0.00497</v>
       </c>
       <c r="U35" s="8" t="n">
-        <v>3.81154</v>
+        <v>3.80698</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Nolan McLean</t>
+          <t>Sandy Alcantara</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3324,39 +3324,39 @@
         <v/>
       </c>
       <c r="N36" s="8" t="n">
-        <v>4.21</v>
+        <v>4.223</v>
       </c>
       <c r="O36" s="8" t="n">
-        <v>0.25368</v>
+        <v>0.19018</v>
       </c>
       <c r="P36" s="8" t="n">
-        <v>0.09253</v>
+        <v>0.06875000000000001</v>
       </c>
       <c r="Q36" s="8" t="n">
-        <v>0.02147</v>
+        <v>0.02673</v>
       </c>
       <c r="R36" s="8" t="n">
-        <v>0.13546</v>
+        <v>0.15449</v>
       </c>
       <c r="S36" s="8" t="n">
-        <v>0.03736</v>
+        <v>0.04578</v>
       </c>
       <c r="T36" s="8" t="n">
-        <v>0.00316</v>
+        <v>0.0044</v>
       </c>
       <c r="U36" s="8" t="n">
-        <v>3.61031</v>
+        <v>4.17694</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Sandy Alcantara</t>
+          <t>Nolan McLean</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3404,28 +3404,28 @@
         <v/>
       </c>
       <c r="N37" s="8" t="n">
-        <v>4.224</v>
+        <v>4.209</v>
       </c>
       <c r="O37" s="8" t="n">
-        <v>0.18972</v>
+        <v>0.25423</v>
       </c>
       <c r="P37" s="8" t="n">
-        <v>0.06865</v>
+        <v>0.09264</v>
       </c>
       <c r="Q37" s="8" t="n">
-        <v>0.02671</v>
+        <v>0.02148</v>
       </c>
       <c r="R37" s="8" t="n">
-        <v>0.15467</v>
+        <v>0.13526</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>0.04585</v>
+        <v>0.03729</v>
       </c>
       <c r="T37" s="8" t="n">
-        <v>0.00441</v>
+        <v>0.00316</v>
       </c>
       <c r="U37" s="8" t="n">
-        <v>4.18123</v>
+        <v>3.60625</v>
       </c>
     </row>
     <row r="38">
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>212.1</v>
+        <v>212.7</v>
       </c>
       <c r="E38" s="6">
         <f>D38*N38</f>
@@ -3484,28 +3484,28 @@
         <v/>
       </c>
       <c r="N38" s="8" t="n">
-        <v>4.335</v>
+        <v>4.334</v>
       </c>
       <c r="O38" s="8" t="n">
-        <v>0.16211</v>
+        <v>0.16252</v>
       </c>
       <c r="P38" s="8" t="n">
-        <v>0.08626</v>
+        <v>0.08638999999999999</v>
       </c>
       <c r="Q38" s="8" t="n">
-        <v>0.02071</v>
+        <v>0.02073</v>
       </c>
       <c r="R38" s="8" t="n">
-        <v>0.17337</v>
+        <v>0.17318</v>
       </c>
       <c r="S38" s="8" t="n">
-        <v>0.03691</v>
+        <v>0.03686</v>
       </c>
       <c r="T38" s="8" t="n">
-        <v>0.00408</v>
+        <v>0.00407</v>
       </c>
       <c r="U38" s="8" t="n">
-        <v>4.21385</v>
+        <v>4.21019</v>
       </c>
     </row>
     <row r="39">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>211.2</v>
+        <v>211.8</v>
       </c>
       <c r="E39" s="6">
         <f>D39*N39</f>
@@ -3567,25 +3567,25 @@
         <v>4.274</v>
       </c>
       <c r="O39" s="8" t="n">
-        <v>0.16461</v>
+        <v>0.16504</v>
       </c>
       <c r="P39" s="8" t="n">
-        <v>0.06444999999999999</v>
+        <v>0.06455</v>
       </c>
       <c r="Q39" s="8" t="n">
-        <v>0.03342</v>
+        <v>0.03345</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>0.16413</v>
+        <v>0.16396</v>
       </c>
       <c r="S39" s="8" t="n">
-        <v>0.04733</v>
+        <v>0.04726</v>
       </c>
       <c r="T39" s="8" t="n">
-        <v>0.0044</v>
+        <v>0.00439</v>
       </c>
       <c r="U39" s="8" t="n">
-        <v>4.67491</v>
+        <v>4.67108</v>
       </c>
     </row>
     <row r="40">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>198.8</v>
+        <v>199</v>
       </c>
       <c r="E40" s="6">
         <f>D40*N40</f>
@@ -3647,25 +3647,25 @@
         <v>4.169</v>
       </c>
       <c r="O40" s="8" t="n">
-        <v>0.19438</v>
+        <v>0.19486</v>
       </c>
       <c r="P40" s="8" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.0687</v>
       </c>
       <c r="Q40" s="8" t="n">
-        <v>0.03149</v>
+        <v>0.03151</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>0.13926</v>
+        <v>0.1391</v>
       </c>
       <c r="S40" s="8" t="n">
-        <v>0.04866</v>
+        <v>0.04859</v>
       </c>
       <c r="T40" s="8" t="n">
-        <v>0.00603</v>
+        <v>0.00602</v>
       </c>
       <c r="U40" s="8" t="n">
-        <v>4.21356</v>
+        <v>4.20948</v>
       </c>
     </row>
     <row r="41">
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>196.2</v>
+        <v>196.5</v>
       </c>
       <c r="E41" s="6">
         <f>D41*N41</f>
@@ -3724,28 +3724,28 @@
         <v/>
       </c>
       <c r="N41" s="8" t="n">
-        <v>4.009</v>
+        <v>4.008</v>
       </c>
       <c r="O41" s="8" t="n">
-        <v>0.28284</v>
+        <v>0.28344</v>
       </c>
       <c r="P41" s="8" t="n">
-        <v>0.06644</v>
+        <v>0.06651</v>
       </c>
       <c r="Q41" s="8" t="n">
-        <v>0.02328</v>
+        <v>0.0233</v>
       </c>
       <c r="R41" s="8" t="n">
-        <v>0.12982</v>
+        <v>0.12962</v>
       </c>
       <c r="S41" s="8" t="n">
-        <v>0.03786</v>
+        <v>0.03779</v>
       </c>
       <c r="T41" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="U41" s="8" t="n">
-        <v>3.11144</v>
+        <v>3.10699</v>
       </c>
     </row>
     <row r="42">
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>195.7</v>
+        <v>195.8</v>
       </c>
       <c r="E42" s="6">
         <f>D42*N42</f>
@@ -3804,28 +3804,28 @@
         <v/>
       </c>
       <c r="N42" s="8" t="n">
-        <v>4.109</v>
+        <v>4.108</v>
       </c>
       <c r="O42" s="8" t="n">
-        <v>0.23924</v>
+        <v>0.2398</v>
       </c>
       <c r="P42" s="8" t="n">
-        <v>0.05788</v>
+        <v>0.05796</v>
       </c>
       <c r="Q42" s="8" t="n">
-        <v>0.02034</v>
+        <v>0.02036</v>
       </c>
       <c r="R42" s="8" t="n">
-        <v>0.16384</v>
+        <v>0.16363</v>
       </c>
       <c r="S42" s="8" t="n">
-        <v>0.03974</v>
+        <v>0.03968</v>
       </c>
       <c r="T42" s="8" t="n">
         <v>0.00258</v>
       </c>
       <c r="U42" s="8" t="n">
-        <v>3.47409</v>
+        <v>3.46961</v>
       </c>
     </row>
     <row r="43">
@@ -3845,7 +3845,7 @@
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>190.9</v>
+        <v>191.4</v>
       </c>
       <c r="E43" s="6">
         <f>D43*N43</f>
@@ -3884,28 +3884,28 @@
         <v/>
       </c>
       <c r="N43" s="8" t="n">
-        <v>4.133</v>
+        <v>4.132</v>
       </c>
       <c r="O43" s="8" t="n">
-        <v>0.2594</v>
+        <v>0.25996</v>
       </c>
       <c r="P43" s="8" t="n">
-        <v>0.09172</v>
+        <v>0.09182999999999999</v>
       </c>
       <c r="Q43" s="8" t="n">
-        <v>0.02049</v>
+        <v>0.0205</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>0.14158</v>
+        <v>0.14138</v>
       </c>
       <c r="S43" s="8" t="n">
-        <v>0.02824</v>
+        <v>0.02819</v>
       </c>
       <c r="T43" s="8" t="n">
         <v>0.00328</v>
       </c>
       <c r="U43" s="8" t="n">
-        <v>3.24033</v>
+        <v>3.23628</v>
       </c>
     </row>
     <row r="44">
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>189.7</v>
+        <v>190.1</v>
       </c>
       <c r="E44" s="6">
         <f>D44*N44</f>
@@ -3964,28 +3964,28 @@
         <v/>
       </c>
       <c r="N44" s="8" t="n">
-        <v>4.251</v>
+        <v>4.25</v>
       </c>
       <c r="O44" s="8" t="n">
-        <v>0.21665</v>
+        <v>0.21715</v>
       </c>
       <c r="P44" s="8" t="n">
-        <v>0.08314000000000001</v>
+        <v>0.08323999999999999</v>
       </c>
       <c r="Q44" s="8" t="n">
-        <v>0.0197</v>
+        <v>0.01972</v>
       </c>
       <c r="R44" s="8" t="n">
-        <v>0.15454</v>
+        <v>0.15434</v>
       </c>
       <c r="S44" s="8" t="n">
-        <v>0.04108</v>
+        <v>0.04101</v>
       </c>
       <c r="T44" s="8" t="n">
         <v>0.00366</v>
       </c>
       <c r="U44" s="8" t="n">
-        <v>3.85845</v>
+        <v>3.85389</v>
       </c>
     </row>
     <row r="45">
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>187.9</v>
+        <v>188.3</v>
       </c>
       <c r="E45" s="6">
         <f>D45*N45</f>
@@ -4044,28 +4044,28 @@
         <v/>
       </c>
       <c r="N45" s="8" t="n">
-        <v>4.34</v>
+        <v>4.339</v>
       </c>
       <c r="O45" s="8" t="n">
-        <v>0.1896</v>
+        <v>0.19004</v>
       </c>
       <c r="P45" s="8" t="n">
-        <v>0.08619</v>
+        <v>0.0863</v>
       </c>
       <c r="Q45" s="8" t="n">
-        <v>0.04325</v>
+        <v>0.04328</v>
       </c>
       <c r="R45" s="8" t="n">
-        <v>0.13977</v>
+        <v>0.13959</v>
       </c>
       <c r="S45" s="8" t="n">
-        <v>0.04412</v>
+        <v>0.04405</v>
       </c>
       <c r="T45" s="8" t="n">
         <v>0.00459</v>
       </c>
       <c r="U45" s="8" t="n">
-        <v>5.0443</v>
+        <v>5.04139</v>
       </c>
     </row>
     <row r="46">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>186.5</v>
+        <v>186.8</v>
       </c>
       <c r="E46" s="6">
         <f>D46*N46</f>
@@ -4124,28 +4124,28 @@
         <v/>
       </c>
       <c r="N46" s="8" t="n">
-        <v>4.05</v>
+        <v>4.049</v>
       </c>
       <c r="O46" s="8" t="n">
-        <v>0.29875</v>
+        <v>0.29938</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>0.0669</v>
+        <v>0.06698</v>
       </c>
       <c r="Q46" s="8" t="n">
-        <v>0.0294</v>
+        <v>0.02941</v>
       </c>
       <c r="R46" s="8" t="n">
-        <v>0.13364</v>
+        <v>0.13344</v>
       </c>
       <c r="S46" s="8" t="n">
-        <v>0.03966</v>
+        <v>0.03959</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0.00272</v>
       </c>
       <c r="U46" s="8" t="n">
-        <v>3.44264</v>
+        <v>3.43729</v>
       </c>
     </row>
     <row r="47">
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>185</v>
+        <v>185.4</v>
       </c>
       <c r="E47" s="6">
         <f>D47*N47</f>
@@ -4204,28 +4204,28 @@
         <v/>
       </c>
       <c r="N47" s="8" t="n">
-        <v>4.345</v>
+        <v>4.344</v>
       </c>
       <c r="O47" s="8" t="n">
-        <v>0.20476</v>
+        <v>0.20524</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>0.07475</v>
+        <v>0.07485</v>
       </c>
       <c r="Q47" s="8" t="n">
-        <v>0.02964</v>
+        <v>0.02966</v>
       </c>
       <c r="R47" s="8" t="n">
-        <v>0.15536</v>
+        <v>0.15516</v>
       </c>
       <c r="S47" s="8" t="n">
-        <v>0.04914</v>
+        <v>0.04907</v>
       </c>
       <c r="T47" s="8" t="n">
         <v>0.0043</v>
       </c>
       <c r="U47" s="8" t="n">
-        <v>4.67824</v>
+        <v>4.67393</v>
       </c>
     </row>
     <row r="48">
@@ -4245,7 +4245,7 @@
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>183.8</v>
+        <v>184.3</v>
       </c>
       <c r="E48" s="6">
         <f>D48*N48</f>
@@ -4284,48 +4284,48 @@
         <v/>
       </c>
       <c r="N48" s="8" t="n">
-        <v>4.285</v>
+        <v>4.284</v>
       </c>
       <c r="O48" s="8" t="n">
-        <v>0.24135</v>
+        <v>0.24189</v>
       </c>
       <c r="P48" s="8" t="n">
-        <v>0.08685</v>
+        <v>0.08696</v>
       </c>
       <c r="Q48" s="8" t="n">
-        <v>0.03498</v>
+        <v>0.03499</v>
       </c>
       <c r="R48" s="8" t="n">
-        <v>0.13608</v>
+        <v>0.13589</v>
       </c>
       <c r="S48" s="8" t="n">
-        <v>0.05158</v>
+        <v>0.05149</v>
       </c>
       <c r="T48" s="8" t="n">
         <v>0.00334</v>
       </c>
       <c r="U48" s="8" t="n">
-        <v>4.57764</v>
+        <v>4.57243</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Noah Cameron</t>
+          <t>Tarik Skubal</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
+          <t>Ace (SP1)</t>
         </is>
       </c>
       <c r="D49" s="5" t="n">
-        <v>181.7</v>
+        <v>182</v>
       </c>
       <c r="E49" s="6">
         <f>D49*N49</f>
@@ -4364,48 +4364,48 @@
         <v/>
       </c>
       <c r="N49" s="8" t="n">
-        <v>4.189</v>
+        <v>3.956</v>
       </c>
       <c r="O49" s="8" t="n">
-        <v>0.2054</v>
+        <v>0.29099</v>
       </c>
       <c r="P49" s="8" t="n">
-        <v>0.07975</v>
+        <v>0.05095</v>
       </c>
       <c r="Q49" s="8" t="n">
-        <v>0.03047</v>
+        <v>0.02316</v>
       </c>
       <c r="R49" s="8" t="n">
-        <v>0.14218</v>
+        <v>0.14109</v>
       </c>
       <c r="S49" s="8" t="n">
-        <v>0.04211</v>
+        <v>0.0371</v>
       </c>
       <c r="T49" s="8" t="n">
-        <v>0.00353</v>
+        <v>0.00319</v>
       </c>
       <c r="U49" s="8" t="n">
-        <v>4.05699</v>
+        <v>2.98544</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Tarik Skubal</t>
+          <t>Noah Cameron</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Ace (SP1)</t>
+          <t>Mid-Rotation Starter (SP2-3)</t>
         </is>
       </c>
       <c r="D50" s="5" t="n">
-        <v>181.6</v>
+        <v>182</v>
       </c>
       <c r="E50" s="6">
         <f>D50*N50</f>
@@ -4444,28 +4444,28 @@
         <v/>
       </c>
       <c r="N50" s="8" t="n">
-        <v>3.957</v>
+        <v>4.188</v>
       </c>
       <c r="O50" s="8" t="n">
-        <v>0.29037</v>
+        <v>0.20589</v>
       </c>
       <c r="P50" s="8" t="n">
-        <v>0.05088</v>
+        <v>0.07985</v>
       </c>
       <c r="Q50" s="8" t="n">
-        <v>0.02315</v>
+        <v>0.03049</v>
       </c>
       <c r="R50" s="8" t="n">
-        <v>0.1413</v>
+        <v>0.14201</v>
       </c>
       <c r="S50" s="8" t="n">
-        <v>0.03717</v>
+        <v>0.04204</v>
       </c>
       <c r="T50" s="8" t="n">
-        <v>0.00319</v>
+        <v>0.00353</v>
       </c>
       <c r="U50" s="8" t="n">
-        <v>2.99038</v>
+        <v>4.05278</v>
       </c>
     </row>
     <row r="51">
@@ -4485,7 +4485,7 @@
         </is>
       </c>
       <c r="D51" s="5" t="n">
-        <v>180.5</v>
+        <v>180.7</v>
       </c>
       <c r="E51" s="6">
         <f>D51*N51</f>
@@ -4524,39 +4524,39 @@
         <v/>
       </c>
       <c r="N51" s="8" t="n">
-        <v>4.034</v>
+        <v>4.033</v>
       </c>
       <c r="O51" s="8" t="n">
-        <v>0.26047</v>
+        <v>0.26106</v>
       </c>
       <c r="P51" s="8" t="n">
-        <v>0.05921</v>
+        <v>0.05928</v>
       </c>
       <c r="Q51" s="8" t="n">
-        <v>0.03685</v>
+        <v>0.03687</v>
       </c>
       <c r="R51" s="8" t="n">
-        <v>0.13085</v>
+        <v>0.13067</v>
       </c>
       <c r="S51" s="8" t="n">
-        <v>0.04077</v>
+        <v>0.0407</v>
       </c>
       <c r="T51" s="8" t="n">
         <v>0.00277</v>
       </c>
       <c r="U51" s="8" t="n">
-        <v>3.71513</v>
+        <v>3.71069</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Seth Lugo</t>
+          <t>Freddy Peralta</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>178.9</v>
+        <v>179.6</v>
       </c>
       <c r="E52" s="6">
         <f>D52*N52</f>
@@ -4604,39 +4604,39 @@
         <v/>
       </c>
       <c r="N52" s="8" t="n">
-        <v>4.285</v>
+        <v>4.175</v>
       </c>
       <c r="O52" s="8" t="n">
-        <v>0.20199</v>
+        <v>0.25531</v>
       </c>
       <c r="P52" s="8" t="n">
-        <v>0.0721</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="Q52" s="8" t="n">
-        <v>0.03645</v>
+        <v>0.02869</v>
       </c>
       <c r="R52" s="8" t="n">
-        <v>0.1485</v>
+        <v>0.13059</v>
       </c>
       <c r="S52" s="8" t="n">
-        <v>0.04779</v>
+        <v>0.03841</v>
       </c>
       <c r="T52" s="8" t="n">
-        <v>0.00532</v>
+        <v>0.00359</v>
       </c>
       <c r="U52" s="8" t="n">
-        <v>4.73875</v>
+        <v>3.78599</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Jeffrey Springs</t>
+          <t>Seth Lugo</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>OAK</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4645,7 +4645,7 @@
         </is>
       </c>
       <c r="D53" s="5" t="n">
-        <v>178.6</v>
+        <v>179.2</v>
       </c>
       <c r="E53" s="6">
         <f>D53*N53</f>
@@ -4684,39 +4684,39 @@
         <v/>
       </c>
       <c r="N53" s="8" t="n">
-        <v>4.234</v>
+        <v>4.284</v>
       </c>
       <c r="O53" s="8" t="n">
-        <v>0.20431</v>
+        <v>0.20247</v>
       </c>
       <c r="P53" s="8" t="n">
-        <v>0.07996</v>
+        <v>0.07219</v>
       </c>
       <c r="Q53" s="8" t="n">
-        <v>0.03975</v>
+        <v>0.03648</v>
       </c>
       <c r="R53" s="8" t="n">
-        <v>0.13812</v>
+        <v>0.14832</v>
       </c>
       <c r="S53" s="8" t="n">
-        <v>0.04587</v>
+        <v>0.04772</v>
       </c>
       <c r="T53" s="8" t="n">
-        <v>0.00309</v>
+        <v>0.00531</v>
       </c>
       <c r="U53" s="8" t="n">
-        <v>4.56302</v>
+        <v>4.73457</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Freddy Peralta</t>
+          <t>Jeffrey Springs</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>OAK</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>178.6</v>
+        <v>178.9</v>
       </c>
       <c r="E54" s="6">
         <f>D54*N54</f>
@@ -4764,28 +4764,28 @@
         <v/>
       </c>
       <c r="N54" s="8" t="n">
-        <v>4.176</v>
+        <v>4.233</v>
       </c>
       <c r="O54" s="8" t="n">
-        <v>0.25476</v>
+        <v>0.20479</v>
       </c>
       <c r="P54" s="8" t="n">
-        <v>0.08928999999999999</v>
+        <v>0.08008</v>
       </c>
       <c r="Q54" s="8" t="n">
-        <v>0.02868</v>
+        <v>0.03977</v>
       </c>
       <c r="R54" s="8" t="n">
-        <v>0.13078</v>
+        <v>0.13796</v>
       </c>
       <c r="S54" s="8" t="n">
-        <v>0.03848</v>
+        <v>0.04579</v>
       </c>
       <c r="T54" s="8" t="n">
-        <v>0.00359</v>
+        <v>0.00309</v>
       </c>
       <c r="U54" s="8" t="n">
-        <v>3.79045</v>
+        <v>4.55937</v>
       </c>
     </row>
     <row r="55">
@@ -4805,7 +4805,7 @@
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>177.7</v>
+        <v>178.3</v>
       </c>
       <c r="E55" s="6">
         <f>D55*N55</f>
@@ -4844,28 +4844,28 @@
         <v/>
       </c>
       <c r="N55" s="8" t="n">
-        <v>4.067</v>
+        <v>4.066</v>
       </c>
       <c r="O55" s="8" t="n">
-        <v>0.22988</v>
+        <v>0.23041</v>
       </c>
       <c r="P55" s="8" t="n">
-        <v>0.06849</v>
+        <v>0.06858</v>
       </c>
       <c r="Q55" s="8" t="n">
         <v>0.01736</v>
       </c>
       <c r="R55" s="8" t="n">
-        <v>0.15085</v>
+        <v>0.15066</v>
       </c>
       <c r="S55" s="8" t="n">
-        <v>0.03607</v>
+        <v>0.03601</v>
       </c>
       <c r="T55" s="8" t="n">
         <v>0.00235</v>
       </c>
       <c r="U55" s="8" t="n">
-        <v>3.13497</v>
+        <v>3.13062</v>
       </c>
     </row>
     <row r="56">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>175.6</v>
+        <v>175.8</v>
       </c>
       <c r="E56" s="6">
         <f>D56*N56</f>
@@ -4924,28 +4924,28 @@
         <v/>
       </c>
       <c r="N56" s="8" t="n">
-        <v>4.041</v>
+        <v>4.04</v>
       </c>
       <c r="O56" s="8" t="n">
-        <v>0.24063</v>
+        <v>0.24118</v>
       </c>
       <c r="P56" s="8" t="n">
-        <v>0.05535</v>
+        <v>0.05543</v>
       </c>
       <c r="Q56" s="8" t="n">
-        <v>0.02812</v>
+        <v>0.02813</v>
       </c>
       <c r="R56" s="8" t="n">
-        <v>0.14159</v>
+        <v>0.1414</v>
       </c>
       <c r="S56" s="8" t="n">
-        <v>0.04116</v>
+        <v>0.04109</v>
       </c>
       <c r="T56" s="8" t="n">
         <v>0.00299</v>
       </c>
       <c r="U56" s="8" t="n">
-        <v>3.50404</v>
+        <v>3.49972</v>
       </c>
     </row>
     <row r="57">
@@ -4965,7 +4965,7 @@
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>175.2</v>
+        <v>175.4</v>
       </c>
       <c r="E57" s="6">
         <f>D57*N57</f>
@@ -5004,28 +5004,28 @@
         <v/>
       </c>
       <c r="N57" s="8" t="n">
-        <v>4.086</v>
+        <v>4.085</v>
       </c>
       <c r="O57" s="8" t="n">
-        <v>0.24363</v>
+        <v>0.24419</v>
       </c>
       <c r="P57" s="8" t="n">
-        <v>0.0655</v>
+        <v>0.06559</v>
       </c>
       <c r="Q57" s="8" t="n">
-        <v>0.02302</v>
+        <v>0.02303</v>
       </c>
       <c r="R57" s="8" t="n">
-        <v>0.15105</v>
+        <v>0.15085</v>
       </c>
       <c r="S57" s="8" t="n">
-        <v>0.03475</v>
+        <v>0.03469</v>
       </c>
       <c r="T57" s="8" t="n">
         <v>0.00296</v>
       </c>
       <c r="U57" s="8" t="n">
-        <v>3.37626</v>
+        <v>3.37174</v>
       </c>
     </row>
     <row r="58">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>174.2</v>
+        <v>174.4</v>
       </c>
       <c r="E58" s="6">
         <f>D58*N58</f>
@@ -5084,28 +5084,28 @@
         <v/>
       </c>
       <c r="N58" s="8" t="n">
-        <v>4.129</v>
+        <v>4.128</v>
       </c>
       <c r="O58" s="8" t="n">
-        <v>0.22156</v>
+        <v>0.22209</v>
       </c>
       <c r="P58" s="8" t="n">
-        <v>0.04808</v>
+        <v>0.04815</v>
       </c>
       <c r="Q58" s="8" t="n">
-        <v>0.02647</v>
+        <v>0.02649</v>
       </c>
       <c r="R58" s="8" t="n">
-        <v>0.16381</v>
+        <v>0.16361</v>
       </c>
       <c r="S58" s="8" t="n">
-        <v>0.04377</v>
+        <v>0.0437</v>
       </c>
       <c r="T58" s="8" t="n">
         <v>0.00373</v>
       </c>
       <c r="U58" s="8" t="n">
-        <v>3.87448</v>
+        <v>3.86991</v>
       </c>
     </row>
     <row r="59">
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="D59" s="5" t="n">
-        <v>173.6</v>
+        <v>174</v>
       </c>
       <c r="E59" s="6">
         <f>D59*N59</f>
@@ -5167,25 +5167,25 @@
         <v>4.214</v>
       </c>
       <c r="O59" s="8" t="n">
-        <v>0.24946</v>
+        <v>0.25001</v>
       </c>
       <c r="P59" s="8" t="n">
-        <v>0.07217999999999999</v>
+        <v>0.07227</v>
       </c>
       <c r="Q59" s="8" t="n">
-        <v>0.02475</v>
+        <v>0.02476</v>
       </c>
       <c r="R59" s="8" t="n">
-        <v>0.15119</v>
+        <v>0.15097</v>
       </c>
       <c r="S59" s="8" t="n">
-        <v>0.033</v>
+        <v>0.03293</v>
       </c>
       <c r="T59" s="8" t="n">
         <v>0.00382</v>
       </c>
       <c r="U59" s="8" t="n">
-        <v>3.78859</v>
+        <v>3.78379</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild 2027 projections (run 36908379827)
Verification PASSED.

Regenerated by .github/workflows/refresh-projections.yml.
Verification and the full baseline audit are in the run summary:
https://github.com/pmammino/DFSSimsFull/actions/runs/36908379827
</commit_message>
<xml_diff>
--- a/out/mlb_2027_what_if.xlsx
+++ b/out/mlb_2027_what_if.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="What-If" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What-If" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -713,37 +713,37 @@
         <v/>
       </c>
       <c r="P6" s="8" t="n">
-        <v>0.11537</v>
+        <v>0.11544</v>
       </c>
       <c r="Q6" s="8" t="n">
-        <v>0.04621</v>
+        <v>0.04624</v>
       </c>
       <c r="R6" s="8" t="n">
         <v>0.00263</v>
       </c>
       <c r="S6" s="8" t="n">
-        <v>0.05012</v>
+        <v>0.05014</v>
       </c>
       <c r="T6" s="8" t="n">
-        <v>0.11085</v>
+        <v>0.11081</v>
       </c>
       <c r="U6" s="8" t="n">
-        <v>0.008449999999999999</v>
+        <v>0.00844</v>
       </c>
       <c r="V6" s="8" t="n">
         <v>0.00606</v>
       </c>
       <c r="W6" s="8" t="n">
-        <v>0.24022</v>
+        <v>0.23989</v>
       </c>
       <c r="X6" s="8" t="n">
         <v>0.00351</v>
       </c>
       <c r="Y6" s="8" t="n">
-        <v>0.1308769126670375</v>
+        <v>0.1309504323723552</v>
       </c>
       <c r="Z6" s="8" t="n">
-        <v>0.1393581231932715</v>
+        <v>0.1394319334900104</v>
       </c>
     </row>
     <row r="7">
@@ -810,37 +810,37 @@
         <v/>
       </c>
       <c r="P7" s="8" t="n">
-        <v>0.1126</v>
+        <v>0.11268</v>
       </c>
       <c r="Q7" s="8" t="n">
-        <v>0.05129</v>
+        <v>0.05133</v>
       </c>
       <c r="R7" s="8" t="n">
         <v>0.0034</v>
       </c>
       <c r="S7" s="8" t="n">
-        <v>0.04689</v>
+        <v>0.04691</v>
       </c>
       <c r="T7" s="8" t="n">
-        <v>0.07511</v>
+        <v>0.07509</v>
       </c>
       <c r="U7" s="8" t="n">
-        <v>0.02598</v>
+        <v>0.02595</v>
       </c>
       <c r="V7" s="8" t="n">
         <v>0.00368</v>
       </c>
       <c r="W7" s="8" t="n">
-        <v>0.27347</v>
+        <v>0.27311</v>
       </c>
       <c r="X7" s="8" t="n">
         <v>0.03728</v>
       </c>
       <c r="Y7" s="8" t="n">
-        <v>0.1305117658570737</v>
+        <v>0.1305842564423994</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>0.1111451414894136</v>
+        <v>0.1112072377444949</v>
       </c>
     </row>
     <row r="8">
@@ -907,37 +907,37 @@
         <v/>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0.11974</v>
+        <v>0.11984</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>0.04585</v>
+        <v>0.04589</v>
       </c>
       <c r="R8" s="8" t="n">
         <v>0.00315</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>0.04506</v>
+        <v>0.04509</v>
       </c>
       <c r="T8" s="8" t="n">
-        <v>0.13211</v>
+        <v>0.13208</v>
       </c>
       <c r="U8" s="8" t="n">
-        <v>0.00555</v>
+        <v>0.00554</v>
       </c>
       <c r="V8" s="8" t="n">
         <v>0.00426</v>
       </c>
       <c r="W8" s="8" t="n">
-        <v>0.30163</v>
+        <v>0.30125</v>
       </c>
       <c r="X8" s="8" t="n">
         <v>0.02916</v>
       </c>
       <c r="Y8" s="8" t="n">
-        <v>0.1313272711072163</v>
+        <v>0.1313971805106357</v>
       </c>
       <c r="Z8" s="8" t="n">
-        <v>0.1188429397064025</v>
+        <v>0.1189029015166095</v>
       </c>
     </row>
     <row r="9">
@@ -1004,37 +1004,37 @@
         <v/>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0.17317</v>
+        <v>0.17324</v>
       </c>
       <c r="Q9" s="8" t="n">
-        <v>0.04147</v>
+        <v>0.04149</v>
       </c>
       <c r="R9" s="8" t="n">
         <v>0.00515</v>
       </c>
       <c r="S9" s="8" t="n">
-        <v>0.02081</v>
+        <v>0.02082</v>
       </c>
       <c r="T9" s="8" t="n">
-        <v>0.06368</v>
+        <v>0.06364</v>
       </c>
       <c r="U9" s="8" t="n">
-        <v>0.00747</v>
+        <v>0.00746</v>
       </c>
       <c r="V9" s="8" t="n">
         <v>0.008970000000000001</v>
       </c>
       <c r="W9" s="8" t="n">
-        <v>0.1508</v>
+        <v>0.15055</v>
       </c>
       <c r="X9" s="8" t="n">
         <v>0.03639</v>
       </c>
       <c r="Y9" s="8" t="n">
-        <v>0.1158223452146403</v>
+        <v>0.1158800774371023</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>0.1036565318325018</v>
+        <v>0.1037046854426036</v>
       </c>
     </row>
     <row r="10">
@@ -1101,37 +1101,37 @@
         <v/>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0.11332</v>
+        <v>0.11341</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>0.04214</v>
+        <v>0.04217</v>
       </c>
       <c r="R10" s="8" t="n">
         <v>0.00305</v>
       </c>
       <c r="S10" s="8" t="n">
-        <v>0.04043</v>
+        <v>0.04045</v>
       </c>
       <c r="T10" s="8" t="n">
-        <v>0.09598</v>
+        <v>0.09594</v>
       </c>
       <c r="U10" s="8" t="n">
-        <v>0.00479</v>
+        <v>0.00478</v>
       </c>
       <c r="V10" s="8" t="n">
         <v>0.00715</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>0.26658</v>
+        <v>0.26622</v>
       </c>
       <c r="X10" s="8" t="n">
         <v>0.01709</v>
       </c>
       <c r="Y10" s="8" t="n">
-        <v>0.1223463927772788</v>
+        <v>0.1224196202016904</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>0.1243483529363782</v>
+        <v>0.1244117867432792</v>
       </c>
     </row>
     <row r="11">
@@ -1198,37 +1198,37 @@
         <v/>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0.14392</v>
+        <v>0.144</v>
       </c>
       <c r="Q11" s="8" t="n">
-        <v>0.04788</v>
+        <v>0.04791</v>
       </c>
       <c r="R11" s="8" t="n">
-        <v>0.01377</v>
+        <v>0.01378</v>
       </c>
       <c r="S11" s="8" t="n">
-        <v>0.03031</v>
+        <v>0.03032</v>
       </c>
       <c r="T11" s="8" t="n">
-        <v>0.06191</v>
+        <v>0.06187</v>
       </c>
       <c r="U11" s="8" t="n">
-        <v>0.009730000000000001</v>
+        <v>0.00971</v>
       </c>
       <c r="V11" s="8" t="n">
-        <v>0.0095</v>
+        <v>0.00949</v>
       </c>
       <c r="W11" s="8" t="n">
-        <v>0.19195</v>
+        <v>0.19166</v>
       </c>
       <c r="X11" s="8" t="n">
         <v>0.02656</v>
       </c>
       <c r="Y11" s="8" t="n">
-        <v>0.1160796094358666</v>
+        <v>0.1161494229705326</v>
       </c>
       <c r="Z11" s="8" t="n">
-        <v>0.1136814335225088</v>
+        <v>0.1137314937813253</v>
       </c>
     </row>
     <row r="12">
@@ -1295,37 +1295,37 @@
         <v/>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0.13311</v>
+        <v>0.13319</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>0.04477</v>
+        <v>0.04479</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>0.00755</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>0.03719</v>
+        <v>0.0372</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>0.06408999999999999</v>
+        <v>0.06406000000000001</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>0.02178</v>
+        <v>0.02176</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>0.00628</v>
       </c>
       <c r="W12" s="8" t="n">
-        <v>0.21601</v>
+        <v>0.2157</v>
       </c>
       <c r="X12" s="8" t="n">
         <v>0.04791</v>
       </c>
       <c r="Y12" s="8" t="n">
-        <v>0.13018246285228</v>
+        <v>0.1302523650577865</v>
       </c>
       <c r="Z12" s="8" t="n">
-        <v>0.1108095438484876</v>
+        <v>0.1108793242479339</v>
       </c>
     </row>
     <row r="13">
@@ -1392,37 +1392,37 @@
         <v/>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0.12874</v>
+        <v>0.12882</v>
       </c>
       <c r="Q13" s="8" t="n">
-        <v>0.04532</v>
+        <v>0.04535</v>
       </c>
       <c r="R13" s="8" t="n">
         <v>0.00096</v>
       </c>
       <c r="S13" s="8" t="n">
-        <v>0.0581</v>
+        <v>0.05813</v>
       </c>
       <c r="T13" s="8" t="n">
-        <v>0.0977</v>
+        <v>0.09767000000000001</v>
       </c>
       <c r="U13" s="8" t="n">
-        <v>0.0203</v>
+        <v>0.02029</v>
       </c>
       <c r="V13" s="8" t="n">
         <v>0.00874</v>
       </c>
       <c r="W13" s="8" t="n">
-        <v>0.23516</v>
+        <v>0.23484</v>
       </c>
       <c r="X13" s="8" t="n">
         <v>0.00442</v>
       </c>
       <c r="Y13" s="8" t="n">
-        <v>0.1231541199933732</v>
+        <v>0.1232192330356798</v>
       </c>
       <c r="Z13" s="8" t="n">
-        <v>0.1485172170670946</v>
+        <v>0.148603283285401</v>
       </c>
     </row>
     <row r="14">
@@ -1489,10 +1489,10 @@
         <v/>
       </c>
       <c r="P14" s="8" t="n">
-        <v>0.14558</v>
+        <v>0.14566</v>
       </c>
       <c r="Q14" s="8" t="n">
-        <v>0.04702</v>
+        <v>0.04705</v>
       </c>
       <c r="R14" s="8" t="n">
         <v>0.00604</v>
@@ -1501,25 +1501,25 @@
         <v>0.02935</v>
       </c>
       <c r="T14" s="8" t="n">
-        <v>0.09539</v>
+        <v>0.09536</v>
       </c>
       <c r="U14" s="8" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.00929</v>
       </c>
       <c r="V14" s="8" t="n">
-        <v>0.0049</v>
+        <v>0.00489</v>
       </c>
       <c r="W14" s="8" t="n">
-        <v>0.23092</v>
+        <v>0.23061</v>
       </c>
       <c r="X14" s="8" t="n">
         <v>0.02686</v>
       </c>
       <c r="Y14" s="8" t="n">
-        <v>0.1291248101605333</v>
+        <v>0.1292099478496693</v>
       </c>
       <c r="Z14" s="8" t="n">
-        <v>0.1021530808599572</v>
+        <v>0.1022073189681618</v>
       </c>
     </row>
     <row r="15">
@@ -1586,10 +1586,10 @@
         <v/>
       </c>
       <c r="P15" s="8" t="n">
-        <v>0.1589</v>
+        <v>0.15897</v>
       </c>
       <c r="Q15" s="8" t="n">
-        <v>0.04706</v>
+        <v>0.04708</v>
       </c>
       <c r="R15" s="8" t="n">
         <v>0.00192</v>
@@ -1598,25 +1598,25 @@
         <v>0.03972</v>
       </c>
       <c r="T15" s="8" t="n">
-        <v>0.07133</v>
+        <v>0.07129000000000001</v>
       </c>
       <c r="U15" s="8" t="n">
         <v>0.00715</v>
       </c>
       <c r="V15" s="8" t="n">
-        <v>0.00707</v>
+        <v>0.00706</v>
       </c>
       <c r="W15" s="8" t="n">
-        <v>0.16073</v>
+        <v>0.16048</v>
       </c>
       <c r="X15" s="8" t="n">
         <v>0.008869999999999999</v>
       </c>
       <c r="Y15" s="8" t="n">
-        <v>0.1078632243978509</v>
+        <v>0.1079168715572707</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>0.1280366537069566</v>
+        <v>0.1281085555872521</v>
       </c>
     </row>
     <row r="16">
@@ -1683,37 +1683,37 @@
         <v/>
       </c>
       <c r="P16" s="8" t="n">
-        <v>0.11156</v>
+        <v>0.11165</v>
       </c>
       <c r="Q16" s="8" t="n">
-        <v>0.03634</v>
+        <v>0.03637</v>
       </c>
       <c r="R16" s="8" t="n">
-        <v>0.00316</v>
+        <v>0.00315</v>
       </c>
       <c r="S16" s="8" t="n">
-        <v>0.04592</v>
+        <v>0.04595</v>
       </c>
       <c r="T16" s="8" t="n">
-        <v>0.14033</v>
+        <v>0.14029</v>
       </c>
       <c r="U16" s="8" t="n">
         <v>0.01368</v>
       </c>
       <c r="V16" s="8" t="n">
-        <v>0.00501</v>
+        <v>0.005</v>
       </c>
       <c r="W16" s="8" t="n">
-        <v>0.28351</v>
+        <v>0.28316</v>
       </c>
       <c r="X16" s="8" t="n">
         <v>0.0123</v>
       </c>
       <c r="Y16" s="8" t="n">
-        <v>0.1349953874482333</v>
+        <v>0.1350774781694497</v>
       </c>
       <c r="Z16" s="8" t="n">
-        <v>0.1084119107908361</v>
+        <v>0.1084738611938727</v>
       </c>
     </row>
     <row r="17">
@@ -1780,37 +1780,37 @@
         <v/>
       </c>
       <c r="P17" s="8" t="n">
-        <v>0.1378</v>
+        <v>0.13788</v>
       </c>
       <c r="Q17" s="8" t="n">
-        <v>0.04265</v>
+        <v>0.04268</v>
       </c>
       <c r="R17" s="8" t="n">
         <v>0.0013</v>
       </c>
       <c r="S17" s="8" t="n">
-        <v>0.05433</v>
+        <v>0.05434</v>
       </c>
       <c r="T17" s="8" t="n">
-        <v>0.08529</v>
+        <v>0.08524</v>
       </c>
       <c r="U17" s="8" t="n">
-        <v>0.00524</v>
+        <v>0.00523</v>
       </c>
       <c r="V17" s="8" t="n">
         <v>0.00626</v>
       </c>
       <c r="W17" s="8" t="n">
-        <v>0.19729</v>
+        <v>0.197</v>
       </c>
       <c r="X17" s="8" t="n">
         <v>0.009010000000000001</v>
       </c>
       <c r="Y17" s="8" t="n">
-        <v>0.1253299002189532</v>
+        <v>0.1253889592414693</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>0.1358544477204062</v>
+        <v>0.1359224420856638</v>
       </c>
     </row>
     <row r="18">
@@ -1877,37 +1877,37 @@
         <v/>
       </c>
       <c r="P18" s="8" t="n">
-        <v>0.13669</v>
+        <v>0.13678</v>
       </c>
       <c r="Q18" s="8" t="n">
-        <v>0.04439</v>
+        <v>0.04442</v>
       </c>
       <c r="R18" s="8" t="n">
         <v>0.00356</v>
       </c>
       <c r="S18" s="8" t="n">
-        <v>0.03161</v>
+        <v>0.03162</v>
       </c>
       <c r="T18" s="8" t="n">
-        <v>0.0728</v>
+        <v>0.07277</v>
       </c>
       <c r="U18" s="8" t="n">
-        <v>0.00861</v>
+        <v>0.0086</v>
       </c>
       <c r="V18" s="8" t="n">
-        <v>0.00523</v>
+        <v>0.00522</v>
       </c>
       <c r="W18" s="8" t="n">
-        <v>0.27099</v>
+        <v>0.27063</v>
       </c>
       <c r="X18" s="8" t="n">
         <v>0.02463</v>
       </c>
       <c r="Y18" s="8" t="n">
-        <v>0.1126209319600726</v>
+        <v>0.1126744668667468</v>
       </c>
       <c r="Z18" s="8" t="n">
-        <v>0.1168916300867914</v>
+        <v>0.1169544295762559</v>
       </c>
     </row>
     <row r="19">
@@ -1974,37 +1974,37 @@
         <v/>
       </c>
       <c r="P19" s="8" t="n">
-        <v>0.1381</v>
+        <v>0.13819</v>
       </c>
       <c r="Q19" s="8" t="n">
-        <v>0.04941</v>
+        <v>0.04945</v>
       </c>
       <c r="R19" s="8" t="n">
         <v>0.00573</v>
       </c>
       <c r="S19" s="8" t="n">
-        <v>0.03478</v>
+        <v>0.03479</v>
       </c>
       <c r="T19" s="8" t="n">
-        <v>0.0946</v>
+        <v>0.09456000000000001</v>
       </c>
       <c r="U19" s="8" t="n">
-        <v>0.0143</v>
+        <v>0.01429</v>
       </c>
       <c r="V19" s="8" t="n">
-        <v>0.00508</v>
+        <v>0.00507</v>
       </c>
       <c r="W19" s="8" t="n">
-        <v>0.23985</v>
+        <v>0.23952</v>
       </c>
       <c r="X19" s="8" t="n">
         <v>0.01286</v>
       </c>
       <c r="Y19" s="8" t="n">
-        <v>0.122874300413643</v>
+        <v>0.1229411148850543</v>
       </c>
       <c r="Z19" s="8" t="n">
-        <v>0.1156687087227195</v>
+        <v>0.1157447515711056</v>
       </c>
     </row>
     <row r="20">
@@ -2071,37 +2071,37 @@
         <v/>
       </c>
       <c r="P20" s="8" t="n">
-        <v>0.18561</v>
+        <v>0.18568</v>
       </c>
       <c r="Q20" s="8" t="n">
-        <v>0.0312</v>
+        <v>0.03121</v>
       </c>
       <c r="R20" s="8" t="n">
-        <v>0.00534</v>
+        <v>0.00535</v>
       </c>
       <c r="S20" s="8" t="n">
         <v>0.00733</v>
       </c>
       <c r="T20" s="8" t="n">
-        <v>0.09424</v>
+        <v>0.09419</v>
       </c>
       <c r="U20" s="8" t="n">
-        <v>0.00283</v>
+        <v>0.00282</v>
       </c>
       <c r="V20" s="8" t="n">
         <v>0.007889999999999999</v>
       </c>
       <c r="W20" s="8" t="n">
-        <v>0.15633</v>
+        <v>0.15608</v>
       </c>
       <c r="X20" s="8" t="n">
         <v>0.04288</v>
       </c>
       <c r="Y20" s="8" t="n">
-        <v>0.1095303386060655</v>
+        <v>0.1095880325500155</v>
       </c>
       <c r="Z20" s="8" t="n">
-        <v>0.0787166143991179</v>
+        <v>0.078755111683385</v>
       </c>
     </row>
     <row r="21">
@@ -2168,37 +2168,37 @@
         <v/>
       </c>
       <c r="P21" s="8" t="n">
-        <v>0.18448</v>
+        <v>0.18455</v>
       </c>
       <c r="Q21" s="8" t="n">
-        <v>0.04554</v>
+        <v>0.04557</v>
       </c>
       <c r="R21" s="8" t="n">
         <v>0.00671</v>
       </c>
       <c r="S21" s="8" t="n">
-        <v>0.01457</v>
+        <v>0.01458</v>
       </c>
       <c r="T21" s="8" t="n">
-        <v>0.06319</v>
+        <v>0.06315</v>
       </c>
       <c r="U21" s="8" t="n">
-        <v>0.01009</v>
+        <v>0.01008</v>
       </c>
       <c r="V21" s="8" t="n">
-        <v>0.00721</v>
+        <v>0.0072</v>
       </c>
       <c r="W21" s="8" t="n">
-        <v>0.1175</v>
+        <v>0.1173</v>
       </c>
       <c r="X21" s="8" t="n">
         <v>0.01942</v>
       </c>
       <c r="Y21" s="8" t="n">
-        <v>0.1132438842706345</v>
+        <v>0.113306937605512</v>
       </c>
       <c r="Z21" s="8" t="n">
-        <v>0.0931355258252959</v>
+        <v>0.09319789018818769</v>
       </c>
     </row>
     <row r="22">
@@ -2265,37 +2265,37 @@
         <v/>
       </c>
       <c r="P22" s="8" t="n">
-        <v>0.14454</v>
+        <v>0.14463</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>0.03965</v>
+        <v>0.03967</v>
       </c>
       <c r="R22" s="8" t="n">
         <v>0.00765</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>0.0177</v>
+        <v>0.01771</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>0.11189</v>
+        <v>0.11184</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>0.01865</v>
+        <v>0.01864</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>0.00268</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>0.212</v>
+        <v>0.21169</v>
       </c>
       <c r="X22" s="8" t="n">
         <v>0.04402</v>
       </c>
       <c r="Y22" s="8" t="n">
-        <v>0.1189968621440421</v>
+        <v>0.1190641182787549</v>
       </c>
       <c r="Z22" s="8" t="n">
-        <v>0.08450488029733851</v>
+        <v>0.084552917395051</v>
       </c>
     </row>
     <row r="23">
@@ -2362,37 +2362,37 @@
         <v/>
       </c>
       <c r="P23" s="8" t="n">
-        <v>0.177</v>
+        <v>0.17709</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>0.03647</v>
+        <v>0.03649</v>
       </c>
       <c r="R23" s="8" t="n">
         <v>0.00173</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>0.02961</v>
+        <v>0.02962</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>0.09182999999999999</v>
+        <v>0.09177</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>0.0106</v>
+        <v>0.01059</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>0.00569</v>
+        <v>0.00568</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>0.14975</v>
+        <v>0.14952</v>
       </c>
       <c r="X23" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="Y23" s="8" t="n">
-        <v>0.1165803451467095</v>
+        <v>0.1166303489644284</v>
       </c>
       <c r="Z23" s="8" t="n">
-        <v>0.1116122956845203</v>
+        <v>0.1116529889391497</v>
       </c>
     </row>
     <row r="24">
@@ -2459,37 +2459,37 @@
         <v/>
       </c>
       <c r="P24" s="8" t="n">
-        <v>0.11644</v>
+        <v>0.11652</v>
       </c>
       <c r="Q24" s="8" t="n">
-        <v>0.04929</v>
+        <v>0.04933</v>
       </c>
       <c r="R24" s="8" t="n">
         <v>0.00157</v>
       </c>
       <c r="S24" s="8" t="n">
-        <v>0.04716</v>
+        <v>0.04717</v>
       </c>
       <c r="T24" s="8" t="n">
-        <v>0.10926</v>
+        <v>0.10922</v>
       </c>
       <c r="U24" s="8" t="n">
-        <v>0.00669</v>
+        <v>0.00668</v>
       </c>
       <c r="V24" s="8" t="n">
-        <v>0.00666</v>
+        <v>0.00665</v>
       </c>
       <c r="W24" s="8" t="n">
-        <v>0.24737</v>
+        <v>0.24703</v>
       </c>
       <c r="X24" s="8" t="n">
         <v>0.00144</v>
       </c>
       <c r="Y24" s="8" t="n">
-        <v>0.1267743118205152</v>
+        <v>0.1268448235725187</v>
       </c>
       <c r="Z24" s="8" t="n">
-        <v>0.13323747662287</v>
+        <v>0.133318170511943</v>
       </c>
     </row>
     <row r="25">
@@ -2556,37 +2556,37 @@
         <v/>
       </c>
       <c r="P25" s="8" t="n">
-        <v>0.11348</v>
+        <v>0.11356</v>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>0.04867</v>
+        <v>0.04871</v>
       </c>
       <c r="R25" s="8" t="n">
         <v>0.00231</v>
       </c>
       <c r="S25" s="8" t="n">
-        <v>0.04956</v>
+        <v>0.04958</v>
       </c>
       <c r="T25" s="8" t="n">
-        <v>0.09097</v>
+        <v>0.09095</v>
       </c>
       <c r="U25" s="8" t="n">
         <v>0.0107</v>
       </c>
       <c r="V25" s="8" t="n">
-        <v>0.00568</v>
+        <v>0.00567</v>
       </c>
       <c r="W25" s="8" t="n">
-        <v>0.27779</v>
+        <v>0.27742</v>
       </c>
       <c r="X25" s="8" t="n">
         <v>0.01097</v>
       </c>
       <c r="Y25" s="8" t="n">
-        <v>0.127395410324242</v>
+        <v>0.1274595313651934</v>
       </c>
       <c r="Z25" s="8" t="n">
-        <v>0.1468158701062275</v>
+        <v>0.1469006423682971</v>
       </c>
     </row>
     <row r="26">
@@ -2653,53 +2653,53 @@
         <v/>
       </c>
       <c r="P26" s="8" t="n">
-        <v>0.14129</v>
+        <v>0.14138</v>
       </c>
       <c r="Q26" s="8" t="n">
-        <v>0.04339</v>
+        <v>0.04341</v>
       </c>
       <c r="R26" s="8" t="n">
-        <v>0.009140000000000001</v>
+        <v>0.00915</v>
       </c>
       <c r="S26" s="8" t="n">
-        <v>0.02751</v>
+        <v>0.02753</v>
       </c>
       <c r="T26" s="8" t="n">
-        <v>0.07277</v>
+        <v>0.07275</v>
       </c>
       <c r="U26" s="8" t="n">
         <v>0.01141</v>
       </c>
       <c r="V26" s="8" t="n">
-        <v>0.00598</v>
+        <v>0.00597</v>
       </c>
       <c r="W26" s="8" t="n">
-        <v>0.25176</v>
+        <v>0.2514</v>
       </c>
       <c r="X26" s="8" t="n">
         <v>0.0397</v>
       </c>
       <c r="Y26" s="8" t="n">
-        <v>0.115240493757318</v>
+        <v>0.1152966838962423</v>
       </c>
       <c r="Z26" s="8" t="n">
-        <v>0.1025389914503331</v>
+        <v>0.1025944232805242</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Everyday DH / 1B-DH</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
@@ -2750,53 +2750,53 @@
         <v/>
       </c>
       <c r="P27" s="8" t="n">
-        <v>0.14576</v>
+        <v>0.13896</v>
       </c>
       <c r="Q27" s="8" t="n">
-        <v>0.04292</v>
+        <v>0.04324</v>
       </c>
       <c r="R27" s="8" t="n">
-        <v>0.00178</v>
+        <v>0.007889999999999999</v>
       </c>
       <c r="S27" s="8" t="n">
-        <v>0.03655</v>
+        <v>0.02951</v>
       </c>
       <c r="T27" s="8" t="n">
-        <v>0.09699000000000001</v>
+        <v>0.12461</v>
       </c>
       <c r="U27" s="8" t="n">
-        <v>0.01604</v>
+        <v>0.0048</v>
       </c>
       <c r="V27" s="8" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.00566</v>
       </c>
       <c r="W27" s="8" t="n">
-        <v>0.25213</v>
+        <v>0.15674</v>
       </c>
       <c r="X27" s="8" t="n">
-        <v>0.00285</v>
+        <v>0.01801</v>
       </c>
       <c r="Y27" s="8" t="n">
-        <v>0.113020713590306</v>
+        <v>0.1298104529584322</v>
       </c>
       <c r="Z27" s="8" t="n">
-        <v>0.1200724498172191</v>
+        <v>0.1025692821317952</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Full Time</t>
+          <t>Everyday DH / 1B-DH</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
@@ -2847,37 +2847,37 @@
         <v/>
       </c>
       <c r="P28" s="8" t="n">
-        <v>0.1389</v>
+        <v>0.14586</v>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>0.04321</v>
+        <v>0.04295</v>
       </c>
       <c r="R28" s="8" t="n">
-        <v>0.007889999999999999</v>
+        <v>0.00178</v>
       </c>
       <c r="S28" s="8" t="n">
-        <v>0.0295</v>
+        <v>0.03656</v>
       </c>
       <c r="T28" s="8" t="n">
-        <v>0.12468</v>
+        <v>0.09694999999999999</v>
       </c>
       <c r="U28" s="8" t="n">
-        <v>0.00481</v>
+        <v>0.01603</v>
       </c>
       <c r="V28" s="8" t="n">
-        <v>0.00567</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="W28" s="8" t="n">
-        <v>0.15699</v>
+        <v>0.25179</v>
       </c>
       <c r="X28" s="8" t="n">
-        <v>0.01801</v>
+        <v>0.00285</v>
       </c>
       <c r="Y28" s="8" t="n">
-        <v>0.1297388573590071</v>
+        <v>0.1130709577835605</v>
       </c>
       <c r="Z28" s="8" t="n">
-        <v>0.1025079654509587</v>
+        <v>0.120122217819372</v>
       </c>
     </row>
     <row r="29">
@@ -2944,37 +2944,37 @@
         <v/>
       </c>
       <c r="P29" s="8" t="n">
-        <v>0.09565</v>
+        <v>0.09573</v>
       </c>
       <c r="Q29" s="8" t="n">
-        <v>0.03733</v>
+        <v>0.03736</v>
       </c>
       <c r="R29" s="8" t="n">
         <v>0.00154</v>
       </c>
       <c r="S29" s="8" t="n">
-        <v>0.06146</v>
+        <v>0.06149</v>
       </c>
       <c r="T29" s="8" t="n">
-        <v>0.14532</v>
+        <v>0.14529</v>
       </c>
       <c r="U29" s="8" t="n">
-        <v>0.00942</v>
+        <v>0.00941</v>
       </c>
       <c r="V29" s="8" t="n">
-        <v>0.0056</v>
+        <v>0.00559</v>
       </c>
       <c r="W29" s="8" t="n">
-        <v>0.29725</v>
+        <v>0.29689</v>
       </c>
       <c r="X29" s="8" t="n">
         <v>0.00756</v>
       </c>
       <c r="Y29" s="8" t="n">
-        <v>0.1374788380219203</v>
+        <v>0.1375454863523066</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>0.1403508871636152</v>
+        <v>0.1404276848359008</v>
       </c>
     </row>
     <row r="30">
@@ -3041,37 +3041,37 @@
         <v/>
       </c>
       <c r="P30" s="8" t="n">
-        <v>0.11346</v>
+        <v>0.11354</v>
       </c>
       <c r="Q30" s="8" t="n">
-        <v>0.04915</v>
+        <v>0.04918</v>
       </c>
       <c r="R30" s="8" t="n">
         <v>0.0066</v>
       </c>
       <c r="S30" s="8" t="n">
-        <v>0.0645</v>
+        <v>0.06453</v>
       </c>
       <c r="T30" s="8" t="n">
-        <v>0.12629</v>
+        <v>0.12625</v>
       </c>
       <c r="U30" s="8" t="n">
         <v>0.00705</v>
       </c>
       <c r="V30" s="8" t="n">
-        <v>0.00531</v>
+        <v>0.0053</v>
       </c>
       <c r="W30" s="8" t="n">
-        <v>0.24667</v>
+        <v>0.24633</v>
       </c>
       <c r="X30" s="8" t="n">
         <v>0.03207</v>
       </c>
       <c r="Y30" s="8" t="n">
-        <v>0.1657200911231141</v>
+        <v>0.1657950155444659</v>
       </c>
       <c r="Z30" s="8" t="n">
-        <v>0.1477317382817687</v>
+        <v>0.1478070775708195</v>
       </c>
     </row>
     <row r="33">
@@ -3244,39 +3244,39 @@
         <v/>
       </c>
       <c r="N35" s="8" t="n">
-        <v>4.177</v>
+        <v>4.176</v>
       </c>
       <c r="O35" s="8" t="n">
-        <v>0.21648</v>
+        <v>0.217</v>
       </c>
       <c r="P35" s="8" t="n">
-        <v>0.05744</v>
+        <v>0.05752</v>
       </c>
       <c r="Q35" s="8" t="n">
-        <v>0.02102</v>
+        <v>0.02104</v>
       </c>
       <c r="R35" s="8" t="n">
-        <v>0.17117</v>
+        <v>0.17097</v>
       </c>
       <c r="S35" s="8" t="n">
-        <v>0.03998</v>
+        <v>0.03992</v>
       </c>
       <c r="T35" s="8" t="n">
-        <v>0.00498</v>
+        <v>0.00497</v>
       </c>
       <c r="U35" s="8" t="n">
-        <v>3.81176</v>
+        <v>3.80698</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Nolan McLean</t>
+          <t>Sandy Alcantara</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3324,39 +3324,39 @@
         <v/>
       </c>
       <c r="N36" s="8" t="n">
-        <v>4.21</v>
+        <v>4.223</v>
       </c>
       <c r="O36" s="8" t="n">
-        <v>0.25368</v>
+        <v>0.19018</v>
       </c>
       <c r="P36" s="8" t="n">
-        <v>0.09253</v>
+        <v>0.06875000000000001</v>
       </c>
       <c r="Q36" s="8" t="n">
-        <v>0.02147</v>
+        <v>0.02673</v>
       </c>
       <c r="R36" s="8" t="n">
-        <v>0.13546</v>
+        <v>0.15449</v>
       </c>
       <c r="S36" s="8" t="n">
-        <v>0.03736</v>
+        <v>0.04578</v>
       </c>
       <c r="T36" s="8" t="n">
-        <v>0.00316</v>
+        <v>0.0044</v>
       </c>
       <c r="U36" s="8" t="n">
-        <v>3.61038</v>
+        <v>4.17694</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Sandy Alcantara</t>
+          <t>Nolan McLean</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3404,28 +3404,28 @@
         <v/>
       </c>
       <c r="N37" s="8" t="n">
-        <v>4.224</v>
+        <v>4.209</v>
       </c>
       <c r="O37" s="8" t="n">
-        <v>0.18972</v>
+        <v>0.25423</v>
       </c>
       <c r="P37" s="8" t="n">
-        <v>0.06865</v>
+        <v>0.09264</v>
       </c>
       <c r="Q37" s="8" t="n">
-        <v>0.02671</v>
+        <v>0.02148</v>
       </c>
       <c r="R37" s="8" t="n">
-        <v>0.15467</v>
+        <v>0.13526</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>0.04585</v>
+        <v>0.03729</v>
       </c>
       <c r="T37" s="8" t="n">
-        <v>0.00441</v>
+        <v>0.00316</v>
       </c>
       <c r="U37" s="8" t="n">
-        <v>4.18097</v>
+        <v>3.60625</v>
       </c>
     </row>
     <row r="38">
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>212</v>
+        <v>212.7</v>
       </c>
       <c r="E38" s="6">
         <f>D38*N38</f>
@@ -3484,28 +3484,28 @@
         <v/>
       </c>
       <c r="N38" s="8" t="n">
-        <v>4.335</v>
+        <v>4.334</v>
       </c>
       <c r="O38" s="8" t="n">
-        <v>0.16211</v>
+        <v>0.16252</v>
       </c>
       <c r="P38" s="8" t="n">
-        <v>0.08626</v>
+        <v>0.08638999999999999</v>
       </c>
       <c r="Q38" s="8" t="n">
-        <v>0.02071</v>
+        <v>0.02073</v>
       </c>
       <c r="R38" s="8" t="n">
-        <v>0.17337</v>
+        <v>0.17318</v>
       </c>
       <c r="S38" s="8" t="n">
-        <v>0.03691</v>
+        <v>0.03686</v>
       </c>
       <c r="T38" s="8" t="n">
-        <v>0.00408</v>
+        <v>0.00407</v>
       </c>
       <c r="U38" s="8" t="n">
-        <v>4.21378</v>
+        <v>4.21019</v>
       </c>
     </row>
     <row r="39">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>211.1</v>
+        <v>211.8</v>
       </c>
       <c r="E39" s="6">
         <f>D39*N39</f>
@@ -3567,25 +3567,25 @@
         <v>4.274</v>
       </c>
       <c r="O39" s="8" t="n">
-        <v>0.16461</v>
+        <v>0.16504</v>
       </c>
       <c r="P39" s="8" t="n">
-        <v>0.06444999999999999</v>
+        <v>0.06455</v>
       </c>
       <c r="Q39" s="8" t="n">
-        <v>0.03342</v>
+        <v>0.03345</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>0.16413</v>
+        <v>0.16396</v>
       </c>
       <c r="S39" s="8" t="n">
-        <v>0.04733</v>
+        <v>0.04726</v>
       </c>
       <c r="T39" s="8" t="n">
-        <v>0.0044</v>
+        <v>0.00439</v>
       </c>
       <c r="U39" s="8" t="n">
-        <v>4.67496</v>
+        <v>4.67108</v>
       </c>
     </row>
     <row r="40">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>198.7</v>
+        <v>199</v>
       </c>
       <c r="E40" s="6">
         <f>D40*N40</f>
@@ -3647,25 +3647,25 @@
         <v>4.169</v>
       </c>
       <c r="O40" s="8" t="n">
-        <v>0.19438</v>
+        <v>0.19486</v>
       </c>
       <c r="P40" s="8" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.0687</v>
       </c>
       <c r="Q40" s="8" t="n">
-        <v>0.03149</v>
+        <v>0.03151</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>0.13926</v>
+        <v>0.1391</v>
       </c>
       <c r="S40" s="8" t="n">
-        <v>0.04866</v>
+        <v>0.04859</v>
       </c>
       <c r="T40" s="8" t="n">
-        <v>0.00604</v>
+        <v>0.00602</v>
       </c>
       <c r="U40" s="8" t="n">
-        <v>4.2136</v>
+        <v>4.20948</v>
       </c>
     </row>
     <row r="41">
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>196.2</v>
+        <v>196.5</v>
       </c>
       <c r="E41" s="6">
         <f>D41*N41</f>
@@ -3724,28 +3724,28 @@
         <v/>
       </c>
       <c r="N41" s="8" t="n">
-        <v>4.009</v>
+        <v>4.008</v>
       </c>
       <c r="O41" s="8" t="n">
-        <v>0.28284</v>
+        <v>0.28344</v>
       </c>
       <c r="P41" s="8" t="n">
-        <v>0.06644</v>
+        <v>0.06651</v>
       </c>
       <c r="Q41" s="8" t="n">
-        <v>0.02328</v>
+        <v>0.0233</v>
       </c>
       <c r="R41" s="8" t="n">
-        <v>0.12982</v>
+        <v>0.12962</v>
       </c>
       <c r="S41" s="8" t="n">
-        <v>0.03786</v>
+        <v>0.03779</v>
       </c>
       <c r="T41" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="U41" s="8" t="n">
-        <v>3.11165</v>
+        <v>3.10699</v>
       </c>
     </row>
     <row r="42">
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>195.7</v>
+        <v>195.8</v>
       </c>
       <c r="E42" s="6">
         <f>D42*N42</f>
@@ -3804,28 +3804,28 @@
         <v/>
       </c>
       <c r="N42" s="8" t="n">
-        <v>4.109</v>
+        <v>4.108</v>
       </c>
       <c r="O42" s="8" t="n">
-        <v>0.23924</v>
+        <v>0.2398</v>
       </c>
       <c r="P42" s="8" t="n">
-        <v>0.05788</v>
+        <v>0.05796</v>
       </c>
       <c r="Q42" s="8" t="n">
-        <v>0.02034</v>
+        <v>0.02036</v>
       </c>
       <c r="R42" s="8" t="n">
-        <v>0.16384</v>
+        <v>0.16363</v>
       </c>
       <c r="S42" s="8" t="n">
-        <v>0.03974</v>
+        <v>0.03968</v>
       </c>
       <c r="T42" s="8" t="n">
         <v>0.00258</v>
       </c>
       <c r="U42" s="8" t="n">
-        <v>3.47409</v>
+        <v>3.46961</v>
       </c>
     </row>
     <row r="43">
@@ -3845,7 +3845,7 @@
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>190.8</v>
+        <v>191.4</v>
       </c>
       <c r="E43" s="6">
         <f>D43*N43</f>
@@ -3884,28 +3884,28 @@
         <v/>
       </c>
       <c r="N43" s="8" t="n">
-        <v>4.133</v>
+        <v>4.132</v>
       </c>
       <c r="O43" s="8" t="n">
-        <v>0.2594</v>
+        <v>0.25996</v>
       </c>
       <c r="P43" s="8" t="n">
-        <v>0.09172</v>
+        <v>0.09182999999999999</v>
       </c>
       <c r="Q43" s="8" t="n">
-        <v>0.02049</v>
+        <v>0.0205</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>0.14158</v>
+        <v>0.14138</v>
       </c>
       <c r="S43" s="8" t="n">
-        <v>0.02824</v>
+        <v>0.02819</v>
       </c>
       <c r="T43" s="8" t="n">
         <v>0.00328</v>
       </c>
       <c r="U43" s="8" t="n">
-        <v>3.24041</v>
+        <v>3.23628</v>
       </c>
     </row>
     <row r="44">
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>189.6</v>
+        <v>190.1</v>
       </c>
       <c r="E44" s="6">
         <f>D44*N44</f>
@@ -3964,28 +3964,28 @@
         <v/>
       </c>
       <c r="N44" s="8" t="n">
-        <v>4.251</v>
+        <v>4.25</v>
       </c>
       <c r="O44" s="8" t="n">
-        <v>0.21665</v>
+        <v>0.21715</v>
       </c>
       <c r="P44" s="8" t="n">
-        <v>0.08314000000000001</v>
+        <v>0.08323999999999999</v>
       </c>
       <c r="Q44" s="8" t="n">
-        <v>0.0197</v>
+        <v>0.01972</v>
       </c>
       <c r="R44" s="8" t="n">
-        <v>0.15454</v>
+        <v>0.15434</v>
       </c>
       <c r="S44" s="8" t="n">
-        <v>0.04108</v>
+        <v>0.04101</v>
       </c>
       <c r="T44" s="8" t="n">
         <v>0.00366</v>
       </c>
       <c r="U44" s="8" t="n">
-        <v>3.85848</v>
+        <v>3.85389</v>
       </c>
     </row>
     <row r="45">
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>187.9</v>
+        <v>188.3</v>
       </c>
       <c r="E45" s="6">
         <f>D45*N45</f>
@@ -4044,28 +4044,28 @@
         <v/>
       </c>
       <c r="N45" s="8" t="n">
-        <v>4.34</v>
+        <v>4.339</v>
       </c>
       <c r="O45" s="8" t="n">
-        <v>0.1896</v>
+        <v>0.19004</v>
       </c>
       <c r="P45" s="8" t="n">
-        <v>0.08619</v>
+        <v>0.0863</v>
       </c>
       <c r="Q45" s="8" t="n">
-        <v>0.04325</v>
+        <v>0.04328</v>
       </c>
       <c r="R45" s="8" t="n">
-        <v>0.13977</v>
+        <v>0.13959</v>
       </c>
       <c r="S45" s="8" t="n">
-        <v>0.04412</v>
+        <v>0.04405</v>
       </c>
       <c r="T45" s="8" t="n">
         <v>0.00459</v>
       </c>
       <c r="U45" s="8" t="n">
-        <v>5.04469</v>
+        <v>5.04139</v>
       </c>
     </row>
     <row r="46">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>186.4</v>
+        <v>186.8</v>
       </c>
       <c r="E46" s="6">
         <f>D46*N46</f>
@@ -4124,28 +4124,28 @@
         <v/>
       </c>
       <c r="N46" s="8" t="n">
-        <v>4.05</v>
+        <v>4.049</v>
       </c>
       <c r="O46" s="8" t="n">
-        <v>0.29876</v>
+        <v>0.29938</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>0.0669</v>
+        <v>0.06698</v>
       </c>
       <c r="Q46" s="8" t="n">
-        <v>0.0294</v>
+        <v>0.02941</v>
       </c>
       <c r="R46" s="8" t="n">
-        <v>0.13364</v>
+        <v>0.13344</v>
       </c>
       <c r="S46" s="8" t="n">
-        <v>0.03966</v>
+        <v>0.03959</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0.00272</v>
       </c>
       <c r="U46" s="8" t="n">
-        <v>3.4427</v>
+        <v>3.43729</v>
       </c>
     </row>
     <row r="47">
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>184.9</v>
+        <v>185.4</v>
       </c>
       <c r="E47" s="6">
         <f>D47*N47</f>
@@ -4204,28 +4204,28 @@
         <v/>
       </c>
       <c r="N47" s="8" t="n">
-        <v>4.345</v>
+        <v>4.344</v>
       </c>
       <c r="O47" s="8" t="n">
-        <v>0.20476</v>
+        <v>0.20524</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>0.07475</v>
+        <v>0.07485</v>
       </c>
       <c r="Q47" s="8" t="n">
-        <v>0.02964</v>
+        <v>0.02966</v>
       </c>
       <c r="R47" s="8" t="n">
-        <v>0.15536</v>
+        <v>0.15516</v>
       </c>
       <c r="S47" s="8" t="n">
-        <v>0.04914</v>
+        <v>0.04907</v>
       </c>
       <c r="T47" s="8" t="n">
         <v>0.0043</v>
       </c>
       <c r="U47" s="8" t="n">
-        <v>4.6786</v>
+        <v>4.67393</v>
       </c>
     </row>
     <row r="48">
@@ -4245,7 +4245,7 @@
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>183.7</v>
+        <v>184.3</v>
       </c>
       <c r="E48" s="6">
         <f>D48*N48</f>
@@ -4284,48 +4284,48 @@
         <v/>
       </c>
       <c r="N48" s="8" t="n">
-        <v>4.285</v>
+        <v>4.284</v>
       </c>
       <c r="O48" s="8" t="n">
-        <v>0.24135</v>
+        <v>0.24189</v>
       </c>
       <c r="P48" s="8" t="n">
-        <v>0.08685</v>
+        <v>0.08696</v>
       </c>
       <c r="Q48" s="8" t="n">
-        <v>0.03498</v>
+        <v>0.03499</v>
       </c>
       <c r="R48" s="8" t="n">
-        <v>0.13607</v>
+        <v>0.13589</v>
       </c>
       <c r="S48" s="8" t="n">
-        <v>0.05158</v>
+        <v>0.05149</v>
       </c>
       <c r="T48" s="8" t="n">
         <v>0.00334</v>
       </c>
       <c r="U48" s="8" t="n">
-        <v>4.57799</v>
+        <v>4.57243</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Noah Cameron</t>
+          <t>Tarik Skubal</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Mid-Rotation Starter (SP2-3)</t>
+          <t>Ace (SP1)</t>
         </is>
       </c>
       <c r="D49" s="5" t="n">
-        <v>181.7</v>
+        <v>182</v>
       </c>
       <c r="E49" s="6">
         <f>D49*N49</f>
@@ -4364,48 +4364,48 @@
         <v/>
       </c>
       <c r="N49" s="8" t="n">
-        <v>4.189</v>
+        <v>3.956</v>
       </c>
       <c r="O49" s="8" t="n">
-        <v>0.2054</v>
+        <v>0.29099</v>
       </c>
       <c r="P49" s="8" t="n">
-        <v>0.07975</v>
+        <v>0.05095</v>
       </c>
       <c r="Q49" s="8" t="n">
-        <v>0.03047</v>
+        <v>0.02316</v>
       </c>
       <c r="R49" s="8" t="n">
-        <v>0.14218</v>
+        <v>0.14109</v>
       </c>
       <c r="S49" s="8" t="n">
-        <v>0.04211</v>
+        <v>0.0371</v>
       </c>
       <c r="T49" s="8" t="n">
-        <v>0.00353</v>
+        <v>0.00319</v>
       </c>
       <c r="U49" s="8" t="n">
-        <v>4.05708</v>
+        <v>2.98544</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Tarik Skubal</t>
+          <t>Noah Cameron</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Ace (SP1)</t>
+          <t>Mid-Rotation Starter (SP2-3)</t>
         </is>
       </c>
       <c r="D50" s="5" t="n">
-        <v>181.6</v>
+        <v>182</v>
       </c>
       <c r="E50" s="6">
         <f>D50*N50</f>
@@ -4444,28 +4444,28 @@
         <v/>
       </c>
       <c r="N50" s="8" t="n">
-        <v>3.957</v>
+        <v>4.188</v>
       </c>
       <c r="O50" s="8" t="n">
-        <v>0.29037</v>
+        <v>0.20589</v>
       </c>
       <c r="P50" s="8" t="n">
-        <v>0.05088</v>
+        <v>0.07985</v>
       </c>
       <c r="Q50" s="8" t="n">
-        <v>0.02315</v>
+        <v>0.03049</v>
       </c>
       <c r="R50" s="8" t="n">
-        <v>0.1413</v>
+        <v>0.14201</v>
       </c>
       <c r="S50" s="8" t="n">
-        <v>0.03717</v>
+        <v>0.04204</v>
       </c>
       <c r="T50" s="8" t="n">
-        <v>0.00319</v>
+        <v>0.00353</v>
       </c>
       <c r="U50" s="8" t="n">
-        <v>2.99035</v>
+        <v>4.05278</v>
       </c>
     </row>
     <row r="51">
@@ -4485,7 +4485,7 @@
         </is>
       </c>
       <c r="D51" s="5" t="n">
-        <v>180.5</v>
+        <v>180.7</v>
       </c>
       <c r="E51" s="6">
         <f>D51*N51</f>
@@ -4524,39 +4524,39 @@
         <v/>
       </c>
       <c r="N51" s="8" t="n">
-        <v>4.034</v>
+        <v>4.033</v>
       </c>
       <c r="O51" s="8" t="n">
-        <v>0.26047</v>
+        <v>0.26106</v>
       </c>
       <c r="P51" s="8" t="n">
-        <v>0.05921</v>
+        <v>0.05928</v>
       </c>
       <c r="Q51" s="8" t="n">
-        <v>0.03685</v>
+        <v>0.03687</v>
       </c>
       <c r="R51" s="8" t="n">
-        <v>0.13085</v>
+        <v>0.13067</v>
       </c>
       <c r="S51" s="8" t="n">
-        <v>0.04077</v>
+        <v>0.0407</v>
       </c>
       <c r="T51" s="8" t="n">
         <v>0.00277</v>
       </c>
       <c r="U51" s="8" t="n">
-        <v>3.71535</v>
+        <v>3.71069</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Seth Lugo</t>
+          <t>Freddy Peralta</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>178.8</v>
+        <v>179.6</v>
       </c>
       <c r="E52" s="6">
         <f>D52*N52</f>
@@ -4604,39 +4604,39 @@
         <v/>
       </c>
       <c r="N52" s="8" t="n">
-        <v>4.285</v>
+        <v>4.175</v>
       </c>
       <c r="O52" s="8" t="n">
-        <v>0.20199</v>
+        <v>0.25531</v>
       </c>
       <c r="P52" s="8" t="n">
-        <v>0.0721</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="Q52" s="8" t="n">
-        <v>0.03645</v>
+        <v>0.02869</v>
       </c>
       <c r="R52" s="8" t="n">
-        <v>0.1485</v>
+        <v>0.13059</v>
       </c>
       <c r="S52" s="8" t="n">
-        <v>0.04779</v>
+        <v>0.03841</v>
       </c>
       <c r="T52" s="8" t="n">
-        <v>0.00533</v>
+        <v>0.00359</v>
       </c>
       <c r="U52" s="8" t="n">
-        <v>4.73904</v>
+        <v>3.78599</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Freddy Peralta</t>
+          <t>Seth Lugo</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4645,7 +4645,7 @@
         </is>
       </c>
       <c r="D53" s="5" t="n">
-        <v>178.6</v>
+        <v>179.2</v>
       </c>
       <c r="E53" s="6">
         <f>D53*N53</f>
@@ -4684,28 +4684,28 @@
         <v/>
       </c>
       <c r="N53" s="8" t="n">
-        <v>4.176</v>
+        <v>4.284</v>
       </c>
       <c r="O53" s="8" t="n">
-        <v>0.25476</v>
+        <v>0.20247</v>
       </c>
       <c r="P53" s="8" t="n">
-        <v>0.08928999999999999</v>
+        <v>0.07219</v>
       </c>
       <c r="Q53" s="8" t="n">
-        <v>0.02868</v>
+        <v>0.03648</v>
       </c>
       <c r="R53" s="8" t="n">
-        <v>0.13078</v>
+        <v>0.14832</v>
       </c>
       <c r="S53" s="8" t="n">
-        <v>0.03848</v>
+        <v>0.04772</v>
       </c>
       <c r="T53" s="8" t="n">
-        <v>0.00359</v>
+        <v>0.00531</v>
       </c>
       <c r="U53" s="8" t="n">
-        <v>3.79051</v>
+        <v>4.73457</v>
       </c>
     </row>
     <row r="54">
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>178.5</v>
+        <v>178.9</v>
       </c>
       <c r="E54" s="6">
         <f>D54*N54</f>
@@ -4764,28 +4764,28 @@
         <v/>
       </c>
       <c r="N54" s="8" t="n">
-        <v>4.234</v>
+        <v>4.233</v>
       </c>
       <c r="O54" s="8" t="n">
-        <v>0.20431</v>
+        <v>0.20479</v>
       </c>
       <c r="P54" s="8" t="n">
-        <v>0.07996</v>
+        <v>0.08008</v>
       </c>
       <c r="Q54" s="8" t="n">
-        <v>0.03975</v>
+        <v>0.03977</v>
       </c>
       <c r="R54" s="8" t="n">
-        <v>0.13812</v>
+        <v>0.13796</v>
       </c>
       <c r="S54" s="8" t="n">
-        <v>0.04587</v>
+        <v>0.04579</v>
       </c>
       <c r="T54" s="8" t="n">
         <v>0.00309</v>
       </c>
       <c r="U54" s="8" t="n">
-        <v>4.56318</v>
+        <v>4.55937</v>
       </c>
     </row>
     <row r="55">
@@ -4805,7 +4805,7 @@
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>177.7</v>
+        <v>178.3</v>
       </c>
       <c r="E55" s="6">
         <f>D55*N55</f>
@@ -4844,28 +4844,28 @@
         <v/>
       </c>
       <c r="N55" s="8" t="n">
-        <v>4.067</v>
+        <v>4.066</v>
       </c>
       <c r="O55" s="8" t="n">
-        <v>0.22988</v>
+        <v>0.23041</v>
       </c>
       <c r="P55" s="8" t="n">
-        <v>0.06849</v>
+        <v>0.06858</v>
       </c>
       <c r="Q55" s="8" t="n">
         <v>0.01736</v>
       </c>
       <c r="R55" s="8" t="n">
-        <v>0.15085</v>
+        <v>0.15066</v>
       </c>
       <c r="S55" s="8" t="n">
-        <v>0.03607</v>
+        <v>0.03601</v>
       </c>
       <c r="T55" s="8" t="n">
         <v>0.00235</v>
       </c>
       <c r="U55" s="8" t="n">
-        <v>3.13524</v>
+        <v>3.13062</v>
       </c>
     </row>
     <row r="56">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>175.6</v>
+        <v>175.8</v>
       </c>
       <c r="E56" s="6">
         <f>D56*N56</f>
@@ -4924,28 +4924,28 @@
         <v/>
       </c>
       <c r="N56" s="8" t="n">
-        <v>4.041</v>
+        <v>4.04</v>
       </c>
       <c r="O56" s="8" t="n">
-        <v>0.24063</v>
+        <v>0.24118</v>
       </c>
       <c r="P56" s="8" t="n">
-        <v>0.05535</v>
+        <v>0.05543</v>
       </c>
       <c r="Q56" s="8" t="n">
-        <v>0.02812</v>
+        <v>0.02813</v>
       </c>
       <c r="R56" s="8" t="n">
-        <v>0.14159</v>
+        <v>0.1414</v>
       </c>
       <c r="S56" s="8" t="n">
-        <v>0.04116</v>
+        <v>0.04109</v>
       </c>
       <c r="T56" s="8" t="n">
         <v>0.00299</v>
       </c>
       <c r="U56" s="8" t="n">
-        <v>3.50438</v>
+        <v>3.49972</v>
       </c>
     </row>
     <row r="57">
@@ -4965,7 +4965,7 @@
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>175.1</v>
+        <v>175.4</v>
       </c>
       <c r="E57" s="6">
         <f>D57*N57</f>
@@ -5004,28 +5004,28 @@
         <v/>
       </c>
       <c r="N57" s="8" t="n">
-        <v>4.086</v>
+        <v>4.085</v>
       </c>
       <c r="O57" s="8" t="n">
-        <v>0.24363</v>
+        <v>0.24419</v>
       </c>
       <c r="P57" s="8" t="n">
-        <v>0.0655</v>
+        <v>0.06559</v>
       </c>
       <c r="Q57" s="8" t="n">
-        <v>0.02302</v>
+        <v>0.02303</v>
       </c>
       <c r="R57" s="8" t="n">
-        <v>0.15105</v>
+        <v>0.15085</v>
       </c>
       <c r="S57" s="8" t="n">
-        <v>0.03475</v>
+        <v>0.03469</v>
       </c>
       <c r="T57" s="8" t="n">
         <v>0.00296</v>
       </c>
       <c r="U57" s="8" t="n">
-        <v>3.37647</v>
+        <v>3.37174</v>
       </c>
     </row>
     <row r="58">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>174.2</v>
+        <v>174.4</v>
       </c>
       <c r="E58" s="6">
         <f>D58*N58</f>
@@ -5084,28 +5084,28 @@
         <v/>
       </c>
       <c r="N58" s="8" t="n">
-        <v>4.129</v>
+        <v>4.128</v>
       </c>
       <c r="O58" s="8" t="n">
-        <v>0.22156</v>
+        <v>0.22209</v>
       </c>
       <c r="P58" s="8" t="n">
-        <v>0.04808</v>
+        <v>0.04815</v>
       </c>
       <c r="Q58" s="8" t="n">
-        <v>0.02647</v>
+        <v>0.02649</v>
       </c>
       <c r="R58" s="8" t="n">
-        <v>0.16381</v>
+        <v>0.16361</v>
       </c>
       <c r="S58" s="8" t="n">
-        <v>0.04377</v>
+        <v>0.0437</v>
       </c>
       <c r="T58" s="8" t="n">
         <v>0.00373</v>
       </c>
       <c r="U58" s="8" t="n">
-        <v>3.87471</v>
+        <v>3.86991</v>
       </c>
     </row>
     <row r="59">
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="D59" s="5" t="n">
-        <v>173.6</v>
+        <v>174</v>
       </c>
       <c r="E59" s="6">
         <f>D59*N59</f>
@@ -5164,28 +5164,28 @@
         <v/>
       </c>
       <c r="N59" s="8" t="n">
-        <v>4.215</v>
+        <v>4.214</v>
       </c>
       <c r="O59" s="8" t="n">
-        <v>0.24946</v>
+        <v>0.25001</v>
       </c>
       <c r="P59" s="8" t="n">
-        <v>0.07217999999999999</v>
+        <v>0.07227</v>
       </c>
       <c r="Q59" s="8" t="n">
-        <v>0.02475</v>
+        <v>0.02476</v>
       </c>
       <c r="R59" s="8" t="n">
-        <v>0.15119</v>
+        <v>0.15097</v>
       </c>
       <c r="S59" s="8" t="n">
-        <v>0.033</v>
+        <v>0.03293</v>
       </c>
       <c r="T59" s="8" t="n">
         <v>0.00382</v>
       </c>
       <c r="U59" s="8" t="n">
-        <v>3.78873</v>
+        <v>3.78379</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild 2027 projections (run 36911591832)
Verification PASSED.

Regenerated by .github/workflows/refresh-projections.yml.
Verification and the full baseline audit are in the run summary:
https://github.com/pmammino/DFSSimsFull/actions/runs/36911591832
</commit_message>
<xml_diff>
--- a/out/mlb_2027_what_if.xlsx
+++ b/out/mlb_2027_what_if.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="What-If" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What-If" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -713,37 +713,37 @@
         <v/>
       </c>
       <c r="P6" s="8" t="n">
-        <v>0.11537</v>
+        <v>0.11544</v>
       </c>
       <c r="Q6" s="8" t="n">
-        <v>0.04621</v>
+        <v>0.04624</v>
       </c>
       <c r="R6" s="8" t="n">
         <v>0.00263</v>
       </c>
       <c r="S6" s="8" t="n">
-        <v>0.05012</v>
+        <v>0.05014</v>
       </c>
       <c r="T6" s="8" t="n">
-        <v>0.11085</v>
+        <v>0.11081</v>
       </c>
       <c r="U6" s="8" t="n">
-        <v>0.008449999999999999</v>
+        <v>0.00844</v>
       </c>
       <c r="V6" s="8" t="n">
         <v>0.00606</v>
       </c>
       <c r="W6" s="8" t="n">
-        <v>0.24022</v>
+        <v>0.23989</v>
       </c>
       <c r="X6" s="8" t="n">
         <v>0.00351</v>
       </c>
       <c r="Y6" s="8" t="n">
-        <v>0.1308769126670375</v>
+        <v>0.1309504323723553</v>
       </c>
       <c r="Z6" s="8" t="n">
-        <v>0.1393581231932715</v>
+        <v>0.1394319334900104</v>
       </c>
     </row>
     <row r="7">
@@ -810,37 +810,37 @@
         <v/>
       </c>
       <c r="P7" s="8" t="n">
-        <v>0.1126</v>
+        <v>0.11268</v>
       </c>
       <c r="Q7" s="8" t="n">
-        <v>0.05129</v>
+        <v>0.05133</v>
       </c>
       <c r="R7" s="8" t="n">
         <v>0.0034</v>
       </c>
       <c r="S7" s="8" t="n">
-        <v>0.04689</v>
+        <v>0.04691</v>
       </c>
       <c r="T7" s="8" t="n">
-        <v>0.07511</v>
+        <v>0.07509</v>
       </c>
       <c r="U7" s="8" t="n">
-        <v>0.02598</v>
+        <v>0.02595</v>
       </c>
       <c r="V7" s="8" t="n">
         <v>0.00368</v>
       </c>
       <c r="W7" s="8" t="n">
-        <v>0.27347</v>
+        <v>0.27311</v>
       </c>
       <c r="X7" s="8" t="n">
         <v>0.03728</v>
       </c>
       <c r="Y7" s="8" t="n">
-        <v>0.1305117658570737</v>
+        <v>0.1305842564423994</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>0.1111451414894136</v>
+        <v>0.111207237744495</v>
       </c>
     </row>
     <row r="8">
@@ -907,37 +907,37 @@
         <v/>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0.11974</v>
+        <v>0.11984</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>0.04585</v>
+        <v>0.04589</v>
       </c>
       <c r="R8" s="8" t="n">
         <v>0.00315</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>0.04506</v>
+        <v>0.04509</v>
       </c>
       <c r="T8" s="8" t="n">
-        <v>0.13211</v>
+        <v>0.13208</v>
       </c>
       <c r="U8" s="8" t="n">
-        <v>0.00555</v>
+        <v>0.00554</v>
       </c>
       <c r="V8" s="8" t="n">
         <v>0.00426</v>
       </c>
       <c r="W8" s="8" t="n">
-        <v>0.30163</v>
+        <v>0.30125</v>
       </c>
       <c r="X8" s="8" t="n">
         <v>0.02916</v>
       </c>
       <c r="Y8" s="8" t="n">
-        <v>0.1313272711072163</v>
+        <v>0.1313971805106357</v>
       </c>
       <c r="Z8" s="8" t="n">
-        <v>0.1188429397064025</v>
+        <v>0.1189029015166095</v>
       </c>
     </row>
     <row r="9">
@@ -1004,37 +1004,37 @@
         <v/>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0.17317</v>
+        <v>0.17324</v>
       </c>
       <c r="Q9" s="8" t="n">
-        <v>0.04147</v>
+        <v>0.04149</v>
       </c>
       <c r="R9" s="8" t="n">
         <v>0.00515</v>
       </c>
       <c r="S9" s="8" t="n">
-        <v>0.02081</v>
+        <v>0.02082</v>
       </c>
       <c r="T9" s="8" t="n">
-        <v>0.06368</v>
+        <v>0.06364</v>
       </c>
       <c r="U9" s="8" t="n">
-        <v>0.00747</v>
+        <v>0.00746</v>
       </c>
       <c r="V9" s="8" t="n">
         <v>0.008970000000000001</v>
       </c>
       <c r="W9" s="8" t="n">
-        <v>0.1508</v>
+        <v>0.15055</v>
       </c>
       <c r="X9" s="8" t="n">
         <v>0.03639</v>
       </c>
       <c r="Y9" s="8" t="n">
-        <v>0.1158223452146403</v>
+        <v>0.1158800774371023</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>0.1036565318325018</v>
+        <v>0.1037046854426036</v>
       </c>
     </row>
     <row r="10">
@@ -1101,37 +1101,37 @@
         <v/>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0.11332</v>
+        <v>0.11341</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>0.04214</v>
+        <v>0.04217</v>
       </c>
       <c r="R10" s="8" t="n">
         <v>0.00305</v>
       </c>
       <c r="S10" s="8" t="n">
-        <v>0.04043</v>
+        <v>0.04045</v>
       </c>
       <c r="T10" s="8" t="n">
-        <v>0.09598</v>
+        <v>0.09594</v>
       </c>
       <c r="U10" s="8" t="n">
-        <v>0.00479</v>
+        <v>0.00478</v>
       </c>
       <c r="V10" s="8" t="n">
         <v>0.00715</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>0.26658</v>
+        <v>0.26622</v>
       </c>
       <c r="X10" s="8" t="n">
         <v>0.01709</v>
       </c>
       <c r="Y10" s="8" t="n">
-        <v>0.1223463927772788</v>
+        <v>0.1224196202016904</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>0.1243483529363782</v>
+        <v>0.1244117867432792</v>
       </c>
     </row>
     <row r="11">
@@ -1198,37 +1198,37 @@
         <v/>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0.14392</v>
+        <v>0.144</v>
       </c>
       <c r="Q11" s="8" t="n">
-        <v>0.04788</v>
+        <v>0.04791</v>
       </c>
       <c r="R11" s="8" t="n">
-        <v>0.01377</v>
+        <v>0.01378</v>
       </c>
       <c r="S11" s="8" t="n">
-        <v>0.03031</v>
+        <v>0.03032</v>
       </c>
       <c r="T11" s="8" t="n">
-        <v>0.06191</v>
+        <v>0.06187</v>
       </c>
       <c r="U11" s="8" t="n">
-        <v>0.009730000000000001</v>
+        <v>0.00971</v>
       </c>
       <c r="V11" s="8" t="n">
-        <v>0.0095</v>
+        <v>0.00949</v>
       </c>
       <c r="W11" s="8" t="n">
-        <v>0.19195</v>
+        <v>0.19166</v>
       </c>
       <c r="X11" s="8" t="n">
         <v>0.02656</v>
       </c>
       <c r="Y11" s="8" t="n">
-        <v>0.1160796094358666</v>
+        <v>0.1161494229705327</v>
       </c>
       <c r="Z11" s="8" t="n">
-        <v>0.1136814335225088</v>
+        <v>0.1137314937813254</v>
       </c>
     </row>
     <row r="12">
@@ -1295,37 +1295,37 @@
         <v/>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0.13311</v>
+        <v>0.13319</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>0.04477</v>
+        <v>0.04479</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>0.00755</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>0.03719</v>
+        <v>0.0372</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>0.06408999999999999</v>
+        <v>0.06406000000000001</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>0.02178</v>
+        <v>0.02176</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>0.00628</v>
       </c>
       <c r="W12" s="8" t="n">
-        <v>0.21601</v>
+        <v>0.2157</v>
       </c>
       <c r="X12" s="8" t="n">
         <v>0.04791</v>
       </c>
       <c r="Y12" s="8" t="n">
-        <v>0.13018246285228</v>
+        <v>0.1302523650577866</v>
       </c>
       <c r="Z12" s="8" t="n">
-        <v>0.1108095438484876</v>
+        <v>0.1108793242479339</v>
       </c>
     </row>
     <row r="13">
@@ -1392,37 +1392,37 @@
         <v/>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0.12874</v>
+        <v>0.12882</v>
       </c>
       <c r="Q13" s="8" t="n">
-        <v>0.04532</v>
+        <v>0.04535</v>
       </c>
       <c r="R13" s="8" t="n">
         <v>0.00096</v>
       </c>
       <c r="S13" s="8" t="n">
-        <v>0.0581</v>
+        <v>0.05813</v>
       </c>
       <c r="T13" s="8" t="n">
-        <v>0.0977</v>
+        <v>0.09767000000000001</v>
       </c>
       <c r="U13" s="8" t="n">
-        <v>0.0203</v>
+        <v>0.02029</v>
       </c>
       <c r="V13" s="8" t="n">
         <v>0.00874</v>
       </c>
       <c r="W13" s="8" t="n">
-        <v>0.23516</v>
+        <v>0.23484</v>
       </c>
       <c r="X13" s="8" t="n">
         <v>0.00442</v>
       </c>
       <c r="Y13" s="8" t="n">
-        <v>0.1231541199933732</v>
+        <v>0.1232192330356799</v>
       </c>
       <c r="Z13" s="8" t="n">
-        <v>0.1485172170670946</v>
+        <v>0.1486032832854011</v>
       </c>
     </row>
     <row r="14">
@@ -1489,10 +1489,10 @@
         <v/>
       </c>
       <c r="P14" s="8" t="n">
-        <v>0.14558</v>
+        <v>0.14566</v>
       </c>
       <c r="Q14" s="8" t="n">
-        <v>0.04702</v>
+        <v>0.04705</v>
       </c>
       <c r="R14" s="8" t="n">
         <v>0.00604</v>
@@ -1501,25 +1501,25 @@
         <v>0.02935</v>
       </c>
       <c r="T14" s="8" t="n">
-        <v>0.09539</v>
+        <v>0.09536</v>
       </c>
       <c r="U14" s="8" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.00929</v>
       </c>
       <c r="V14" s="8" t="n">
-        <v>0.0049</v>
+        <v>0.00489</v>
       </c>
       <c r="W14" s="8" t="n">
-        <v>0.23092</v>
+        <v>0.23061</v>
       </c>
       <c r="X14" s="8" t="n">
         <v>0.02686</v>
       </c>
       <c r="Y14" s="8" t="n">
-        <v>0.1291248101605333</v>
+        <v>0.1292099478496693</v>
       </c>
       <c r="Z14" s="8" t="n">
-        <v>0.1021530808599572</v>
+        <v>0.1022073189681618</v>
       </c>
     </row>
     <row r="15">
@@ -1586,10 +1586,10 @@
         <v/>
       </c>
       <c r="P15" s="8" t="n">
-        <v>0.1589</v>
+        <v>0.15897</v>
       </c>
       <c r="Q15" s="8" t="n">
-        <v>0.04706</v>
+        <v>0.04708</v>
       </c>
       <c r="R15" s="8" t="n">
         <v>0.00192</v>
@@ -1598,25 +1598,25 @@
         <v>0.03972</v>
       </c>
       <c r="T15" s="8" t="n">
-        <v>0.07133</v>
+        <v>0.07129000000000001</v>
       </c>
       <c r="U15" s="8" t="n">
         <v>0.00715</v>
       </c>
       <c r="V15" s="8" t="n">
-        <v>0.00707</v>
+        <v>0.00706</v>
       </c>
       <c r="W15" s="8" t="n">
-        <v>0.16073</v>
+        <v>0.16048</v>
       </c>
       <c r="X15" s="8" t="n">
         <v>0.008869999999999999</v>
       </c>
       <c r="Y15" s="8" t="n">
-        <v>0.1078632243978509</v>
+        <v>0.1079168715572707</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>0.1280366537069566</v>
+        <v>0.1281085555872521</v>
       </c>
     </row>
     <row r="16">
@@ -1683,37 +1683,37 @@
         <v/>
       </c>
       <c r="P16" s="8" t="n">
-        <v>0.11156</v>
+        <v>0.11165</v>
       </c>
       <c r="Q16" s="8" t="n">
-        <v>0.03634</v>
+        <v>0.03637</v>
       </c>
       <c r="R16" s="8" t="n">
-        <v>0.00316</v>
+        <v>0.00315</v>
       </c>
       <c r="S16" s="8" t="n">
-        <v>0.04592</v>
+        <v>0.04595</v>
       </c>
       <c r="T16" s="8" t="n">
-        <v>0.14033</v>
+        <v>0.14029</v>
       </c>
       <c r="U16" s="8" t="n">
         <v>0.01368</v>
       </c>
       <c r="V16" s="8" t="n">
-        <v>0.00501</v>
+        <v>0.005</v>
       </c>
       <c r="W16" s="8" t="n">
-        <v>0.28351</v>
+        <v>0.28316</v>
       </c>
       <c r="X16" s="8" t="n">
         <v>0.0123</v>
       </c>
       <c r="Y16" s="8" t="n">
-        <v>0.1349953874482333</v>
+        <v>0.1350774781694497</v>
       </c>
       <c r="Z16" s="8" t="n">
-        <v>0.1084119107908361</v>
+        <v>0.1084738611938727</v>
       </c>
     </row>
     <row r="17">
@@ -1780,37 +1780,37 @@
         <v/>
       </c>
       <c r="P17" s="8" t="n">
-        <v>0.1378</v>
+        <v>0.13788</v>
       </c>
       <c r="Q17" s="8" t="n">
-        <v>0.04265</v>
+        <v>0.04268</v>
       </c>
       <c r="R17" s="8" t="n">
         <v>0.0013</v>
       </c>
       <c r="S17" s="8" t="n">
-        <v>0.05433</v>
+        <v>0.05434</v>
       </c>
       <c r="T17" s="8" t="n">
-        <v>0.08529</v>
+        <v>0.08524</v>
       </c>
       <c r="U17" s="8" t="n">
-        <v>0.00524</v>
+        <v>0.00523</v>
       </c>
       <c r="V17" s="8" t="n">
         <v>0.00626</v>
       </c>
       <c r="W17" s="8" t="n">
-        <v>0.19729</v>
+        <v>0.197</v>
       </c>
       <c r="X17" s="8" t="n">
         <v>0.009010000000000001</v>
       </c>
       <c r="Y17" s="8" t="n">
-        <v>0.1253299002189532</v>
+        <v>0.1253889592414694</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>0.1358544477204062</v>
+        <v>0.1359224420856639</v>
       </c>
     </row>
     <row r="18">
@@ -1877,37 +1877,37 @@
         <v/>
       </c>
       <c r="P18" s="8" t="n">
-        <v>0.13669</v>
+        <v>0.13678</v>
       </c>
       <c r="Q18" s="8" t="n">
-        <v>0.04439</v>
+        <v>0.04442</v>
       </c>
       <c r="R18" s="8" t="n">
         <v>0.00356</v>
       </c>
       <c r="S18" s="8" t="n">
-        <v>0.03161</v>
+        <v>0.03162</v>
       </c>
       <c r="T18" s="8" t="n">
-        <v>0.0728</v>
+        <v>0.07277</v>
       </c>
       <c r="U18" s="8" t="n">
-        <v>0.00861</v>
+        <v>0.0086</v>
       </c>
       <c r="V18" s="8" t="n">
-        <v>0.00523</v>
+        <v>0.00522</v>
       </c>
       <c r="W18" s="8" t="n">
-        <v>0.27099</v>
+        <v>0.27063</v>
       </c>
       <c r="X18" s="8" t="n">
         <v>0.02463</v>
       </c>
       <c r="Y18" s="8" t="n">
-        <v>0.1126209319600726</v>
+        <v>0.1126744668667469</v>
       </c>
       <c r="Z18" s="8" t="n">
-        <v>0.1168916300867914</v>
+        <v>0.1169544295762559</v>
       </c>
     </row>
     <row r="19">
@@ -1974,37 +1974,37 @@
         <v/>
       </c>
       <c r="P19" s="8" t="n">
-        <v>0.1381</v>
+        <v>0.13819</v>
       </c>
       <c r="Q19" s="8" t="n">
-        <v>0.04941</v>
+        <v>0.04945</v>
       </c>
       <c r="R19" s="8" t="n">
         <v>0.00573</v>
       </c>
       <c r="S19" s="8" t="n">
-        <v>0.03478</v>
+        <v>0.03479</v>
       </c>
       <c r="T19" s="8" t="n">
-        <v>0.0946</v>
+        <v>0.09456000000000001</v>
       </c>
       <c r="U19" s="8" t="n">
-        <v>0.0143</v>
+        <v>0.01429</v>
       </c>
       <c r="V19" s="8" t="n">
-        <v>0.00508</v>
+        <v>0.00507</v>
       </c>
       <c r="W19" s="8" t="n">
-        <v>0.23985</v>
+        <v>0.23952</v>
       </c>
       <c r="X19" s="8" t="n">
         <v>0.01286</v>
       </c>
       <c r="Y19" s="8" t="n">
-        <v>0.122874300413643</v>
+        <v>0.1229411148850544</v>
       </c>
       <c r="Z19" s="8" t="n">
-        <v>0.1156687087227195</v>
+        <v>0.1157447515711056</v>
       </c>
     </row>
     <row r="20">
@@ -2071,37 +2071,37 @@
         <v/>
       </c>
       <c r="P20" s="8" t="n">
-        <v>0.18561</v>
+        <v>0.18568</v>
       </c>
       <c r="Q20" s="8" t="n">
-        <v>0.0312</v>
+        <v>0.03121</v>
       </c>
       <c r="R20" s="8" t="n">
-        <v>0.00534</v>
+        <v>0.00535</v>
       </c>
       <c r="S20" s="8" t="n">
         <v>0.00733</v>
       </c>
       <c r="T20" s="8" t="n">
-        <v>0.09424</v>
+        <v>0.09419</v>
       </c>
       <c r="U20" s="8" t="n">
-        <v>0.00283</v>
+        <v>0.00282</v>
       </c>
       <c r="V20" s="8" t="n">
         <v>0.007889999999999999</v>
       </c>
       <c r="W20" s="8" t="n">
-        <v>0.15633</v>
+        <v>0.15608</v>
       </c>
       <c r="X20" s="8" t="n">
         <v>0.04288</v>
       </c>
       <c r="Y20" s="8" t="n">
-        <v>0.1095303386060655</v>
+        <v>0.1095880325500156</v>
       </c>
       <c r="Z20" s="8" t="n">
-        <v>0.0787166143991179</v>
+        <v>0.078755111683385</v>
       </c>
     </row>
     <row r="21">
@@ -2168,37 +2168,37 @@
         <v/>
       </c>
       <c r="P21" s="8" t="n">
-        <v>0.18448</v>
+        <v>0.18455</v>
       </c>
       <c r="Q21" s="8" t="n">
-        <v>0.04554</v>
+        <v>0.04557</v>
       </c>
       <c r="R21" s="8" t="n">
         <v>0.00671</v>
       </c>
       <c r="S21" s="8" t="n">
-        <v>0.01457</v>
+        <v>0.01458</v>
       </c>
       <c r="T21" s="8" t="n">
-        <v>0.06319</v>
+        <v>0.06315</v>
       </c>
       <c r="U21" s="8" t="n">
-        <v>0.01009</v>
+        <v>0.01008</v>
       </c>
       <c r="V21" s="8" t="n">
-        <v>0.00721</v>
+        <v>0.0072</v>
       </c>
       <c r="W21" s="8" t="n">
-        <v>0.1175</v>
+        <v>0.1173</v>
       </c>
       <c r="X21" s="8" t="n">
         <v>0.01942</v>
       </c>
       <c r="Y21" s="8" t="n">
-        <v>0.1132438842706345</v>
+        <v>0.1133069376055121</v>
       </c>
       <c r="Z21" s="8" t="n">
-        <v>0.0931355258252959</v>
+        <v>0.09319789018818769</v>
       </c>
     </row>
     <row r="22">
@@ -2265,37 +2265,37 @@
         <v/>
       </c>
       <c r="P22" s="8" t="n">
-        <v>0.14454</v>
+        <v>0.14463</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>0.03965</v>
+        <v>0.03967</v>
       </c>
       <c r="R22" s="8" t="n">
         <v>0.00765</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>0.0177</v>
+        <v>0.01771</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>0.11189</v>
+        <v>0.11184</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>0.01865</v>
+        <v>0.01864</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>0.00268</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>0.212</v>
+        <v>0.21169</v>
       </c>
       <c r="X22" s="8" t="n">
         <v>0.04402</v>
       </c>
       <c r="Y22" s="8" t="n">
-        <v>0.1189968621440421</v>
+        <v>0.119064118278755</v>
       </c>
       <c r="Z22" s="8" t="n">
-        <v>0.08450488029733851</v>
+        <v>0.084552917395051</v>
       </c>
     </row>
     <row r="23">
@@ -2362,37 +2362,37 @@
         <v/>
       </c>
       <c r="P23" s="8" t="n">
-        <v>0.177</v>
+        <v>0.17709</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>0.03647</v>
+        <v>0.03649</v>
       </c>
       <c r="R23" s="8" t="n">
         <v>0.00173</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>0.02961</v>
+        <v>0.02962</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>0.09182999999999999</v>
+        <v>0.09177</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>0.0106</v>
+        <v>0.01059</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>0.00569</v>
+        <v>0.00568</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>0.14975</v>
+        <v>0.14952</v>
       </c>
       <c r="X23" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="Y23" s="8" t="n">
-        <v>0.1165803451467095</v>
+        <v>0.1166303489644285</v>
       </c>
       <c r="Z23" s="8" t="n">
-        <v>0.1116122956845203</v>
+        <v>0.1116529889391498</v>
       </c>
     </row>
     <row r="24">
@@ -2459,37 +2459,37 @@
         <v/>
       </c>
       <c r="P24" s="8" t="n">
-        <v>0.11644</v>
+        <v>0.11652</v>
       </c>
       <c r="Q24" s="8" t="n">
-        <v>0.04929</v>
+        <v>0.04933</v>
       </c>
       <c r="R24" s="8" t="n">
         <v>0.00157</v>
       </c>
       <c r="S24" s="8" t="n">
-        <v>0.04716</v>
+        <v>0.04717</v>
       </c>
       <c r="T24" s="8" t="n">
-        <v>0.10926</v>
+        <v>0.10922</v>
       </c>
       <c r="U24" s="8" t="n">
-        <v>0.00669</v>
+        <v>0.00668</v>
       </c>
       <c r="V24" s="8" t="n">
-        <v>0.00666</v>
+        <v>0.00665</v>
       </c>
       <c r="W24" s="8" t="n">
-        <v>0.24737</v>
+        <v>0.24703</v>
       </c>
       <c r="X24" s="8" t="n">
         <v>0.00144</v>
       </c>
       <c r="Y24" s="8" t="n">
-        <v>0.1267743118205152</v>
+        <v>0.1268448235725187</v>
       </c>
       <c r="Z24" s="8" t="n">
-        <v>0.13323747662287</v>
+        <v>0.1333181705119431</v>
       </c>
     </row>
     <row r="25">
@@ -2556,37 +2556,37 @@
         <v/>
       </c>
       <c r="P25" s="8" t="n">
-        <v>0.11348</v>
+        <v>0.11356</v>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>0.04867</v>
+        <v>0.04871</v>
       </c>
       <c r="R25" s="8" t="n">
         <v>0.00231</v>
       </c>
       <c r="S25" s="8" t="n">
-        <v>0.04956</v>
+        <v>0.04958</v>
       </c>
       <c r="T25" s="8" t="n">
-        <v>0.09097</v>
+        <v>0.09095</v>
       </c>
       <c r="U25" s="8" t="n">
         <v>0.0107</v>
       </c>
       <c r="V25" s="8" t="n">
-        <v>0.00568</v>
+        <v>0.00567</v>
       </c>
       <c r="W25" s="8" t="n">
-        <v>0.27779</v>
+        <v>0.27742</v>
       </c>
       <c r="X25" s="8" t="n">
         <v>0.01097</v>
       </c>
       <c r="Y25" s="8" t="n">
-        <v>0.127395410324242</v>
+        <v>0.1274595313651934</v>
       </c>
       <c r="Z25" s="8" t="n">
-        <v>0.1468158701062275</v>
+        <v>0.1469006423682971</v>
       </c>
     </row>
     <row r="26">
@@ -2653,53 +2653,53 @@
         <v/>
       </c>
       <c r="P26" s="8" t="n">
-        <v>0.14129</v>
+        <v>0.14138</v>
       </c>
       <c r="Q26" s="8" t="n">
-        <v>0.04339</v>
+        <v>0.04341</v>
       </c>
       <c r="R26" s="8" t="n">
-        <v>0.009140000000000001</v>
+        <v>0.00915</v>
       </c>
       <c r="S26" s="8" t="n">
-        <v>0.02751</v>
+        <v>0.02753</v>
       </c>
       <c r="T26" s="8" t="n">
-        <v>0.07277</v>
+        <v>0.07275</v>
       </c>
       <c r="U26" s="8" t="n">
         <v>0.01141</v>
       </c>
       <c r="V26" s="8" t="n">
-        <v>0.00598</v>
+        <v>0.00597</v>
       </c>
       <c r="W26" s="8" t="n">
-        <v>0.25176</v>
+        <v>0.2514</v>
       </c>
       <c r="X26" s="8" t="n">
         <v>0.0397</v>
       </c>
       <c r="Y26" s="8" t="n">
-        <v>0.115240493757318</v>
+        <v>0.1152966838962423</v>
       </c>
       <c r="Z26" s="8" t="n">
-        <v>0.1025389914503331</v>
+        <v>0.1025944232805242</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Everyday DH / 1B-DH</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
@@ -2750,53 +2750,53 @@
         <v/>
       </c>
       <c r="P27" s="8" t="n">
-        <v>0.14576</v>
+        <v>0.13896</v>
       </c>
       <c r="Q27" s="8" t="n">
-        <v>0.04292</v>
+        <v>0.04324</v>
       </c>
       <c r="R27" s="8" t="n">
-        <v>0.00178</v>
+        <v>0.007889999999999999</v>
       </c>
       <c r="S27" s="8" t="n">
-        <v>0.03655</v>
+        <v>0.02951</v>
       </c>
       <c r="T27" s="8" t="n">
-        <v>0.09699000000000001</v>
+        <v>0.12461</v>
       </c>
       <c r="U27" s="8" t="n">
-        <v>0.01604</v>
+        <v>0.0048</v>
       </c>
       <c r="V27" s="8" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.00566</v>
       </c>
       <c r="W27" s="8" t="n">
-        <v>0.25213</v>
+        <v>0.15674</v>
       </c>
       <c r="X27" s="8" t="n">
-        <v>0.00285</v>
+        <v>0.01801</v>
       </c>
       <c r="Y27" s="8" t="n">
-        <v>0.113020713590306</v>
+        <v>0.1298104529584322</v>
       </c>
       <c r="Z27" s="8" t="n">
-        <v>0.1200724498172191</v>
+        <v>0.1025692821317952</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Full Time</t>
+          <t>Everyday DH / 1B-DH</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
@@ -2847,37 +2847,37 @@
         <v/>
       </c>
       <c r="P28" s="8" t="n">
-        <v>0.1389</v>
+        <v>0.14586</v>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>0.04321</v>
+        <v>0.04295</v>
       </c>
       <c r="R28" s="8" t="n">
-        <v>0.007889999999999999</v>
+        <v>0.00178</v>
       </c>
       <c r="S28" s="8" t="n">
-        <v>0.0295</v>
+        <v>0.03656</v>
       </c>
       <c r="T28" s="8" t="n">
-        <v>0.12468</v>
+        <v>0.09694999999999999</v>
       </c>
       <c r="U28" s="8" t="n">
-        <v>0.00481</v>
+        <v>0.01603</v>
       </c>
       <c r="V28" s="8" t="n">
-        <v>0.00567</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="W28" s="8" t="n">
-        <v>0.15699</v>
+        <v>0.25179</v>
       </c>
       <c r="X28" s="8" t="n">
-        <v>0.01801</v>
+        <v>0.00285</v>
       </c>
       <c r="Y28" s="8" t="n">
-        <v>0.1297388573590071</v>
+        <v>0.1130709577835606</v>
       </c>
       <c r="Z28" s="8" t="n">
-        <v>0.1025079654509587</v>
+        <v>0.1201222178193721</v>
       </c>
     </row>
     <row r="29">
@@ -2944,37 +2944,37 @@
         <v/>
       </c>
       <c r="P29" s="8" t="n">
-        <v>0.09565</v>
+        <v>0.09573</v>
       </c>
       <c r="Q29" s="8" t="n">
-        <v>0.03733</v>
+        <v>0.03736</v>
       </c>
       <c r="R29" s="8" t="n">
         <v>0.00154</v>
       </c>
       <c r="S29" s="8" t="n">
-        <v>0.06146</v>
+        <v>0.06149</v>
       </c>
       <c r="T29" s="8" t="n">
-        <v>0.14532</v>
+        <v>0.14529</v>
       </c>
       <c r="U29" s="8" t="n">
-        <v>0.00942</v>
+        <v>0.00941</v>
       </c>
       <c r="V29" s="8" t="n">
-        <v>0.0056</v>
+        <v>0.00559</v>
       </c>
       <c r="W29" s="8" t="n">
-        <v>0.29725</v>
+        <v>0.29689</v>
       </c>
       <c r="X29" s="8" t="n">
         <v>0.00756</v>
       </c>
       <c r="Y29" s="8" t="n">
-        <v>0.1374788380219203</v>
+        <v>0.1375454863523067</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>0.1403508871636152</v>
+        <v>0.1404276848359009</v>
       </c>
     </row>
     <row r="30">
@@ -3041,37 +3041,37 @@
         <v/>
       </c>
       <c r="P30" s="8" t="n">
-        <v>0.11346</v>
+        <v>0.11354</v>
       </c>
       <c r="Q30" s="8" t="n">
-        <v>0.04915</v>
+        <v>0.04918</v>
       </c>
       <c r="R30" s="8" t="n">
         <v>0.0066</v>
       </c>
       <c r="S30" s="8" t="n">
-        <v>0.0645</v>
+        <v>0.06453</v>
       </c>
       <c r="T30" s="8" t="n">
-        <v>0.12629</v>
+        <v>0.12625</v>
       </c>
       <c r="U30" s="8" t="n">
         <v>0.00705</v>
       </c>
       <c r="V30" s="8" t="n">
-        <v>0.00531</v>
+        <v>0.0053</v>
       </c>
       <c r="W30" s="8" t="n">
-        <v>0.24667</v>
+        <v>0.24633</v>
       </c>
       <c r="X30" s="8" t="n">
         <v>0.03207</v>
       </c>
       <c r="Y30" s="8" t="n">
-        <v>0.1657200911231141</v>
+        <v>0.165795015544466</v>
       </c>
       <c r="Z30" s="8" t="n">
-        <v>0.1477317382817687</v>
+        <v>0.1478070775708195</v>
       </c>
     </row>
     <row r="33">
@@ -3244,28 +3244,28 @@
         <v/>
       </c>
       <c r="N35" s="8" t="n">
-        <v>4.177</v>
+        <v>4.176</v>
       </c>
       <c r="O35" s="8" t="n">
-        <v>0.21648</v>
+        <v>0.217</v>
       </c>
       <c r="P35" s="8" t="n">
-        <v>0.05744</v>
+        <v>0.05752</v>
       </c>
       <c r="Q35" s="8" t="n">
-        <v>0.02102</v>
+        <v>0.02104</v>
       </c>
       <c r="R35" s="8" t="n">
-        <v>0.17117</v>
+        <v>0.17097</v>
       </c>
       <c r="S35" s="8" t="n">
-        <v>0.03998</v>
+        <v>0.03992</v>
       </c>
       <c r="T35" s="8" t="n">
-        <v>0.00498</v>
+        <v>0.00497</v>
       </c>
       <c r="U35" s="8" t="n">
-        <v>3.81176</v>
+        <v>3.80698</v>
       </c>
     </row>
     <row r="36">
@@ -3324,28 +3324,28 @@
         <v/>
       </c>
       <c r="N36" s="8" t="n">
-        <v>4.21</v>
+        <v>4.209</v>
       </c>
       <c r="O36" s="8" t="n">
-        <v>0.25368</v>
+        <v>0.25423</v>
       </c>
       <c r="P36" s="8" t="n">
-        <v>0.09253</v>
+        <v>0.09264</v>
       </c>
       <c r="Q36" s="8" t="n">
-        <v>0.02147</v>
+        <v>0.02148</v>
       </c>
       <c r="R36" s="8" t="n">
-        <v>0.13546</v>
+        <v>0.13526</v>
       </c>
       <c r="S36" s="8" t="n">
-        <v>0.03736</v>
+        <v>0.03729</v>
       </c>
       <c r="T36" s="8" t="n">
         <v>0.00316</v>
       </c>
       <c r="U36" s="8" t="n">
-        <v>3.61038</v>
+        <v>3.60625</v>
       </c>
     </row>
     <row r="37">
@@ -3404,28 +3404,28 @@
         <v/>
       </c>
       <c r="N37" s="8" t="n">
-        <v>4.224</v>
+        <v>4.223</v>
       </c>
       <c r="O37" s="8" t="n">
-        <v>0.18972</v>
+        <v>0.19018</v>
       </c>
       <c r="P37" s="8" t="n">
-        <v>0.06865</v>
+        <v>0.06875000000000001</v>
       </c>
       <c r="Q37" s="8" t="n">
-        <v>0.02671</v>
+        <v>0.02673</v>
       </c>
       <c r="R37" s="8" t="n">
-        <v>0.15467</v>
+        <v>0.15449</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>0.04585</v>
+        <v>0.04578</v>
       </c>
       <c r="T37" s="8" t="n">
-        <v>0.00441</v>
+        <v>0.0044</v>
       </c>
       <c r="U37" s="8" t="n">
-        <v>4.18097</v>
+        <v>4.17694</v>
       </c>
     </row>
     <row r="38">
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>212</v>
+        <v>212.7</v>
       </c>
       <c r="E38" s="6">
         <f>D38*N38</f>
@@ -3484,28 +3484,28 @@
         <v/>
       </c>
       <c r="N38" s="8" t="n">
-        <v>4.335</v>
+        <v>4.334</v>
       </c>
       <c r="O38" s="8" t="n">
-        <v>0.16211</v>
+        <v>0.16252</v>
       </c>
       <c r="P38" s="8" t="n">
-        <v>0.08626</v>
+        <v>0.08638999999999999</v>
       </c>
       <c r="Q38" s="8" t="n">
-        <v>0.02071</v>
+        <v>0.02073</v>
       </c>
       <c r="R38" s="8" t="n">
-        <v>0.17337</v>
+        <v>0.17318</v>
       </c>
       <c r="S38" s="8" t="n">
-        <v>0.03691</v>
+        <v>0.03686</v>
       </c>
       <c r="T38" s="8" t="n">
-        <v>0.00408</v>
+        <v>0.00407</v>
       </c>
       <c r="U38" s="8" t="n">
-        <v>4.21378</v>
+        <v>4.21019</v>
       </c>
     </row>
     <row r="39">
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>211.1</v>
+        <v>211.8</v>
       </c>
       <c r="E39" s="6">
         <f>D39*N39</f>
@@ -3567,25 +3567,25 @@
         <v>4.274</v>
       </c>
       <c r="O39" s="8" t="n">
-        <v>0.16461</v>
+        <v>0.16504</v>
       </c>
       <c r="P39" s="8" t="n">
-        <v>0.06444999999999999</v>
+        <v>0.06455</v>
       </c>
       <c r="Q39" s="8" t="n">
-        <v>0.03342</v>
+        <v>0.03345</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>0.16413</v>
+        <v>0.16396</v>
       </c>
       <c r="S39" s="8" t="n">
-        <v>0.04733</v>
+        <v>0.04726</v>
       </c>
       <c r="T39" s="8" t="n">
-        <v>0.0044</v>
+        <v>0.00439</v>
       </c>
       <c r="U39" s="8" t="n">
-        <v>4.67496</v>
+        <v>4.67108</v>
       </c>
     </row>
     <row r="40">
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>198.7</v>
+        <v>199</v>
       </c>
       <c r="E40" s="6">
         <f>D40*N40</f>
@@ -3647,25 +3647,25 @@
         <v>4.169</v>
       </c>
       <c r="O40" s="8" t="n">
-        <v>0.19438</v>
+        <v>0.19486</v>
       </c>
       <c r="P40" s="8" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.0687</v>
       </c>
       <c r="Q40" s="8" t="n">
-        <v>0.03149</v>
+        <v>0.03151</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>0.13926</v>
+        <v>0.1391</v>
       </c>
       <c r="S40" s="8" t="n">
-        <v>0.04866</v>
+        <v>0.04859</v>
       </c>
       <c r="T40" s="8" t="n">
-        <v>0.00604</v>
+        <v>0.00602</v>
       </c>
       <c r="U40" s="8" t="n">
-        <v>4.2136</v>
+        <v>4.20948</v>
       </c>
     </row>
     <row r="41">
@@ -3685,7 +3685,7 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>196.2</v>
+        <v>196.5</v>
       </c>
       <c r="E41" s="6">
         <f>D41*N41</f>
@@ -3724,28 +3724,28 @@
         <v/>
       </c>
       <c r="N41" s="8" t="n">
-        <v>4.009</v>
+        <v>4.008</v>
       </c>
       <c r="O41" s="8" t="n">
-        <v>0.28284</v>
+        <v>0.28344</v>
       </c>
       <c r="P41" s="8" t="n">
-        <v>0.06644</v>
+        <v>0.06651</v>
       </c>
       <c r="Q41" s="8" t="n">
-        <v>0.02328</v>
+        <v>0.0233</v>
       </c>
       <c r="R41" s="8" t="n">
-        <v>0.12982</v>
+        <v>0.12962</v>
       </c>
       <c r="S41" s="8" t="n">
-        <v>0.03786</v>
+        <v>0.03779</v>
       </c>
       <c r="T41" s="8" t="n">
         <v>0.00386</v>
       </c>
       <c r="U41" s="8" t="n">
-        <v>3.11165</v>
+        <v>3.10699</v>
       </c>
     </row>
     <row r="42">
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>195.7</v>
+        <v>195.8</v>
       </c>
       <c r="E42" s="6">
         <f>D42*N42</f>
@@ -3804,28 +3804,28 @@
         <v/>
       </c>
       <c r="N42" s="8" t="n">
-        <v>4.109</v>
+        <v>4.108</v>
       </c>
       <c r="O42" s="8" t="n">
-        <v>0.23924</v>
+        <v>0.2398</v>
       </c>
       <c r="P42" s="8" t="n">
-        <v>0.05788</v>
+        <v>0.05796</v>
       </c>
       <c r="Q42" s="8" t="n">
-        <v>0.02034</v>
+        <v>0.02036</v>
       </c>
       <c r="R42" s="8" t="n">
-        <v>0.16384</v>
+        <v>0.16363</v>
       </c>
       <c r="S42" s="8" t="n">
-        <v>0.03974</v>
+        <v>0.03968</v>
       </c>
       <c r="T42" s="8" t="n">
         <v>0.00258</v>
       </c>
       <c r="U42" s="8" t="n">
-        <v>3.47409</v>
+        <v>3.46961</v>
       </c>
     </row>
     <row r="43">
@@ -3845,7 +3845,7 @@
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>190.8</v>
+        <v>191.4</v>
       </c>
       <c r="E43" s="6">
         <f>D43*N43</f>
@@ -3884,28 +3884,28 @@
         <v/>
       </c>
       <c r="N43" s="8" t="n">
-        <v>4.133</v>
+        <v>4.132</v>
       </c>
       <c r="O43" s="8" t="n">
-        <v>0.2594</v>
+        <v>0.25996</v>
       </c>
       <c r="P43" s="8" t="n">
-        <v>0.09172</v>
+        <v>0.09182999999999999</v>
       </c>
       <c r="Q43" s="8" t="n">
-        <v>0.02049</v>
+        <v>0.0205</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>0.14158</v>
+        <v>0.14138</v>
       </c>
       <c r="S43" s="8" t="n">
-        <v>0.02824</v>
+        <v>0.02819</v>
       </c>
       <c r="T43" s="8" t="n">
         <v>0.00328</v>
       </c>
       <c r="U43" s="8" t="n">
-        <v>3.24041</v>
+        <v>3.23628</v>
       </c>
     </row>
     <row r="44">
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>189.6</v>
+        <v>190.1</v>
       </c>
       <c r="E44" s="6">
         <f>D44*N44</f>
@@ -3964,28 +3964,28 @@
         <v/>
       </c>
       <c r="N44" s="8" t="n">
-        <v>4.251</v>
+        <v>4.25</v>
       </c>
       <c r="O44" s="8" t="n">
-        <v>0.21665</v>
+        <v>0.21715</v>
       </c>
       <c r="P44" s="8" t="n">
-        <v>0.08314000000000001</v>
+        <v>0.08323999999999999</v>
       </c>
       <c r="Q44" s="8" t="n">
-        <v>0.0197</v>
+        <v>0.01972</v>
       </c>
       <c r="R44" s="8" t="n">
-        <v>0.15454</v>
+        <v>0.15434</v>
       </c>
       <c r="S44" s="8" t="n">
-        <v>0.04108</v>
+        <v>0.04101</v>
       </c>
       <c r="T44" s="8" t="n">
         <v>0.00366</v>
       </c>
       <c r="U44" s="8" t="n">
-        <v>3.85848</v>
+        <v>3.85389</v>
       </c>
     </row>
     <row r="45">
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>187.9</v>
+        <v>188.3</v>
       </c>
       <c r="E45" s="6">
         <f>D45*N45</f>
@@ -4044,28 +4044,28 @@
         <v/>
       </c>
       <c r="N45" s="8" t="n">
-        <v>4.34</v>
+        <v>4.339</v>
       </c>
       <c r="O45" s="8" t="n">
-        <v>0.1896</v>
+        <v>0.19004</v>
       </c>
       <c r="P45" s="8" t="n">
-        <v>0.08619</v>
+        <v>0.0863</v>
       </c>
       <c r="Q45" s="8" t="n">
-        <v>0.04325</v>
+        <v>0.04328</v>
       </c>
       <c r="R45" s="8" t="n">
-        <v>0.13977</v>
+        <v>0.13959</v>
       </c>
       <c r="S45" s="8" t="n">
-        <v>0.04412</v>
+        <v>0.04405</v>
       </c>
       <c r="T45" s="8" t="n">
         <v>0.00459</v>
       </c>
       <c r="U45" s="8" t="n">
-        <v>5.04469</v>
+        <v>5.04139</v>
       </c>
     </row>
     <row r="46">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>186.4</v>
+        <v>186.8</v>
       </c>
       <c r="E46" s="6">
         <f>D46*N46</f>
@@ -4124,28 +4124,28 @@
         <v/>
       </c>
       <c r="N46" s="8" t="n">
-        <v>4.05</v>
+        <v>4.049</v>
       </c>
       <c r="O46" s="8" t="n">
-        <v>0.29876</v>
+        <v>0.29938</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>0.0669</v>
+        <v>0.06698</v>
       </c>
       <c r="Q46" s="8" t="n">
-        <v>0.0294</v>
+        <v>0.02941</v>
       </c>
       <c r="R46" s="8" t="n">
-        <v>0.13364</v>
+        <v>0.13344</v>
       </c>
       <c r="S46" s="8" t="n">
-        <v>0.03966</v>
+        <v>0.03959</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0.00272</v>
       </c>
       <c r="U46" s="8" t="n">
-        <v>3.4427</v>
+        <v>3.43729</v>
       </c>
     </row>
     <row r="47">
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>184.9</v>
+        <v>185.4</v>
       </c>
       <c r="E47" s="6">
         <f>D47*N47</f>
@@ -4204,28 +4204,28 @@
         <v/>
       </c>
       <c r="N47" s="8" t="n">
-        <v>4.345</v>
+        <v>4.344</v>
       </c>
       <c r="O47" s="8" t="n">
-        <v>0.20476</v>
+        <v>0.20524</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>0.07475</v>
+        <v>0.07485</v>
       </c>
       <c r="Q47" s="8" t="n">
-        <v>0.02964</v>
+        <v>0.02966</v>
       </c>
       <c r="R47" s="8" t="n">
-        <v>0.15536</v>
+        <v>0.15516</v>
       </c>
       <c r="S47" s="8" t="n">
-        <v>0.04914</v>
+        <v>0.04907</v>
       </c>
       <c r="T47" s="8" t="n">
         <v>0.0043</v>
       </c>
       <c r="U47" s="8" t="n">
-        <v>4.6786</v>
+        <v>4.67393</v>
       </c>
     </row>
     <row r="48">
@@ -4245,7 +4245,7 @@
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>183.7</v>
+        <v>184.3</v>
       </c>
       <c r="E48" s="6">
         <f>D48*N48</f>
@@ -4284,28 +4284,28 @@
         <v/>
       </c>
       <c r="N48" s="8" t="n">
-        <v>4.285</v>
+        <v>4.284</v>
       </c>
       <c r="O48" s="8" t="n">
-        <v>0.24135</v>
+        <v>0.24189</v>
       </c>
       <c r="P48" s="8" t="n">
-        <v>0.08685</v>
+        <v>0.08696</v>
       </c>
       <c r="Q48" s="8" t="n">
-        <v>0.03498</v>
+        <v>0.03499</v>
       </c>
       <c r="R48" s="8" t="n">
-        <v>0.13607</v>
+        <v>0.13589</v>
       </c>
       <c r="S48" s="8" t="n">
-        <v>0.05158</v>
+        <v>0.05149</v>
       </c>
       <c r="T48" s="8" t="n">
         <v>0.00334</v>
       </c>
       <c r="U48" s="8" t="n">
-        <v>4.57799</v>
+        <v>4.57243</v>
       </c>
     </row>
     <row r="49">
@@ -4325,7 +4325,7 @@
         </is>
       </c>
       <c r="D49" s="5" t="n">
-        <v>181.7</v>
+        <v>182</v>
       </c>
       <c r="E49" s="6">
         <f>D49*N49</f>
@@ -4364,28 +4364,28 @@
         <v/>
       </c>
       <c r="N49" s="8" t="n">
-        <v>4.189</v>
+        <v>4.188</v>
       </c>
       <c r="O49" s="8" t="n">
-        <v>0.2054</v>
+        <v>0.20589</v>
       </c>
       <c r="P49" s="8" t="n">
-        <v>0.07975</v>
+        <v>0.07985</v>
       </c>
       <c r="Q49" s="8" t="n">
-        <v>0.03047</v>
+        <v>0.03049</v>
       </c>
       <c r="R49" s="8" t="n">
-        <v>0.14218</v>
+        <v>0.14201</v>
       </c>
       <c r="S49" s="8" t="n">
-        <v>0.04211</v>
+        <v>0.04204</v>
       </c>
       <c r="T49" s="8" t="n">
         <v>0.00353</v>
       </c>
       <c r="U49" s="8" t="n">
-        <v>4.05708</v>
+        <v>4.05278</v>
       </c>
     </row>
     <row r="50">
@@ -4405,7 +4405,7 @@
         </is>
       </c>
       <c r="D50" s="5" t="n">
-        <v>181.6</v>
+        <v>182</v>
       </c>
       <c r="E50" s="6">
         <f>D50*N50</f>
@@ -4444,28 +4444,28 @@
         <v/>
       </c>
       <c r="N50" s="8" t="n">
-        <v>3.957</v>
+        <v>3.956</v>
       </c>
       <c r="O50" s="8" t="n">
-        <v>0.29037</v>
+        <v>0.29099</v>
       </c>
       <c r="P50" s="8" t="n">
-        <v>0.05088</v>
+        <v>0.05095</v>
       </c>
       <c r="Q50" s="8" t="n">
-        <v>0.02315</v>
+        <v>0.02316</v>
       </c>
       <c r="R50" s="8" t="n">
-        <v>0.1413</v>
+        <v>0.14109</v>
       </c>
       <c r="S50" s="8" t="n">
-        <v>0.03717</v>
+        <v>0.0371</v>
       </c>
       <c r="T50" s="8" t="n">
         <v>0.00319</v>
       </c>
       <c r="U50" s="8" t="n">
-        <v>2.99035</v>
+        <v>2.98544</v>
       </c>
     </row>
     <row r="51">
@@ -4485,7 +4485,7 @@
         </is>
       </c>
       <c r="D51" s="5" t="n">
-        <v>180.5</v>
+        <v>180.7</v>
       </c>
       <c r="E51" s="6">
         <f>D51*N51</f>
@@ -4524,39 +4524,39 @@
         <v/>
       </c>
       <c r="N51" s="8" t="n">
-        <v>4.034</v>
+        <v>4.033</v>
       </c>
       <c r="O51" s="8" t="n">
-        <v>0.26047</v>
+        <v>0.26106</v>
       </c>
       <c r="P51" s="8" t="n">
-        <v>0.05921</v>
+        <v>0.05928</v>
       </c>
       <c r="Q51" s="8" t="n">
-        <v>0.03685</v>
+        <v>0.03687</v>
       </c>
       <c r="R51" s="8" t="n">
-        <v>0.13085</v>
+        <v>0.13067</v>
       </c>
       <c r="S51" s="8" t="n">
-        <v>0.04077</v>
+        <v>0.0407</v>
       </c>
       <c r="T51" s="8" t="n">
         <v>0.00277</v>
       </c>
       <c r="U51" s="8" t="n">
-        <v>3.71535</v>
+        <v>3.71069</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Seth Lugo</t>
+          <t>Freddy Peralta</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>178.8</v>
+        <v>179.6</v>
       </c>
       <c r="E52" s="6">
         <f>D52*N52</f>
@@ -4604,39 +4604,39 @@
         <v/>
       </c>
       <c r="N52" s="8" t="n">
-        <v>4.285</v>
+        <v>4.175</v>
       </c>
       <c r="O52" s="8" t="n">
-        <v>0.20199</v>
+        <v>0.25531</v>
       </c>
       <c r="P52" s="8" t="n">
-        <v>0.0721</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="Q52" s="8" t="n">
-        <v>0.03645</v>
+        <v>0.02869</v>
       </c>
       <c r="R52" s="8" t="n">
-        <v>0.1485</v>
+        <v>0.13059</v>
       </c>
       <c r="S52" s="8" t="n">
-        <v>0.04779</v>
+        <v>0.03841</v>
       </c>
       <c r="T52" s="8" t="n">
-        <v>0.00533</v>
+        <v>0.00359</v>
       </c>
       <c r="U52" s="8" t="n">
-        <v>4.73904</v>
+        <v>3.78599</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Freddy Peralta</t>
+          <t>Seth Lugo</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4645,7 +4645,7 @@
         </is>
       </c>
       <c r="D53" s="5" t="n">
-        <v>178.6</v>
+        <v>179.2</v>
       </c>
       <c r="E53" s="6">
         <f>D53*N53</f>
@@ -4684,28 +4684,28 @@
         <v/>
       </c>
       <c r="N53" s="8" t="n">
-        <v>4.176</v>
+        <v>4.284</v>
       </c>
       <c r="O53" s="8" t="n">
-        <v>0.25476</v>
+        <v>0.20247</v>
       </c>
       <c r="P53" s="8" t="n">
-        <v>0.08928999999999999</v>
+        <v>0.07219</v>
       </c>
       <c r="Q53" s="8" t="n">
-        <v>0.02868</v>
+        <v>0.03648</v>
       </c>
       <c r="R53" s="8" t="n">
-        <v>0.13078</v>
+        <v>0.14832</v>
       </c>
       <c r="S53" s="8" t="n">
-        <v>0.03848</v>
+        <v>0.04772</v>
       </c>
       <c r="T53" s="8" t="n">
-        <v>0.00359</v>
+        <v>0.00531</v>
       </c>
       <c r="U53" s="8" t="n">
-        <v>3.79051</v>
+        <v>4.73457</v>
       </c>
     </row>
     <row r="54">
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>178.5</v>
+        <v>178.9</v>
       </c>
       <c r="E54" s="6">
         <f>D54*N54</f>
@@ -4764,28 +4764,28 @@
         <v/>
       </c>
       <c r="N54" s="8" t="n">
-        <v>4.234</v>
+        <v>4.233</v>
       </c>
       <c r="O54" s="8" t="n">
-        <v>0.20431</v>
+        <v>0.20479</v>
       </c>
       <c r="P54" s="8" t="n">
-        <v>0.07996</v>
+        <v>0.08008</v>
       </c>
       <c r="Q54" s="8" t="n">
-        <v>0.03975</v>
+        <v>0.03977</v>
       </c>
       <c r="R54" s="8" t="n">
-        <v>0.13812</v>
+        <v>0.13796</v>
       </c>
       <c r="S54" s="8" t="n">
-        <v>0.04587</v>
+        <v>0.04579</v>
       </c>
       <c r="T54" s="8" t="n">
         <v>0.00309</v>
       </c>
       <c r="U54" s="8" t="n">
-        <v>4.56318</v>
+        <v>4.55937</v>
       </c>
     </row>
     <row r="55">
@@ -4805,7 +4805,7 @@
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>177.7</v>
+        <v>178.3</v>
       </c>
       <c r="E55" s="6">
         <f>D55*N55</f>
@@ -4844,28 +4844,28 @@
         <v/>
       </c>
       <c r="N55" s="8" t="n">
-        <v>4.067</v>
+        <v>4.066</v>
       </c>
       <c r="O55" s="8" t="n">
-        <v>0.22988</v>
+        <v>0.23041</v>
       </c>
       <c r="P55" s="8" t="n">
-        <v>0.06849</v>
+        <v>0.06858</v>
       </c>
       <c r="Q55" s="8" t="n">
         <v>0.01736</v>
       </c>
       <c r="R55" s="8" t="n">
-        <v>0.15085</v>
+        <v>0.15066</v>
       </c>
       <c r="S55" s="8" t="n">
-        <v>0.03607</v>
+        <v>0.03601</v>
       </c>
       <c r="T55" s="8" t="n">
         <v>0.00235</v>
       </c>
       <c r="U55" s="8" t="n">
-        <v>3.13524</v>
+        <v>3.13062</v>
       </c>
     </row>
     <row r="56">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>175.6</v>
+        <v>175.8</v>
       </c>
       <c r="E56" s="6">
         <f>D56*N56</f>
@@ -4924,28 +4924,28 @@
         <v/>
       </c>
       <c r="N56" s="8" t="n">
-        <v>4.041</v>
+        <v>4.04</v>
       </c>
       <c r="O56" s="8" t="n">
-        <v>0.24063</v>
+        <v>0.24118</v>
       </c>
       <c r="P56" s="8" t="n">
-        <v>0.05535</v>
+        <v>0.05543</v>
       </c>
       <c r="Q56" s="8" t="n">
-        <v>0.02812</v>
+        <v>0.02813</v>
       </c>
       <c r="R56" s="8" t="n">
-        <v>0.14159</v>
+        <v>0.1414</v>
       </c>
       <c r="S56" s="8" t="n">
-        <v>0.04116</v>
+        <v>0.04109</v>
       </c>
       <c r="T56" s="8" t="n">
         <v>0.00299</v>
       </c>
       <c r="U56" s="8" t="n">
-        <v>3.50438</v>
+        <v>3.49972</v>
       </c>
     </row>
     <row r="57">
@@ -4965,7 +4965,7 @@
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>175.1</v>
+        <v>175.4</v>
       </c>
       <c r="E57" s="6">
         <f>D57*N57</f>
@@ -5004,28 +5004,28 @@
         <v/>
       </c>
       <c r="N57" s="8" t="n">
-        <v>4.086</v>
+        <v>4.085</v>
       </c>
       <c r="O57" s="8" t="n">
-        <v>0.24363</v>
+        <v>0.24419</v>
       </c>
       <c r="P57" s="8" t="n">
-        <v>0.0655</v>
+        <v>0.06559</v>
       </c>
       <c r="Q57" s="8" t="n">
-        <v>0.02302</v>
+        <v>0.02303</v>
       </c>
       <c r="R57" s="8" t="n">
-        <v>0.15105</v>
+        <v>0.15085</v>
       </c>
       <c r="S57" s="8" t="n">
-        <v>0.03475</v>
+        <v>0.03469</v>
       </c>
       <c r="T57" s="8" t="n">
         <v>0.00296</v>
       </c>
       <c r="U57" s="8" t="n">
-        <v>3.37647</v>
+        <v>3.37174</v>
       </c>
     </row>
     <row r="58">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>174.2</v>
+        <v>174.4</v>
       </c>
       <c r="E58" s="6">
         <f>D58*N58</f>
@@ -5084,28 +5084,28 @@
         <v/>
       </c>
       <c r="N58" s="8" t="n">
-        <v>4.129</v>
+        <v>4.128</v>
       </c>
       <c r="O58" s="8" t="n">
-        <v>0.22156</v>
+        <v>0.22209</v>
       </c>
       <c r="P58" s="8" t="n">
-        <v>0.04808</v>
+        <v>0.04815</v>
       </c>
       <c r="Q58" s="8" t="n">
-        <v>0.02647</v>
+        <v>0.02649</v>
       </c>
       <c r="R58" s="8" t="n">
-        <v>0.16381</v>
+        <v>0.16361</v>
       </c>
       <c r="S58" s="8" t="n">
-        <v>0.04377</v>
+        <v>0.0437</v>
       </c>
       <c r="T58" s="8" t="n">
         <v>0.00373</v>
       </c>
       <c r="U58" s="8" t="n">
-        <v>3.87471</v>
+        <v>3.86991</v>
       </c>
     </row>
     <row r="59">
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="D59" s="5" t="n">
-        <v>173.6</v>
+        <v>174</v>
       </c>
       <c r="E59" s="6">
         <f>D59*N59</f>
@@ -5164,28 +5164,28 @@
         <v/>
       </c>
       <c r="N59" s="8" t="n">
-        <v>4.215</v>
+        <v>4.214</v>
       </c>
       <c r="O59" s="8" t="n">
-        <v>0.24946</v>
+        <v>0.25001</v>
       </c>
       <c r="P59" s="8" t="n">
-        <v>0.07217999999999999</v>
+        <v>0.07227</v>
       </c>
       <c r="Q59" s="8" t="n">
-        <v>0.02475</v>
+        <v>0.02476</v>
       </c>
       <c r="R59" s="8" t="n">
-        <v>0.15119</v>
+        <v>0.15097</v>
       </c>
       <c r="S59" s="8" t="n">
-        <v>0.033</v>
+        <v>0.03293</v>
       </c>
       <c r="T59" s="8" t="n">
         <v>0.00382</v>
       </c>
       <c r="U59" s="8" t="n">
-        <v>3.78873</v>
+        <v>3.78379</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add season simulation: direction-aware floor (P25) and ceiling (P75) for every projected stat
season_sim.py simulates each projected player's season (role mixture draw,
health, talent uncertainty from SD_*, event luck) and the export now carries
<stat>_floor / <stat>_ceil beside each stat. For stats where lower is better
(ERA, WHIP, BB, H and HR allowed, hitter SO/CS) the ceiling is the 25th
percentile. Regenerated the committed export files.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q9BVygbWYQ2F3GpBZTE3wi
</commit_message>
<xml_diff>
--- a/out/mlb_2027_what_if.xlsx
+++ b/out/mlb_2027_what_if.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="What-If" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What-If" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>